<commit_message>
feat(ours): whose email, which code, and a waiting screen that says so
A couple field report (2026-09-13): en route to "share with my wife",
the sign-in email field read as the share form and an address typed
there silently became an account; the invite code went into the wrong
code field; and after leaving the one-time code screen there was "no
easy way to regenerate". Four fixes, five locales: the Menu line stops
saying "needs your email", the sign-in field is labelled "Your own
email" with a subtitle that places sharing later inside Ours, the two
code fields hint at each other's codes beside honest failures, and the
waiting-with-no-code state is titled truthfully with "Get a new code"
promoted to a real button. Re-showing codes stays impossible on
purpose: the server keeps only a hash.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$390</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$392</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J390"/>
+  <dimension ref="A1:J392"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -11894,7 +11894,7 @@
     <row r="280">
       <c r="A280" s="6" t="inlineStr">
         <is>
-          <t>OUR-15</t>
+          <t>OUR-120</t>
         </is>
       </c>
       <c r="B280" s="7" t="inlineStr">
@@ -11909,17 +11909,17 @@
       </c>
       <c r="D280" s="9" t="inlineStr">
         <is>
-          <t>Leave a list, then start a new one WITHOUT deleting the old</t>
+          <t>Waiting-with-no-code says so, and the re-mint is a real button</t>
         </is>
       </c>
       <c r="E280" s="9" t="inlineStr">
         <is>
-          <t>Leave a shared list. On the closed screen, start a new shared list with someone else.</t>
+          <t>Mint a code, leave Ours entirely (back to Today), then come back to Ours before anyone joins.</t>
         </is>
       </c>
       <c r="F280" s="9" t="inlineStr">
         <is>
-          <t>Starting a new list is offered on the closed screen itself and works. The old list is NOT deleted and is still readable. At no point is destroying it the only way forward.</t>
+          <t>The screen is titled 'Waiting for your person', NOT 'Read this to your person' over an empty space (the code renders exactly once; the server keeps only a hash, so it can never be re-shown). 'Get a new code' is a full primary button in this state, not a quiet text link (the 2026-09-13 field report walked right past the link: 'no easy way to... regenerate the code'). While the code IS still on screen, the title and the quiet link stay as they were.</t>
         </is>
       </c>
       <c r="G280" s="7" t="inlineStr">
@@ -11934,7 +11934,7 @@
     <row r="281">
       <c r="A281" s="6" t="inlineStr">
         <is>
-          <t>OUR-16</t>
+          <t>OUR-121</t>
         </is>
       </c>
       <c r="B281" s="7" t="inlineStr">
@@ -11949,17 +11949,17 @@
       </c>
       <c r="D281" s="9" t="inlineStr">
         <is>
-          <t>A failed read never offers to start a list you already have</t>
+          <t>Whose email, and which code goes where</t>
         </is>
       </c>
       <c r="E281" s="9" t="inlineStr">
         <is>
-          <t>With a live shared list, turn the network off and open Ours.</t>
+          <t>Signed out: read the Menu's Ours line, open Ours, read the signed-out screen, tap Sign in and read the field. Then, on the sign-in code step, paste an Ours-style code (letters in it). Separately, signed in, open Ours 'I have a code' and type a 6-digit emailed sign-in code.</t>
         </is>
       </c>
       <c r="F281" s="9" t="inlineStr">
         <is>
-          <t>A calm connection line. The screen never says you have no shared list and never offers to start one. Turning the network back on recovers without a restart.</t>
+          <t>The Menu's Ours line reads 'A list kept with one person. Sign in first.' (the old 'Needs your email, no password' invited typing the PARTNER'S email; a real user did exactly that on 2026-09-13 and it became their account). The Ours signed-out screen opens with the plain fact 'You're not signed in on this phone.' The sign-in email field is labelled 'Your own email', and the subtitle says sharing happens later, in Ours, with a code, never by typing the partner's email here. Letters in the 6-digit code field draw the calm hint that it will be an Ours invite code (a hint, never an auto-redirect or a cleared field). Six bare digits failing in the Ours join field add one line naming the emailed sign-in code as the likely mix-up, alongside the unchanged honest failure.</t>
         </is>
       </c>
       <c r="G281" s="7" t="inlineStr">
@@ -11974,7 +11974,7 @@
     <row r="282">
       <c r="A282" s="6" t="inlineStr">
         <is>
-          <t>OUR-17</t>
+          <t>OUR-15</t>
         </is>
       </c>
       <c r="B282" s="7" t="inlineStr">
@@ -11982,24 +11982,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C282" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C282" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D282" s="9" t="inlineStr">
         <is>
-          <t>A list nobody joined can be left</t>
+          <t>Leave a list, then start a new one WITHOUT deleting the old</t>
         </is>
       </c>
       <c r="E282" s="9" t="inlineStr">
         <is>
-          <t>Create a list, get a code, give it to nobody. Return to Ours.</t>
+          <t>Leave a shared list. On the closed screen, start a new shared list with someone else.</t>
         </is>
       </c>
       <c r="F282" s="9" t="inlineStr">
         <is>
-          <t>There is a way out on the waiting screen, and its wording does not claim it closes for two people. After leaving, you can start or join a list again.</t>
+          <t>Starting a new list is offered on the closed screen itself and works. The old list is NOT deleted and is still readable. At no point is destroying it the only way forward.</t>
         </is>
       </c>
       <c r="G282" s="7" t="inlineStr">
@@ -12014,7 +12014,7 @@
     <row r="283">
       <c r="A283" s="6" t="inlineStr">
         <is>
-          <t>OUR-18</t>
+          <t>OUR-16</t>
         </is>
       </c>
       <c r="B283" s="7" t="inlineStr">
@@ -12022,24 +12022,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C283" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C283" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D283" s="9" t="inlineStr">
         <is>
-          <t>The arrival announces once and stays announced</t>
+          <t>A failed read never offers to start a list you already have</t>
         </is>
       </c>
       <c r="E283" s="9" t="inlineStr">
         <is>
-          <t>Sit on the waiting screen while the other account joins. Background the app and return.</t>
+          <t>With a live shared list, turn the network off and open Ours.</t>
         </is>
       </c>
       <c r="F283" s="9" t="inlineStr">
         <is>
-          <t>The name appears once and does not flicker back to waiting and re-announce. The way out beside it ('that wasn't who I meant') never appears on a list you did not just gain a person on.</t>
+          <t>A calm connection line. The screen never says you have no shared list and never offers to start one. Turning the network back on recovers without a restart.</t>
         </is>
       </c>
       <c r="G283" s="7" t="inlineStr">
@@ -12054,7 +12054,7 @@
     <row r="284">
       <c r="A284" s="6" t="inlineStr">
         <is>
-          <t>OUR-19</t>
+          <t>OUR-17</t>
         </is>
       </c>
       <c r="B284" s="7" t="inlineStr">
@@ -12069,17 +12069,17 @@
       </c>
       <c r="D284" s="9" t="inlineStr">
         <is>
-          <t>A repeat the app cannot read is SHOWN, never hidden</t>
+          <t>A list nobody joined can be left</t>
         </is>
       </c>
       <c r="E284" s="9" t="inlineStr">
         <is>
-          <t>Requires two app versions. On the newer one, set a shared task to a cadence the older build does not have. Open the list on the older build.</t>
+          <t>Create a list, get a code, give it to nobody. Return to Ours.</t>
         </is>
       </c>
       <c r="F284" s="9" t="inlineStr">
         <is>
-          <t>The task is visible on both, with whatever cadence line the newer app left. It is never silently absent from one person's list, and the older app does not erase the schedule when it syncs.</t>
+          <t>There is a way out on the waiting screen, and its wording does not claim it closes for two people. After leaving, you can start or join a list again.</t>
         </is>
       </c>
       <c r="G284" s="7" t="inlineStr">
@@ -12094,7 +12094,7 @@
     <row r="285">
       <c r="A285" s="6" t="inlineStr">
         <is>
-          <t>OUR-20</t>
+          <t>OUR-18</t>
         </is>
       </c>
       <c r="B285" s="7" t="inlineStr">
@@ -12102,24 +12102,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C285" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C285" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D285" s="9" t="inlineStr">
         <is>
-          <t>The room opens from Today and from the Menu</t>
+          <t>The arrival announces once and stays announced</t>
         </is>
       </c>
       <c r="E285" s="9" t="inlineStr">
         <is>
-          <t>With a live shared list, tap the 'Ours · {name}' row on Today. Then go back and reach it through Menu › Ours.</t>
+          <t>Sit on the waiting screen while the other account joins. Background the app and return.</t>
         </is>
       </c>
       <c r="F285" s="9" t="inlineStr">
         <is>
-          <t>Both land on the shared list itself, not the pairing screen. The header line reads 'Kept with {their name}' and tapping it goes to the pairing/management screen.</t>
+          <t>The name appears once and does not flicker back to waiting and re-announce. The way out beside it ('that wasn't who I meant') never appears on a list you did not just gain a person on.</t>
         </is>
       </c>
       <c r="G285" s="7" t="inlineStr">
@@ -12134,7 +12134,7 @@
     <row r="286">
       <c r="A286" s="6" t="inlineStr">
         <is>
-          <t>OUR-21</t>
+          <t>OUR-19</t>
         </is>
       </c>
       <c r="B286" s="7" t="inlineStr">
@@ -12142,24 +12142,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C286" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C286" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D286" s="9" t="inlineStr">
         <is>
-          <t>Add, tick and UN-tick on the shared list</t>
+          <t>A repeat the app cannot read is SHOWN, never hidden</t>
         </is>
       </c>
       <c r="E286" s="9" t="inlineStr">
         <is>
-          <t>Add a task in the room. Tick it. Un-tick it. Watch the other account (reload or wait ~15s).</t>
+          <t>Requires two app versions. On the newer one, set a shared task to a cadence the older build does not have. Open the list on the older build.</t>
         </is>
       </c>
       <c r="F286" s="9" t="inlineStr">
         <is>
-          <t>Every step appears on both. Un-ticking works as easily as ticking, on both sides. No affirmation or celebration fires on Ours.</t>
+          <t>The task is visible on both, with whatever cadence line the newer app left. It is never silently absent from one person's list, and the older app does not erase the schedule when it syncs.</t>
         </is>
       </c>
       <c r="G286" s="7" t="inlineStr">
@@ -12174,7 +12174,7 @@
     <row r="287">
       <c r="A287" s="6" t="inlineStr">
         <is>
-          <t>OUR-22</t>
+          <t>OUR-20</t>
         </is>
       </c>
       <c r="B287" s="7" t="inlineStr">
@@ -12189,17 +12189,17 @@
       </c>
       <c r="D287" s="9" t="inlineStr">
         <is>
-          <t>Un-tick a one-off the DAY AFTER it was ticked</t>
+          <t>The room opens from Today and from the Menu</t>
         </is>
       </c>
       <c r="E287" s="9" t="inlineStr">
         <is>
-          <t>Tick a shared one-off. Change the device date to tomorrow (or wait a day), reopen the room, tap it again.</t>
+          <t>With a live shared list, tap the 'Ours · {name}' row on Today. Then go back and reach it through Menu › Ours.</t>
         </is>
       </c>
       <c r="F287" s="9" t="inlineStr">
         <is>
-          <t>It un-ticks. (The pre-fix build could never un-tick it again, on any device, forever.)</t>
+          <t>Both land on the shared list itself, not the pairing screen. The header line reads 'Kept with {their name}' and tapping it goes to the pairing/management screen.</t>
         </is>
       </c>
       <c r="G287" s="7" t="inlineStr">
@@ -12214,7 +12214,7 @@
     <row r="288">
       <c r="A288" s="6" t="inlineStr">
         <is>
-          <t>OUR-23</t>
+          <t>OUR-21</t>
         </is>
       </c>
       <c r="B288" s="7" t="inlineStr">
@@ -12229,17 +12229,17 @@
       </c>
       <c r="D288" s="9" t="inlineStr">
         <is>
-          <t>Bring to my Today makes a COPY, and marks only yours</t>
+          <t>Add, tick and UN-tick on the shared list</t>
         </is>
       </c>
       <c r="E288" s="9" t="inlineStr">
         <is>
-          <t>Hold a shared row, tap 'Bring to my Today'. Look at your Today, then at the shared list on BOTH accounts.</t>
+          <t>Add a task in the room. Tick it. Un-tick it. Watch the other account (reload or wait ~15s).</t>
         </is>
       </c>
       <c r="F288" s="9" t="inlineStr">
         <is>
-          <t>Your Today shows the task with a faint '· Ours'. The shared row is completely unchanged on both sides, with no marker of any kind. The held card now reads 'Already on your Today' and cannot make a second copy.</t>
+          <t>Every step appears on both. Un-ticking works as easily as ticking, on both sides. No affirmation or celebration fires on Ours.</t>
         </is>
       </c>
       <c r="G288" s="7" t="inlineStr">
@@ -12254,7 +12254,7 @@
     <row r="289">
       <c r="A289" s="6" t="inlineStr">
         <is>
-          <t>OUR-24</t>
+          <t>OUR-22</t>
         </is>
       </c>
       <c r="B289" s="7" t="inlineStr">
@@ -12269,17 +12269,17 @@
       </c>
       <c r="D289" s="9" t="inlineStr">
         <is>
-          <t>Your tick on the copy closes both</t>
+          <t>Un-tick a one-off the DAY AFTER it was ticked</t>
         </is>
       </c>
       <c r="E289" s="9" t="inlineStr">
         <is>
-          <t>Tick the brought copy on your Today. Check the shared list on the other account.</t>
+          <t>Tick a shared one-off. Change the device date to tomorrow (or wait a day), reopen the room, tap it again.</t>
         </is>
       </c>
       <c r="F289" s="9" t="inlineStr">
         <is>
-          <t>The shared row is done. It enters YOUR Lookback. Nothing on the other side says who did it.</t>
+          <t>It un-ticks. (The pre-fix build could never un-tick it again, on any device, forever.)</t>
         </is>
       </c>
       <c r="G289" s="7" t="inlineStr">
@@ -12294,7 +12294,7 @@
     <row r="290">
       <c r="A290" s="6" t="inlineStr">
         <is>
-          <t>OUR-25</t>
+          <t>OUR-23</t>
         </is>
       </c>
       <c r="B290" s="7" t="inlineStr">
@@ -12309,17 +12309,17 @@
       </c>
       <c r="D290" s="9" t="inlineStr">
         <is>
-          <t>Ticking a brought copy on a device that has NEVER opened the room</t>
+          <t>Bring to my Today makes a COPY, and marks only yours</t>
         </is>
       </c>
       <c r="E290" s="9" t="inlineStr">
         <is>
-          <t>Bring a task over on phone A. Sign in on a second device (or clear its local data) and go straight to Today WITHOUT opening Ours. Tick the copy there.</t>
+          <t>Hold a shared row, tap 'Bring to my Today'. Look at your Today, then at the shared list on BOTH accounts.</t>
         </is>
       </c>
       <c r="F290" s="9" t="inlineStr">
         <is>
-          <t>The shared row closes. (The pre-fix build silently discarded the tick with no error.)</t>
+          <t>Your Today shows the task with a faint '· Ours'. The shared row is completely unchanged on both sides, with no marker of any kind. The held card now reads 'Already on your Today' and cannot make a second copy.</t>
         </is>
       </c>
       <c r="G290" s="7" t="inlineStr">
@@ -12334,7 +12334,7 @@
     <row r="291">
       <c r="A291" s="6" t="inlineStr">
         <is>
-          <t>OUR-26</t>
+          <t>OUR-24</t>
         </is>
       </c>
       <c r="B291" s="7" t="inlineStr">
@@ -12349,17 +12349,17 @@
       </c>
       <c r="D291" s="9" t="inlineStr">
         <is>
-          <t>Their tick leaves a rest-note, never a strike-through</t>
+          <t>Your tick on the copy closes both</t>
         </is>
       </c>
       <c r="E291" s="9" t="inlineStr">
         <is>
-          <t>Bring a task over. On the OTHER account, tick the shared row. Return to your Today.</t>
+          <t>Tick the brought copy on your Today. Check the shared list on the other account.</t>
         </is>
       </c>
       <c r="F291" s="9" t="inlineStr">
         <is>
-          <t>Your copy is gone from the day, replaced by a dashed sage line: 'Handled on Ours. It's off your day.' It is NOT struck through and does NOT appear in your Lookback. Leaving Today and coming back clears the note.</t>
+          <t>The shared row is done. It enters YOUR Lookback. Nothing on the other side says who did it.</t>
         </is>
       </c>
       <c r="G291" s="7" t="inlineStr">
@@ -12374,7 +12374,7 @@
     <row r="292">
       <c r="A292" s="6" t="inlineStr">
         <is>
-          <t>OUR-27</t>
+          <t>OUR-25</t>
         </is>
       </c>
       <c r="B292" s="7" t="inlineStr">
@@ -12382,24 +12382,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C292" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C292" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D292" s="9" t="inlineStr">
         <is>
-          <t>Share to Ours warns about the length BEFORE it copies</t>
+          <t>Ticking a brought copy on a device that has NEVER opened the room</t>
         </is>
       </c>
       <c r="E292" s="9" t="inlineStr">
         <is>
-          <t>Hold one of your own Today tasks with a very long title (500+ chars), open More, tap 'Share to Ours'.</t>
+          <t>Bring a task over on phone A. Sign in on a second device (or clear its local data) and go straight to Today WITHOUT opening Ours. Tick the copy there.</t>
         </is>
       </c>
       <c r="F292" s="9" t="inlineStr">
         <is>
-          <t>A line says Ours keeps titles shorter and this one will be trimmed, BEFORE the copy is made. The copy appears on the shared list. 'Share to Ours' is absent entirely when there is no live list.</t>
+          <t>The shared row closes. (The pre-fix build silently discarded the tick with no error.)</t>
         </is>
       </c>
       <c r="G292" s="7" t="inlineStr">
@@ -12414,7 +12414,7 @@
     <row r="293">
       <c r="A293" s="6" t="inlineStr">
         <is>
-          <t>OUR-28</t>
+          <t>OUR-26</t>
         </is>
       </c>
       <c r="B293" s="7" t="inlineStr">
@@ -12429,17 +12429,17 @@
       </c>
       <c r="D293" s="9" t="inlineStr">
         <is>
-          <t>A repeat set on Ours uses the SAME cadence sheet as home</t>
+          <t>Their tick leaves a rest-note, never a strike-through</t>
         </is>
       </c>
       <c r="E293" s="9" t="inlineStr">
         <is>
-          <t>Hold a shared row, tap 'Repeat…'. Compare with Menu › Repeating › Edit on a personal task.</t>
+          <t>Bring a task over. On the OTHER account, tick the shared row. Return to your Today.</t>
         </is>
       </c>
       <c r="F293" s="9" t="inlineStr">
         <is>
-          <t>Identical controls. The commit button NAMES the cadence ('Every day', 'Every 2 days'), on both. The Ours sheet adds one line: 'You'll both see it on its day.' It appears on its days for both people.</t>
+          <t>Your copy is gone from the day, replaced by a dashed sage line: 'Handled on Ours. It's off your day.' It is NOT struck through and does NOT appear in your Lookback. Leaving Today and coming back clears the note.</t>
         </is>
       </c>
       <c r="G293" s="7" t="inlineStr">
@@ -12454,7 +12454,7 @@
     <row r="294">
       <c r="A294" s="6" t="inlineStr">
         <is>
-          <t>OUR-29</t>
+          <t>OUR-27</t>
         </is>
       </c>
       <c r="B294" s="7" t="inlineStr">
@@ -12462,24 +12462,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C294" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C294" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D294" s="9" t="inlineStr">
         <is>
-          <t>A cadence this build cannot read is inert, and says why</t>
+          <t>Share to Ours warns about the length BEFORE it copies</t>
         </is>
       </c>
       <c r="E294" s="9" t="inlineStr">
         <is>
-          <t>Get a shared row carrying a recurrence this build does not understand (a newer build, or hand-write one via the API).</t>
+          <t>Hold one of your own Today tasks with a very long title (500+ chars), open More, tap 'Share to Ours'.</t>
         </is>
       </c>
       <c r="F294" s="9" t="inlineStr">
         <is>
-          <t>The row is SHOWN, never hidden. Tapping it does nothing and a line explains it is safe and will appear on its days after an update. 'Repeat…' is withheld. It never marks itself done.</t>
+          <t>A line says Ours keeps titles shorter and this one will be trimmed, BEFORE the copy is made. The copy appears on the shared list. 'Share to Ours' is absent entirely when there is no live list.</t>
         </is>
       </c>
       <c r="G294" s="7" t="inlineStr">
@@ -12494,7 +12494,7 @@
     <row r="295">
       <c r="A295" s="6" t="inlineStr">
         <is>
-          <t>OUR-30</t>
+          <t>OUR-28</t>
         </is>
       </c>
       <c r="B295" s="7" t="inlineStr">
@@ -12502,24 +12502,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C295" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C295" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D295" s="9" t="inlineStr">
         <is>
-          <t>The quiet wash marks what changed, and never your own edits</t>
+          <t>A repeat set on Ours uses the SAME cadence sheet as home</t>
         </is>
       </c>
       <c r="E295" s="9" t="inlineStr">
         <is>
-          <t>Have the other account add and change a few rows. Open the room. Then tick something yourself and reopen.</t>
+          <t>Hold a shared row, tap 'Repeat…'. Compare with Menu › Repeating › Edit on a personal task.</t>
         </is>
       </c>
       <c r="F295" s="9" t="inlineStr">
         <is>
-          <t>Their changed rows carry a tint and a firmer border on arrival; a screen reader says 'changed since you last looked'. Your OWN edits are never washed. Leaving and returning clears it.</t>
+          <t>Identical controls. The commit button NAMES the cadence ('Every day', 'Every 2 days'), on both. The Ours sheet adds one line: 'You'll both see it on its day.' It appears on its days for both people.</t>
         </is>
       </c>
       <c r="G295" s="7" t="inlineStr">
@@ -12534,7 +12534,7 @@
     <row r="296">
       <c r="A296" s="6" t="inlineStr">
         <is>
-          <t>OUR-31</t>
+          <t>OUR-29</t>
         </is>
       </c>
       <c r="B296" s="7" t="inlineStr">
@@ -12542,24 +12542,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C296" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C296" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D296" s="9" t="inlineStr">
         <is>
-          <t>Recently removed puts a task back</t>
+          <t>A cadence this build cannot read is inert, and says why</t>
         </is>
       </c>
       <c r="E296" s="9" t="inlineStr">
         <is>
-          <t>Remove a shared row. Scroll to the foot of the list.</t>
+          <t>Get a shared row carrying a recurrence this build does not understand (a newer build, or hand-write one via the API).</t>
         </is>
       </c>
       <c r="F296" s="9" t="inlineStr">
         <is>
-          <t>It sits under 'Recently removed', dimmed, with 'Put it back'. Restoring returns it for both people. Nothing anywhere says which of you removed it.</t>
+          <t>The row is SHOWN, never hidden. Tapping it does nothing and a line explains it is safe and will appear on its days after an update. 'Repeat…' is withheld. It never marks itself done.</t>
         </is>
       </c>
       <c r="G296" s="7" t="inlineStr">
@@ -12574,7 +12574,7 @@
     <row r="297">
       <c r="A297" s="6" t="inlineStr">
         <is>
-          <t>OUR-32</t>
+          <t>OUR-30</t>
         </is>
       </c>
       <c r="B297" s="7" t="inlineStr">
@@ -12589,17 +12589,17 @@
       </c>
       <c r="D297" s="9" t="inlineStr">
         <is>
-          <t>Removing a shared REPEAT does not pretend to be 'Skip today'</t>
+          <t>The quiet wash marks what changed, and never your own edits</t>
         </is>
       </c>
       <c r="E297" s="9" t="inlineStr">
         <is>
-          <t>Hold a repeating shared row and look at the shelf.</t>
+          <t>Have the other account add and change a few rows. Open the room. Then tick something yourself and reopen.</t>
         </is>
       </c>
       <c r="F297" s="9" t="inlineStr">
         <is>
-          <t>It reads 'Remove', not 'Skip today', and the spoken label names removing the repeat. (The shared list has no per-day skip; the pre-fix build promised one and deleted the series for both people.)</t>
+          <t>Their changed rows carry a tint and a firmer border on arrival; a screen reader says 'changed since you last looked'. Your OWN edits are never washed. Leaving and returning clears it.</t>
         </is>
       </c>
       <c r="G297" s="7" t="inlineStr">
@@ -12614,7 +12614,7 @@
     <row r="298">
       <c r="A298" s="6" t="inlineStr">
         <is>
-          <t>OUR-33</t>
+          <t>OUR-31</t>
         </is>
       </c>
       <c r="B298" s="7" t="inlineStr">
@@ -12622,24 +12622,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C298" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C298" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D298" s="9" t="inlineStr">
         <is>
-          <t>A closed list is still readable, and read-only</t>
+          <t>Recently removed puts a task back</t>
         </is>
       </c>
       <c r="E298" s="9" t="inlineStr">
         <is>
-          <t>Leave a list. Open it from the archive on the pairing screen.</t>
+          <t>Remove a shared row. Scroll to the foot of the list.</t>
         </is>
       </c>
       <c r="F298" s="9" t="inlineStr">
         <is>
-          <t>Every row is readable. The capture bar is GONE. Ticking, renaming, removing and re-cadencing all do nothing, and each row says why. Each row still offers taking a copy for yourself.</t>
+          <t>It sits under 'Recently removed', dimmed, with 'Put it back'. Restoring returns it for both people. Nothing anywhere says which of you removed it.</t>
         </is>
       </c>
       <c r="G298" s="7" t="inlineStr">
@@ -12654,7 +12654,7 @@
     <row r="299">
       <c r="A299" s="6" t="inlineStr">
         <is>
-          <t>OUR-34</t>
+          <t>OUR-32</t>
         </is>
       </c>
       <c r="B299" s="7" t="inlineStr">
@@ -12669,17 +12669,17 @@
       </c>
       <c r="D299" s="9" t="inlineStr">
         <is>
-          <t>The archive lists closed lists, and puts them away</t>
+          <t>Removing a shared REPEAT does not pretend to be 'Skip today'</t>
         </is>
       </c>
       <c r="E299" s="9" t="inlineStr">
         <is>
-          <t>With at least one closed list, look under 'Lists you have kept' on the pairing screen.</t>
+          <t>Hold a repeating shared row and look at the shelf.</t>
         </is>
       </c>
       <c r="F299" s="9" t="inlineStr">
         <is>
-          <t>Purpose and closed MONTH only, no counts of any kind. 'Put it away' hides it from the default view; 'Show the ones put away' brings it back. Nothing is deleted.</t>
+          <t>It reads 'Remove', not 'Skip today', and the spoken label names removing the repeat. (The shared list has no per-day skip; the pre-fix build promised one and deleted the series for both people.)</t>
         </is>
       </c>
       <c r="G299" s="7" t="inlineStr">
@@ -12694,7 +12694,7 @@
     <row r="300">
       <c r="A300" s="6" t="inlineStr">
         <is>
-          <t>OUR-35</t>
+          <t>OUR-33</t>
         </is>
       </c>
       <c r="B300" s="7" t="inlineStr">
@@ -12709,17 +12709,17 @@
       </c>
       <c r="D300" s="9" t="inlineStr">
         <is>
-          <t>Reopening together is a handshake, never unilateral</t>
+          <t>A closed list is still readable, and read-only</t>
         </is>
       </c>
       <c r="E300" s="9" t="inlineStr">
         <is>
-          <t>On a closed list, tap 'Reopen together…'. Read the code to the second account and enter it in the ordinary join field.</t>
+          <t>Leave a list. Open it from the archive on the pairing screen.</t>
         </is>
       </c>
       <c r="F300" s="9" t="inlineStr">
         <is>
-          <t>The offering side gets a code and nothing reopens yet. Entering it in the SAME field used for a new list reopens the list for both, with everything as it was. It is never asked which kind of code it is.</t>
+          <t>Every row is readable. The capture bar is GONE. Ticking, renaming, removing and re-cadencing all do nothing, and each row says why. Each row still offers taking a copy for yourself.</t>
         </is>
       </c>
       <c r="G300" s="7" t="inlineStr">
@@ -12734,7 +12734,7 @@
     <row r="301">
       <c r="A301" s="6" t="inlineStr">
         <is>
-          <t>OUR-36</t>
+          <t>OUR-34</t>
         </is>
       </c>
       <c r="B301" s="7" t="inlineStr">
@@ -12742,24 +12742,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C301" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C301" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D301" s="9" t="inlineStr">
         <is>
-          <t>Delete for good commits when the screen closes, not on a timer</t>
+          <t>The archive lists closed lists, and puts them away</t>
         </is>
       </c>
       <c r="E301" s="9" t="inlineStr">
         <is>
-          <t>On a closed list, tap 'Delete this list for good'. Read what appears. Tap 'Keep it'. Then do it again and navigate away instead.</t>
+          <t>With at least one closed list, look under 'Lists you have kept' on the pairing screen.</t>
         </is>
       </c>
       <c r="F301" s="9" t="inlineStr">
         <is>
-          <t>The line says nothing has been told to anyone yet and that it deletes when you leave this screen. There is NO countdown anywhere. 'Keep it' cancels it entirely. Leaving the screen with it standing actually deletes it.</t>
+          <t>Purpose and closed MONTH only, no counts of any kind. 'Put it away' hides it from the default view; 'Show the ones put away' brings it back. Nothing is deleted.</t>
         </is>
       </c>
       <c r="G301" s="7" t="inlineStr">
@@ -12774,7 +12774,7 @@
     <row r="302">
       <c r="A302" s="6" t="inlineStr">
         <is>
-          <t>OUR-37</t>
+          <t>OUR-35</t>
         </is>
       </c>
       <c r="B302" s="7" t="inlineStr">
@@ -12782,24 +12782,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C302" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C302" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D302" s="9" t="inlineStr">
         <is>
-          <t>Rename yourself, and only yourself</t>
+          <t>Reopening together is a handshake, never unilateral</t>
         </is>
       </c>
       <c r="E302" s="9" t="inlineStr">
         <is>
-          <t>On a live list, tap the line reading 'They see you as {name}' and type a new name.</t>
+          <t>On a closed list, tap 'Reopen together…'. Read the code to the second account and enter it in the ordinary join field.</t>
         </is>
       </c>
       <c r="F302" s="9" t="inlineStr">
         <is>
-          <t>Your name changes for both of you. There is no affordance anywhere to edit the OTHER person's name.</t>
+          <t>The offering side gets a code and nothing reopens yet. Entering it in the SAME field used for a new list reopens the list for both, with everything as it was. It is never asked which kind of code it is.</t>
         </is>
       </c>
       <c r="G302" s="7" t="inlineStr">
@@ -12814,7 +12814,7 @@
     <row r="303">
       <c r="A303" s="6" t="inlineStr">
         <is>
-          <t>OUR-38</t>
+          <t>OUR-36</t>
         </is>
       </c>
       <c r="B303" s="7" t="inlineStr">
@@ -12822,24 +12822,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C303" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C303" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D303" s="9" t="inlineStr">
         <is>
-          <t>A dropped signal never throws you out of the room</t>
+          <t>Delete for good commits when the screen closes, not on a timer</t>
         </is>
       </c>
       <c r="E303" s="9" t="inlineStr">
         <is>
-          <t>Open the room, then turn off the network and wait for a poll (~15s).</t>
+          <t>On a closed list, tap 'Delete this list for good'. Read what appears. Tap 'Keep it'. Then do it again and navigate away instead.</t>
         </is>
       </c>
       <c r="F303" s="9" t="inlineStr">
         <is>
-          <t>The list stays on screen with a quiet 'no connection' line. You are NOT redirected to the pairing screen, and nothing looks deleted.</t>
+          <t>The line says nothing has been told to anyone yet and that it deletes when you leave this screen. There is NO countdown anywhere. 'Keep it' cancels it entirely. Leaving the screen with it standing actually deletes it.</t>
         </is>
       </c>
       <c r="G303" s="7" t="inlineStr">
@@ -12854,7 +12854,7 @@
     <row r="304">
       <c r="A304" s="6" t="inlineStr">
         <is>
-          <t>OUR-39</t>
+          <t>OUR-37</t>
         </is>
       </c>
       <c r="B304" s="7" t="inlineStr">
@@ -12862,24 +12862,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C304" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C304" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D304" s="9" t="inlineStr">
         <is>
-          <t>Report this list reaches us and tells nobody else</t>
+          <t>Rename yourself, and only yourself</t>
         </is>
       </c>
       <c r="E304" s="9" t="inlineStr">
         <is>
-          <t>On a live shared list, scroll to the foot of the pairing screen and tap 'Report this list'. Then check the other account.</t>
+          <t>On a live list, tap the line reading 'They see you as {name}' and type a new name.</t>
         </is>
       </c>
       <c r="F304" s="9" t="inlineStr">
         <is>
-          <t>The row is quiet, never a red button, and says plainly that only we are told. After tapping it thanks you and says your person has not been told. NOTHING changes on the other account's screen, anywhere. The report email arrives carrying the pair id and no task text.</t>
+          <t>Your name changes for both of you. There is no affordance anywhere to edit the OTHER person's name.</t>
         </is>
       </c>
       <c r="G304" s="7" t="inlineStr">
@@ -12894,7 +12894,7 @@
     <row r="305">
       <c r="A305" s="6" t="inlineStr">
         <is>
-          <t>OUR-40</t>
+          <t>OUR-38</t>
         </is>
       </c>
       <c r="B305" s="7" t="inlineStr">
@@ -12902,24 +12902,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C305" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C305" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D305" s="9" t="inlineStr">
         <is>
-          <t>A disabled list reads EXACTLY like an ordinary closed one</t>
+          <t>A dropped signal never throws you out of the room</t>
         </is>
       </c>
       <c r="E305" s="9" t="inlineStr">
         <is>
-          <t>Set pairs.disabled_at by hand in Supabase for a test pair, then open it on both accounts.</t>
+          <t>Open the room, then turn off the network and wait for a poll (~15s).</t>
         </is>
       </c>
       <c r="F305" s="9" t="inlineStr">
         <is>
-          <t>Both see the ordinary 'This list is closed' state, read-only, with the archive row. There is NO mark, word, colour or ordering anywhere that distinguishes it from a list somebody simply left. (Any difference would tell a reported person they were reported.)</t>
+          <t>The list stays on screen with a quiet 'no connection' line. You are NOT redirected to the pairing screen, and nothing looks deleted.</t>
         </is>
       </c>
       <c r="G305" s="7" t="inlineStr">
@@ -12934,7 +12934,7 @@
     <row r="306">
       <c r="A306" s="6" t="inlineStr">
         <is>
-          <t>OUR-41</t>
+          <t>OUR-39</t>
         </is>
       </c>
       <c r="B306" s="7" t="inlineStr">
@@ -12942,24 +12942,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C306" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C306" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D306" s="9" t="inlineStr">
         <is>
-          <t>Leaving is the block, and needs no reason</t>
+          <t>Report this list reaches us and tells nobody else</t>
         </is>
       </c>
       <c r="E306" s="9" t="inlineStr">
         <is>
-          <t>On a live list, tap 'Leave this list'.</t>
+          <t>On a live shared list, scroll to the foot of the pairing screen and tap 'Report this list'. Then check the other account.</t>
         </is>
       </c>
       <c r="F306" s="9" t="inlineStr">
         <is>
-          <t>It closes immediately for both people, with no confirmation gauntlet, no reason asked, and no way for the other person to reopen it alone. Both can still read everything.</t>
+          <t>The row is quiet, never a red button, and says plainly that only we are told. After tapping it thanks you and says your person has not been told. NOTHING changes on the other account's screen, anywhere. The report email arrives carrying the pair id and no task text.</t>
         </is>
       </c>
       <c r="G306" s="7" t="inlineStr">
@@ -12974,32 +12974,32 @@
     <row r="307">
       <c r="A307" s="6" t="inlineStr">
         <is>
-          <t>LEG-05</t>
+          <t>OUR-40</t>
         </is>
       </c>
       <c r="B307" s="7" t="inlineStr">
         <is>
-          <t>Legal</t>
-        </is>
-      </c>
-      <c r="C307" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>Ours</t>
+        </is>
+      </c>
+      <c r="C307" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D307" s="9" t="inlineStr">
         <is>
-          <t>The shared-list clauses are in both copies of both documents</t>
+          <t>A disabled list reads EXACTLY like an ordinary closed one</t>
         </is>
       </c>
       <c r="E307" s="9" t="inlineStr">
         <is>
-          <t>Read Settings &gt; Privacy and Settings &gt; Terms in-app, then doubledone.app/privacy.html and /terms.html.</t>
+          <t>Set pairs.disabled_at by hand in Supabase for a test pair, then open it on both accounts.</t>
         </is>
       </c>
       <c r="F307" s="9" t="inlineStr">
         <is>
-          <t>Privacy carries the shared-lists sections (what the other person sees, that authorship is not stored, freezing, the 30-day window). Terms carry 'Shared lists, and what is not allowed on them' plus 'Reporting, and what we will do' with the 24-hour aim. In-app and web wording match.</t>
+          <t>Both see the ordinary 'This list is closed' state, read-only, with the archive row. There is NO mark, word, colour or ordering anywhere that distinguishes it from a list somebody simply left. (Any difference would tell a reported person they were reported.)</t>
         </is>
       </c>
       <c r="G307" s="7" t="inlineStr">
@@ -13014,7 +13014,7 @@
     <row r="308">
       <c r="A308" s="6" t="inlineStr">
         <is>
-          <t>OUR-42</t>
+          <t>OUR-41</t>
         </is>
       </c>
       <c r="B308" s="7" t="inlineStr">
@@ -13022,24 +13022,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C308" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C308" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D308" s="9" t="inlineStr">
         <is>
-          <t>A change on one phone appears on the other WITHOUT touching it</t>
+          <t>Leaving is the block, and needs no reason</t>
         </is>
       </c>
       <c r="E308" s="9" t="inlineStr">
         <is>
-          <t>Both sit on the shared list. One adds a task. Do not touch the other device.</t>
+          <t>On a live list, tap 'Leave this list'.</t>
         </is>
       </c>
       <c r="F308" s="9" t="inlineStr">
         <is>
-          <t>It appears within about 15 seconds. (The poll never fired once before 2026-08-09: setPair rebuilt the pair object every sync, which restarted the interval before it could tick.)</t>
+          <t>It closes immediately for both people, with no confirmation gauntlet, no reason asked, and no way for the other person to reopen it alone. Both can still read everything.</t>
         </is>
       </c>
       <c r="G308" s="7" t="inlineStr">
@@ -13054,32 +13054,32 @@
     <row r="309">
       <c r="A309" s="6" t="inlineStr">
         <is>
-          <t>OUR-43</t>
+          <t>LEG-05</t>
         </is>
       </c>
       <c r="B309" s="7" t="inlineStr">
         <is>
-          <t>Ours</t>
-        </is>
-      </c>
-      <c r="C309" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="C309" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D309" s="9" t="inlineStr">
         <is>
-          <t>Opening your own list does not bounce you back</t>
+          <t>The shared-list clauses are in both copies of both documents</t>
         </is>
       </c>
       <c r="E309" s="9" t="inlineStr">
         <is>
-          <t>With a live list, tap Ours then 'Open the list'. Also try /ours-list directly in a cold tab.</t>
+          <t>Read Settings &gt; Privacy and Settings &gt; Terms in-app, then doubledone.app/privacy.html and /terms.html.</t>
         </is>
       </c>
       <c r="F309" s="9" t="inlineStr">
         <is>
-          <t>You land on the list and stay. (useSession returns null while hydrating; the room used to read that as signed-out and redirect, making the button an endless loop.)</t>
+          <t>Privacy carries the shared-lists sections (what the other person sees, that authorship is not stored, freezing, the 30-day window). Terms carry 'Shared lists, and what is not allowed on them' plus 'Reporting, and what we will do' with the 24-hour aim. In-app and web wording match.</t>
         </is>
       </c>
       <c r="G309" s="7" t="inlineStr">
@@ -13094,7 +13094,7 @@
     <row r="310">
       <c r="A310" s="6" t="inlineStr">
         <is>
-          <t>OUR-44</t>
+          <t>OUR-42</t>
         </is>
       </c>
       <c r="B310" s="7" t="inlineStr">
@@ -13102,24 +13102,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C310" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C310" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D310" s="9" t="inlineStr">
         <is>
-          <t>The pairing screen offers a way INTO the list</t>
+          <t>A change on one phone appears on the other WITHOUT touching it</t>
         </is>
       </c>
       <c r="E310" s="9" t="inlineStr">
         <is>
-          <t>Finish pairing, then look at the pairing screen.</t>
+          <t>Both sit on the shared list. One adds a task. Do not touch the other device.</t>
         </is>
       </c>
       <c r="F310" s="9" t="inlineStr">
         <is>
-          <t>There is an 'Open the list' button. (It used to dead-end: the only route to the room was Today's door or the Menu, which a new pair has no reason to know about.)</t>
+          <t>It appears within about 15 seconds. (The poll never fired once before 2026-08-09: setPair rebuilt the pair object every sync, which restarted the interval before it could tick.)</t>
         </is>
       </c>
       <c r="G310" s="7" t="inlineStr">
@@ -13134,7 +13134,7 @@
     <row r="311">
       <c r="A311" s="6" t="inlineStr">
         <is>
-          <t>OUR-45</t>
+          <t>OUR-43</t>
         </is>
       </c>
       <c r="B311" s="7" t="inlineStr">
@@ -13142,24 +13142,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C311" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C311" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D311" s="9" t="inlineStr">
         <is>
-          <t>The quiet wash appears and then takes itself away</t>
+          <t>Opening your own list does not bounce you back</t>
         </is>
       </c>
       <c r="E311" s="9" t="inlineStr">
         <is>
-          <t>Have the other account change a row while you are elsewhere, then open the list.</t>
+          <t>With a live list, tap Ours then 'Open the list'. Also try /ours-list directly in a cold tab.</t>
         </is>
       </c>
       <c r="F311" s="9" t="inlineStr">
         <is>
-          <t>The changed row carries ONE warmed border, on the card itself, never a second ring around it. It clears itself after about 8 seconds without animating. It does not return on the next visit, even if the other phone's clock runs ahead.</t>
+          <t>You land on the list and stay. (useSession returns null while hydrating; the room used to read that as signed-out and redirect, making the button an endless loop.)</t>
         </is>
       </c>
       <c r="G311" s="7" t="inlineStr">
@@ -13174,7 +13174,7 @@
     <row r="312">
       <c r="A312" s="6" t="inlineStr">
         <is>
-          <t>OUR-47</t>
+          <t>OUR-44</t>
         </is>
       </c>
       <c r="B312" s="7" t="inlineStr">
@@ -13189,17 +13189,17 @@
       </c>
       <c r="D312" s="9" t="inlineStr">
         <is>
-          <t>The Ours door on Today is findable</t>
+          <t>The pairing screen offers a way INTO the list</t>
         </is>
       </c>
       <c r="E312" s="9" t="inlineStr">
         <is>
-          <t>With a live list, look at Today.</t>
+          <t>Finish pairing, then look at the pairing screen.</t>
         </is>
       </c>
       <c r="F312" s="9" t="inlineStr">
         <is>
-          <t>A tinted, accented card carrying the list's name, not a hairline footnote. Absent entirely when there is no live list.</t>
+          <t>There is an 'Open the list' button. (It used to dead-end: the only route to the room was Today's door or the Menu, which a new pair has no reason to know about.)</t>
         </is>
       </c>
       <c r="G312" s="7" t="inlineStr">
@@ -13214,7 +13214,7 @@
     <row r="313">
       <c r="A313" s="6" t="inlineStr">
         <is>
-          <t>OUR-48</t>
+          <t>OUR-45</t>
         </is>
       </c>
       <c r="B313" s="7" t="inlineStr">
@@ -13222,24 +13222,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C313" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C313" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D313" s="9" t="inlineStr">
         <is>
-          <t>Their tick marks your copy DONE and leaves it on your day</t>
+          <t>The quiet wash appears and then takes itself away</t>
         </is>
       </c>
       <c r="E313" s="9" t="inlineStr">
         <is>
-          <t>A has an open brought copy on Today. B ticks that row in Ours. A backgrounds the app and returns to Today WITHOUT navigating.</t>
+          <t>Have the other account change a row while you are elsewhere, then open the list.</t>
         </is>
       </c>
       <c r="F313" s="9" t="inlineStr">
         <is>
-          <t>The copy is still there, ticked, NOT gone. It appears in A's Lookback. Nothing anywhere says which of them did it. (Before 2026-08-11 it was tombstoned and replaced by a note, and for three rounds it vanished outright because it was marked done with no completion date.)</t>
+          <t>The changed row carries ONE warmed border, on the card itself, never a second ring around it. It clears itself after about 8 seconds without animating. It does not return on the next visit, even if the other phone's clock runs ahead.</t>
         </is>
       </c>
       <c r="G313" s="7" t="inlineStr">
@@ -13254,7 +13254,7 @@
     <row r="314">
       <c r="A314" s="6" t="inlineStr">
         <is>
-          <t>OUR-49</t>
+          <t>OUR-47</t>
         </is>
       </c>
       <c r="B314" s="7" t="inlineStr">
@@ -13262,24 +13262,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C314" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C314" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D314" s="9" t="inlineStr">
         <is>
-          <t>A settled copy carries a completion DATE, not just a done flag</t>
+          <t>The Ours door on Today is findable</t>
         </is>
       </c>
       <c r="E314" s="9" t="inlineStr">
         <is>
-          <t>After OUR-48, open Today with ?debug=1 and read the `copy` line for that task.</t>
+          <t>With a live list, look at Today.</t>
         </is>
       </c>
       <c r="F314" s="9" t="inlineStr">
         <is>
-          <t>done=true, doneDay = today's date, showsToday=true. A done task with doneDay=none is invisible on Today AND absent from Lookback: tasksForToday places a finished task by its completion day.</t>
+          <t>A tinted, accented card carrying the list's name, not a hairline footnote. Absent entirely when there is no live list.</t>
         </is>
       </c>
       <c r="G314" s="7" t="inlineStr">
@@ -13294,7 +13294,7 @@
     <row r="315">
       <c r="A315" s="6" t="inlineStr">
         <is>
-          <t>OUR-50</t>
+          <t>OUR-48</t>
         </is>
       </c>
       <c r="B315" s="7" t="inlineStr">
@@ -13302,24 +13302,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C315" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C315" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D315" s="9" t="inlineStr">
         <is>
-          <t>A finished copy can be brought over again</t>
+          <t>Their tick marks your copy DONE and leaves it on your day</t>
         </is>
       </c>
       <c r="E315" s="9" t="inlineStr">
         <is>
-          <t>After OUR-48, hold that row in Ours.</t>
+          <t>A has an open brought copy on Today. B ticks that row in Ours. A backgrounds the app and returns to Today WITHOUT navigating.</t>
         </is>
       </c>
       <c r="F315" s="9" t="inlineStr">
         <is>
-          <t>'Bring to my Today' is offered again, not 'Already on your Today'. (A done copy is not on your plate; while only tombstones were skipped you had a task you could neither see nor re-add.)</t>
+          <t>The copy is still there, ticked, NOT gone. It appears in A's Lookback. Nothing anywhere says which of them did it. (Before 2026-08-11 it was tombstoned and replaced by a note, and for three rounds it vanished outright because it was marked done with no completion date.)</t>
         </is>
       </c>
       <c r="G315" s="7" t="inlineStr">
@@ -13334,7 +13334,7 @@
     <row r="316">
       <c r="A316" s="6" t="inlineStr">
         <is>
-          <t>OUR-51</t>
+          <t>OUR-49</t>
         </is>
       </c>
       <c r="B316" s="7" t="inlineStr">
@@ -13349,17 +13349,17 @@
       </c>
       <c r="D316" s="9" t="inlineStr">
         <is>
-          <t>Your own edit never highlights; their later edit always does</t>
+          <t>A settled copy carries a completion DATE, not just a done flag</t>
         </is>
       </c>
       <c r="E316" s="9" t="inlineStr">
         <is>
-          <t>B ticks a row (A highlights). A un-ticks it. B ticks it again. Watch both screens throughout.</t>
+          <t>After OUR-48, open Today with ?debug=1 and read the `copy` line for that task.</t>
         </is>
       </c>
       <c r="F316" s="9" t="inlineStr">
         <is>
-          <t>Each side lights up for the OTHER's change every time, including repeatedly on the same row, and never for its own. (`mine` records WHEN you wrote a row, not merely that you did; as a plain id set, one touch made that row permanently dark on that device.)</t>
+          <t>done=true, doneDay = today's date, showsToday=true. A done task with doneDay=none is invisible on Today AND absent from Lookback: tasksForToday places a finished task by its completion day.</t>
         </is>
       </c>
       <c r="G316" s="7" t="inlineStr">
@@ -13374,7 +13374,7 @@
     <row r="317">
       <c r="A317" s="6" t="inlineStr">
         <is>
-          <t>OUR-52</t>
+          <t>OUR-50</t>
         </is>
       </c>
       <c r="B317" s="7" t="inlineStr">
@@ -13389,17 +13389,17 @@
       </c>
       <c r="D317" s="9" t="inlineStr">
         <is>
-          <t>The highlight arrives at once and fades away</t>
+          <t>A finished copy can be brought over again</t>
         </is>
       </c>
       <c r="E317" s="9" t="inlineStr">
         <is>
-          <t>Have B change a row while A is on the list.</t>
+          <t>After OUR-48, hold that row in Ours.</t>
         </is>
       </c>
       <c r="F317" s="9" t="inlineStr">
         <is>
-          <t>A's row warms immediately, holds about 8 seconds, then fades over roughly 700ms. It does not snap off, does not strobe, and does not return on the next poll for the same change. Reduce-motion gets an instant disappearance instead of a fade.</t>
+          <t>'Bring to my Today' is offered again, not 'Already on your Today'. (A done copy is not on your plate; while only tombstones were skipped you had a task you could neither see nor re-add.)</t>
         </is>
       </c>
       <c r="G317" s="7" t="inlineStr">
@@ -13414,7 +13414,7 @@
     <row r="318">
       <c r="A318" s="6" t="inlineStr">
         <is>
-          <t>OUR-53</t>
+          <t>OUR-51</t>
         </is>
       </c>
       <c r="B318" s="7" t="inlineStr">
@@ -13422,24 +13422,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C318" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C318" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D318" s="9" t="inlineStr">
         <is>
-          <t>Two devices share ONE clock</t>
+          <t>Your own edit never highlights; their later edit always does</t>
         </is>
       </c>
       <c r="E318" s="9" t="inlineStr">
         <is>
-          <t>Open the list on both devices with ?debug=1 and read `skew` on the wash line.</t>
+          <t>B ticks a row (A highlights). A un-ticks it. B ticks it again. Watch both screens throughout.</t>
         </is>
       </c>
       <c r="F318" s="9" t="inlineStr">
         <is>
-          <t>A small value in seconds, not minutes, on both. Every stamp (completion log, last-look, last-write-wins) is compared against server time via server_now(). A device whose clock ran ahead used to stamp its own last-look into the future and could never highlight anything again.</t>
+          <t>Each side lights up for the OTHER's change every time, including repeatedly on the same row, and never for its own. (`mine` records WHEN you wrote a row, not merely that you did; as a plain id set, one touch made that row permanently dark on that device.)</t>
         </is>
       </c>
       <c r="G318" s="7" t="inlineStr">
@@ -13454,7 +13454,7 @@
     <row r="319">
       <c r="A319" s="6" t="inlineStr">
         <is>
-          <t>OUR-54</t>
+          <t>OUR-52</t>
         </is>
       </c>
       <c r="B319" s="7" t="inlineStr">
@@ -13462,24 +13462,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C319" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C319" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D319" s="9" t="inlineStr">
         <is>
-          <t>The debug panel is opt-in and carries no task text</t>
+          <t>The highlight arrives at once and fades away</t>
         </is>
       </c>
       <c r="E319" s="9" t="inlineStr">
         <is>
-          <t>Open /ours-list?debug=1 and /today?debug=1, then the same URLs without the flag.</t>
+          <t>Have B change a row while A is on the list.</t>
         </is>
       </c>
       <c r="F319" s="9" t="inlineStr">
         <is>
-          <t>A small log appears only with the flag, at the top of Today and the foot of the list. Every line is counts, ids and flags. NO task title ever appears in it: these get screenshotted and pasted, and a shared list is two people's words.</t>
+          <t>A's row warms immediately, holds about 8 seconds, then fades over roughly 700ms. It does not snap off, does not strobe, and does not return on the next poll for the same change. Reduce-motion gets an instant disappearance instead of a fade.</t>
         </is>
       </c>
       <c r="G319" s="7" t="inlineStr">
@@ -13494,7 +13494,7 @@
     <row r="320">
       <c r="A320" s="6" t="inlineStr">
         <is>
-          <t>OUR-55</t>
+          <t>OUR-53</t>
         </is>
       </c>
       <c r="B320" s="7" t="inlineStr">
@@ -13502,24 +13502,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C320" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C320" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D320" s="9" t="inlineStr">
         <is>
-          <t>Capture on Ours IS Today's capture</t>
+          <t>Two devices share ONE clock</t>
         </is>
       </c>
       <c r="E320" s="9" t="inlineStr">
         <is>
-          <t>Open a shared list and tap the launcher at the foot of the screen.</t>
+          <t>Open the list on both devices with ?debug=1 and read `skew` on the wash line.</t>
         </is>
       </c>
       <c r="F320" s="9" t="inlineStr">
         <is>
-          <t>The same panel Today opens: the same input, the same Speak button (web), the same door, the same Add button naming its own consequence. Not a lookalike, the same component, so the two can never drift apart.</t>
+          <t>A small value in seconds, not minutes, on both. Every stamp (completion log, last-look, last-write-wins) is compared against server time via server_now(). A device whose clock ran ahead used to stamp its own last-look into the future and could never highlight anything again.</t>
         </is>
       </c>
       <c r="G320" s="7" t="inlineStr">
@@ -13534,7 +13534,7 @@
     <row r="321">
       <c r="A321" s="6" t="inlineStr">
         <is>
-          <t>OUR-56</t>
+          <t>OUR-54</t>
         </is>
       </c>
       <c r="B321" s="7" t="inlineStr">
@@ -13542,24 +13542,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C321" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C321" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D321" s="9" t="inlineStr">
         <is>
-          <t>Repeating can be set AT capture, without knowing a gesture</t>
+          <t>The debug panel is opt-in and carries no task text</t>
         </is>
       </c>
       <c r="E321" s="9" t="inlineStr">
         <is>
-          <t>In that panel, open the door and choose Daily (or Weekly, or Every N days), then Add.</t>
+          <t>Open /ours-list?debug=1 and /today?debug=1, then the same URLs without the flag.</t>
         </is>
       </c>
       <c r="F321" s="9" t="inlineStr">
         <is>
-          <t>The button reads 'Add · Daily' before the tap, and the row lands already repeating, visible to both of you. (Before this, the only way to make a repeating shared task was to add it and then somehow know to long-press it. Melroy: 'there is no way to add Repeating Tasks.')</t>
+          <t>A small log appears only with the flag, at the top of Today and the foot of the list. Every line is counts, ids and flags. NO task title ever appears in it: these get screenshotted and pasted, and a shared list is two people's words.</t>
         </is>
       </c>
       <c r="G321" s="7" t="inlineStr">
@@ -13574,7 +13574,7 @@
     <row r="322">
       <c r="A322" s="6" t="inlineStr">
         <is>
-          <t>OUR-57</t>
+          <t>OUR-55</t>
         </is>
       </c>
       <c r="B322" s="7" t="inlineStr">
@@ -13582,24 +13582,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C322" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C322" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D322" s="9" t="inlineStr">
         <is>
-          <t>A dump becomes several shared rows, in the order typed</t>
+          <t>Capture on Ours IS Today's capture</t>
         </is>
       </c>
       <c r="E322" s="9" t="inlineStr">
         <is>
-          <t>Type three lines into the Ours capture and Add.</t>
+          <t>Open a shared list and tap the launcher at the foot of the screen.</t>
         </is>
       </c>
       <c r="F322" s="9" t="inlineStr">
         <is>
-          <t>The button reads 'Add 3' and three rows land, in the typed order, on both devices. With a cadence set, all three carry it.</t>
+          <t>The same panel Today opens: the same input, the same Speak button (web), the same door, the same Add button naming its own consequence. Not a lookalike, the same component, so the two can never drift apart.</t>
         </is>
       </c>
       <c r="G322" s="7" t="inlineStr">
@@ -13614,7 +13614,7 @@
     <row r="323">
       <c r="A323" s="6" t="inlineStr">
         <is>
-          <t>OUR-58</t>
+          <t>OUR-56</t>
         </is>
       </c>
       <c r="B323" s="7" t="inlineStr">
@@ -13629,17 +13629,17 @@
       </c>
       <c r="D323" s="9" t="inlineStr">
         <is>
-          <t>The shared door offers When and Repeating, never Steps</t>
+          <t>Repeating can be set AT capture, without knowing a gesture</t>
         </is>
       </c>
       <c r="E323" s="9" t="inlineStr">
         <is>
-          <t>Open the door on Ours and compare it with the door on Today.</t>
+          <t>In that panel, open the door and choose Daily (or Weekly, or Every N days), then Add.</t>
         </is>
       </c>
       <c r="F323" s="9" t="inlineStr">
         <is>
-          <t>Ours shows a When row and a Repeating row, and NO Steps row (a shared row has no slices field, and breaking a thing down is personal). The When row is deliberate: a dated or repeating shared row now reaches BOTH Todays, so a day here is a real act rather than a word that means nothing. See OUR-71 for what the When row rests on.</t>
+          <t>The button reads 'Add · Daily' before the tap, and the row lands already repeating, visible to both of you. (Before this, the only way to make a repeating shared task was to add it and then somehow know to long-press it. Melroy: 'there is no way to add Repeating Tasks.')</t>
         </is>
       </c>
       <c r="G323" s="7" t="inlineStr">
@@ -13654,7 +13654,7 @@
     <row r="324">
       <c r="A324" s="6" t="inlineStr">
         <is>
-          <t>OUR-59</t>
+          <t>OUR-57</t>
         </is>
       </c>
       <c r="B324" s="7" t="inlineStr">
@@ -13669,17 +13669,17 @@
       </c>
       <c r="D324" s="9" t="inlineStr">
         <is>
-          <t>Typed text survives closing the panel</t>
+          <t>A dump becomes several shared rows, in the order typed</t>
         </is>
       </c>
       <c r="E324" s="9" t="inlineStr">
         <is>
-          <t>Type half a sentence into the Ours capture, tap Close, tick something, then reopen the panel.</t>
+          <t>Type three lines into the Ours capture and Add.</t>
         </is>
       </c>
       <c r="F324" s="9" t="inlineStr">
         <is>
-          <t>The half sentence is still there. The panel is hidden, never unmounted. The door resets to no-repeat, the words never reset.</t>
+          <t>The button reads 'Add 3' and three rows land, in the typed order, on both devices. With a cadence set, all three carry it.</t>
         </is>
       </c>
       <c r="G324" s="7" t="inlineStr">
@@ -13694,7 +13694,7 @@
     <row r="325">
       <c r="A325" s="6" t="inlineStr">
         <is>
-          <t>OUR-60</t>
+          <t>OUR-58</t>
         </is>
       </c>
       <c r="B325" s="7" t="inlineStr">
@@ -13702,29 +13702,29 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C325" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C325" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D325" s="9" t="inlineStr">
         <is>
-          <t>The Ours capture rides above the keyboard</t>
+          <t>The shared door offers When and Repeating, never Steps</t>
         </is>
       </c>
       <c r="E325" s="9" t="inlineStr">
         <is>
-          <t>On a real Android device, open the Ours capture and start typing.</t>
+          <t>Open the door on Ours and compare it with the door on Today.</t>
         </is>
       </c>
       <c r="F325" s="9" t="inlineStr">
         <is>
-          <t>The panel and its Add button stay visible above the keyboard. Nothing on this stack does this by itself (edge-to-edge Android ignores softwareKeyboardLayoutMode), so it is done by hand and must be re-checked on a device, never only in a browser.</t>
+          <t>Ours shows a When row and a Repeating row, and NO Steps row (a shared row has no slices field, and breaking a thing down is personal). The When row is deliberate: a dated or repeating shared row now reaches BOTH Todays, so a day here is a real act rather than a word that means nothing. See OUR-71 for what the When row rests on.</t>
         </is>
       </c>
       <c r="G325" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H325" s="7" t="inlineStr"/>
@@ -13734,7 +13734,7 @@
     <row r="326">
       <c r="A326" s="6" t="inlineStr">
         <is>
-          <t>OUR-61</t>
+          <t>OUR-59</t>
         </is>
       </c>
       <c r="B326" s="7" t="inlineStr">
@@ -13742,24 +13742,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C326" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C326" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D326" s="9" t="inlineStr">
         <is>
-          <t>No AI on the shared capture</t>
+          <t>Typed text survives closing the panel</t>
         </is>
       </c>
       <c r="E326" s="9" t="inlineStr">
         <is>
-          <t>Open the Ours capture with AI enabled in Settings.</t>
+          <t>Type half a sentence into the Ours capture, tap Close, tick something, then reopen the panel.</t>
         </is>
       </c>
       <c r="F326" s="9" t="inlineStr">
         <is>
-          <t>No 'Break it down' and no 'Sort for me': steps a model proposes would land on a list another person reads, and pointing a model at somebody else's screen is a decision about them. Speak stays (on-device dictation, not a server call) and so does Scan, which reads a photo INTO the box for you to edit rather than authoring anything, and is the one AI action that belongs here. See OUR-62.</t>
+          <t>The half sentence is still there. The panel is hidden, never unmounted. The door resets to no-repeat, the words never reset.</t>
         </is>
       </c>
       <c r="G326" s="7" t="inlineStr">
@@ -13774,7 +13774,7 @@
     <row r="327">
       <c r="A327" s="6" t="inlineStr">
         <is>
-          <t>OUR-62</t>
+          <t>OUR-60</t>
         </is>
       </c>
       <c r="B327" s="7" t="inlineStr">
@@ -13782,24 +13782,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C327" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C327" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D327" s="9" t="inlineStr">
         <is>
-          <t>Scan (premium) reaches the shared capture</t>
+          <t>The Ours capture rides above the keyboard</t>
         </is>
       </c>
       <c r="E327" s="9" t="inlineStr">
         <is>
-          <t>Premium, AI enabled in Settings. Open the Ours capture on a phone. Tap Scan and photograph a handwritten shopping list.</t>
+          <t>On a real Android device, open the Ours capture and start typing.</t>
         </is>
       </c>
       <c r="F327" s="9" t="inlineStr">
         <is>
-          <t>The words land IN the capture box, not on the list. You read them, edit them, and Add them yourself. This is the surface Scan most belongs on: the most photographed list anybody owns is the one on the fridge, and that list is shared by definition.</t>
+          <t>The panel and its Add button stay visible above the keyboard. Nothing on this stack does this by itself (edge-to-edge Android ignores softwareKeyboardLayoutMode), so it is done by hand and must be re-checked on a device, never only in a browser.</t>
         </is>
       </c>
       <c r="G327" s="7" t="inlineStr">
@@ -13814,7 +13814,7 @@
     <row r="328">
       <c r="A328" s="6" t="inlineStr">
         <is>
-          <t>OUR-63</t>
+          <t>OUR-61</t>
         </is>
       </c>
       <c r="B328" s="7" t="inlineStr">
@@ -13822,24 +13822,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C328" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C328" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D328" s="9" t="inlineStr">
         <is>
-          <t>Scan on Ours meets the paywall, tagged apart from Today's</t>
+          <t>No AI on the shared capture</t>
         </is>
       </c>
       <c r="E328" s="9" t="inlineStr">
         <is>
-          <t>Sign in as a NON-premium user, open the Ours capture, tap Scan.</t>
+          <t>Open the Ours capture with AI enabled in Settings.</t>
         </is>
       </c>
       <c r="F328" s="9" t="inlineStr">
         <is>
-          <t>The premium screen opens, the same one Today's Scan opens. Nothing is scanned and nothing is charged. The gate logs reason 'ocr_ours', not 'ocr': a paywall met on a surface a second person can see is a different moment from one met alone.</t>
+          <t>No 'Break it down' and no 'Sort for me': steps a model proposes would land on a list another person reads, and pointing a model at somebody else's screen is a decision about them. Speak stays (on-device dictation, not a server call) and so does Scan, which reads a photo INTO the box for you to edit rather than authoring anything, and is the one AI action that belongs here. See OUR-62.</t>
         </is>
       </c>
       <c r="G328" s="7" t="inlineStr">
@@ -13854,7 +13854,7 @@
     <row r="329">
       <c r="A329" s="6" t="inlineStr">
         <is>
-          <t>OUR-64</t>
+          <t>OUR-62</t>
         </is>
       </c>
       <c r="B329" s="7" t="inlineStr">
@@ -13862,29 +13862,29 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C329" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C329" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D329" s="9" t="inlineStr">
         <is>
-          <t>The photo never reaches the shared list</t>
+          <t>Scan (premium) reaches the shared capture</t>
         </is>
       </c>
       <c r="E329" s="9" t="inlineStr">
         <is>
-          <t>Scan something into Ours and Add it. Check the other device.</t>
+          <t>Premium, AI enabled in Settings. Open the Ours capture on a phone. Tap Scan and photograph a handwritten shopping list.</t>
         </is>
       </c>
       <c r="F329" s="9" t="inlineStr">
         <is>
-          <t>Your person sees the rows you added and nothing else, exactly as if you had typed them. No image is stored anywhere, shared or otherwise: it is sent to be read, then discarded.</t>
+          <t>The words land IN the capture box, not on the list. You read them, edit them, and Add them yourself. This is the surface Scan most belongs on: the most photographed list anybody owns is the one on the fridge, and that list is shared by definition.</t>
         </is>
       </c>
       <c r="G329" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H329" s="7" t="inlineStr"/>
@@ -13894,7 +13894,7 @@
     <row r="330">
       <c r="A330" s="6" t="inlineStr">
         <is>
-          <t>OUR-65</t>
+          <t>OUR-63</t>
         </is>
       </c>
       <c r="B330" s="7" t="inlineStr">
@@ -13902,24 +13902,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C330" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C330" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D330" s="9" t="inlineStr">
         <is>
-          <t>Scan is absent when AI is off</t>
+          <t>Scan on Ours meets the paywall, tagged apart from Today's</t>
         </is>
       </c>
       <c r="E330" s="9" t="inlineStr">
         <is>
-          <t>Turn AI off in Settings, then open the Ours capture.</t>
+          <t>Sign in as a NON-premium user, open the Ours capture, tap Scan.</t>
         </is>
       </c>
       <c r="F330" s="9" t="inlineStr">
         <is>
-          <t>No Scan button, on either screen. Speak stays: it is on-device dictation, not a server call.</t>
+          <t>The premium screen opens, the same one Today's Scan opens. Nothing is scanned and nothing is charged. The gate logs reason 'ocr_ours', not 'ocr': a paywall met on a surface a second person can see is a different moment from one met alone.</t>
         </is>
       </c>
       <c r="G330" s="7" t="inlineStr">
@@ -13934,7 +13934,7 @@
     <row r="331">
       <c r="A331" s="6" t="inlineStr">
         <is>
-          <t>OUR-66</t>
+          <t>OUR-64</t>
         </is>
       </c>
       <c r="B331" s="7" t="inlineStr">
@@ -13942,24 +13942,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C331" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C331" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D331" s="9" t="inlineStr">
         <is>
-          <t>A repeating shared row appears on BOTH Todays on its day</t>
+          <t>The photo never reaches the shared list</t>
         </is>
       </c>
       <c r="E331" s="9" t="inlineStr">
         <is>
-          <t>Make a shared task repeat weekly on today's weekday. Open Today on both devices.</t>
+          <t>Scan something into Ours and Add it. Check the other device.</t>
         </is>
       </c>
       <c r="F331" s="9" t="inlineStr">
         <is>
-          <t>It appears on each Today under a 'From Ours' heading, below the day's own tasks. Neither person had to fetch it. This is the answer to 'I do not want to manually decide what gets added to my list for today'.</t>
+          <t>Your person sees the rows you added and nothing else, exactly as if you had typed them. No image is stored anywhere, shared or otherwise: it is sent to be read, then discarded.</t>
         </is>
       </c>
       <c r="G331" s="7" t="inlineStr">
@@ -13974,7 +13974,7 @@
     <row r="332">
       <c r="A332" s="6" t="inlineStr">
         <is>
-          <t>OUR-67</t>
+          <t>OUR-65</t>
         </is>
       </c>
       <c r="B332" s="7" t="inlineStr">
@@ -13982,24 +13982,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C332" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C332" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D332" s="9" t="inlineStr">
         <is>
-          <t>An UNDATED shared row never reaches Today</t>
+          <t>Scan is absent when AI is off</t>
         </is>
       </c>
       <c r="E332" s="9" t="inlineStr">
         <is>
-          <t>Add an ordinary shared task with the door left on Anytime. Check Today on both devices.</t>
+          <t>Turn AI off in Settings, then open the Ours capture.</t>
         </is>
       </c>
       <c r="F332" s="9" t="inlineStr">
         <is>
-          <t>It is in the room and NOWHERE on Today. This is the load-bearing rule: without it, your person adding eight things to the shopping list makes your morning eight heavier without you agreeing to any of it.</t>
+          <t>No Scan button, on either screen. Speak stays: it is on-device dictation, not a server call.</t>
         </is>
       </c>
       <c r="G332" s="7" t="inlineStr">
@@ -14014,7 +14014,7 @@
     <row r="333">
       <c r="A333" s="6" t="inlineStr">
         <is>
-          <t>OUR-68</t>
+          <t>OUR-66</t>
         </is>
       </c>
       <c r="B333" s="7" t="inlineStr">
@@ -14029,17 +14029,17 @@
       </c>
       <c r="D333" s="9" t="inlineStr">
         <is>
-          <t>Shared rows never make the day look heavier</t>
+          <t>A repeating shared row appears on BOTH Todays on its day</t>
         </is>
       </c>
       <c r="E333" s="9" t="inlineStr">
         <is>
-          <t>With several shared rows showing on Today, check the weight gauge, Plan my day, Lighten, and the close-the-day count.</t>
+          <t>Make a shared task repeat weekly on today's weekday. Open Today on both devices.</t>
         </is>
       </c>
       <c r="F333" s="9" t="inlineStr">
         <is>
-          <t>All of them ignore the shared rows entirely. They are not in `tasks`, so they cannot reach any of it by construction. The day the app promises is finite stays finite.</t>
+          <t>It appears on each Today under a 'From Ours' heading, below the day's own tasks. Neither person had to fetch it. This is the answer to 'I do not want to manually decide what gets added to my list for today'.</t>
         </is>
       </c>
       <c r="G333" s="7" t="inlineStr">
@@ -14054,7 +14054,7 @@
     <row r="334">
       <c r="A334" s="6" t="inlineStr">
         <is>
-          <t>OUR-69</t>
+          <t>OUR-67</t>
         </is>
       </c>
       <c r="B334" s="7" t="inlineStr">
@@ -14069,17 +14069,17 @@
       </c>
       <c r="D334" s="9" t="inlineStr">
         <is>
-          <t>Ticking a shared row from Today closes it for both</t>
+          <t>An UNDATED shared row never reaches Today</t>
         </is>
       </c>
       <c r="E334" s="9" t="inlineStr">
         <is>
-          <t>Tick a row in the From Ours strip on device A. Look at device B's Ours list and Today.</t>
+          <t>Add an ordinary shared task with the door left on Anytime. Check Today on both devices.</t>
         </is>
       </c>
       <c r="F334" s="9" t="inlineStr">
         <is>
-          <t>Done on both, within a poll. Nothing anywhere says who did it, and neither room tints it as a stranger's change on the device that did it (noteOursMine).</t>
+          <t>It is in the room and NOWHERE on Today. This is the load-bearing rule: without it, your person adding eight things to the shopping list makes your morning eight heavier without you agreeing to any of it.</t>
         </is>
       </c>
       <c r="G334" s="7" t="inlineStr">
@@ -14094,7 +14094,7 @@
     <row r="335">
       <c r="A335" s="6" t="inlineStr">
         <is>
-          <t>OUR-70</t>
+          <t>OUR-68</t>
         </is>
       </c>
       <c r="B335" s="7" t="inlineStr">
@@ -14102,24 +14102,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C335" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C335" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D335" s="9" t="inlineStr">
         <is>
-          <t>A dated shared row shows from its day onward, never before</t>
+          <t>Shared rows never make the day look heavier</t>
         </is>
       </c>
       <c r="E335" s="9" t="inlineStr">
         <is>
-          <t>Add a shared task with the door set to a date two days out. Check Today now, then on the day.</t>
+          <t>With several shared rows showing on Today, check the weight gauge, Plan my day, Lighten, and the close-the-day count.</t>
         </is>
       </c>
       <c r="F335" s="9" t="inlineStr">
         <is>
-          <t>Absent today, present on the day and on any day after (a shared thing nobody did does not stop being one). The room shows its date on the row all along, so it is never a surprise.</t>
+          <t>All of them ignore the shared rows entirely. They are not in `tasks`, so they cannot reach any of it by construction. The day the app promises is finite stays finite.</t>
         </is>
       </c>
       <c r="G335" s="7" t="inlineStr">
@@ -14134,7 +14134,7 @@
     <row r="336">
       <c r="A336" s="6" t="inlineStr">
         <is>
-          <t>OUR-71</t>
+          <t>OUR-69</t>
         </is>
       </c>
       <c r="B336" s="7" t="inlineStr">
@@ -14149,17 +14149,17 @@
       </c>
       <c r="D336" s="9" t="inlineStr">
         <is>
-          <t>The shared capture rests on Anytime</t>
+          <t>Ticking a shared row from Today closes it for both</t>
         </is>
       </c>
       <c r="E336" s="9" t="inlineStr">
         <is>
-          <t>Open the Ours capture and open the door.</t>
+          <t>Tick a row in the From Ours strip on device A. Look at device B's Ours list and Today.</t>
         </is>
       </c>
       <c r="F336" s="9" t="inlineStr">
         <is>
-          <t>The When row reads Anytime / Today / Tomorrow / Pick a date, with Anytime selected. The Add button says just 'Add'. Choosing Today makes it read 'Add . Today', because that is the notable case: it will appear on both your days.</t>
+          <t>Done on both, within a poll. Nothing anywhere says who did it, and neither room tints it as a stranger's change on the device that did it (noteOursMine).</t>
         </is>
       </c>
       <c r="G336" s="7" t="inlineStr">
@@ -14174,7 +14174,7 @@
     <row r="337">
       <c r="A337" s="6" t="inlineStr">
         <is>
-          <t>OUR-112</t>
+          <t>OUR-70</t>
         </is>
       </c>
       <c r="B337" s="7" t="inlineStr">
@@ -14182,24 +14182,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C337" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C337" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D337" s="9" t="inlineStr">
         <is>
-          <t>A shared row's WHEN can be changed, and cleared</t>
+          <t>A dated shared row shows from its day onward, never before</t>
         </is>
       </c>
       <c r="E337" s="9" t="inlineStr">
         <is>
-          <t>In the room, hold a row. The door reads 'When…' with the row's current answer beside it. Open it. Set a date, Set. Reopen, pick a different date, Set. Reopen, tap Anytime, Set.</t>
+          <t>Add a shared task with the door set to a date two days out. Check Today now, then on the day.</t>
         </is>
       </c>
       <c r="F337" s="9" t="inlineStr">
         <is>
-          <t>All three land: date set, date CHANGED, and back to plain. Changing a date and getting back to a plain row were both impossible before this; remove-and-recreate was the only way out, and on a repeat that ends the series for both people. The button always names the outcome ('Set . Thu 20 Aug', 'Set . Anytime'), never 'Save'.</t>
+          <t>Absent today, present on the day and on any day after (a shared thing nobody did does not stop being one). The room shows its date on the row all along, so it is never a surprise.</t>
         </is>
       </c>
       <c r="G337" s="7" t="inlineStr">
@@ -14214,7 +14214,7 @@
     <row r="338">
       <c r="A338" s="6" t="inlineStr">
         <is>
-          <t>OUR-113</t>
+          <t>OUR-71</t>
         </is>
       </c>
       <c r="B338" s="7" t="inlineStr">
@@ -14229,17 +14229,17 @@
       </c>
       <c r="D338" s="9" t="inlineStr">
         <is>
-          <t>Ending a rhythm does NOT mark the row done for both people</t>
+          <t>The shared capture rests on Anytime</t>
         </is>
       </c>
       <c r="E338" s="9" t="inlineStr">
         <is>
-          <t>Make a shared row repeat weekly and tick it on one of its days, on either device. Then hold it, open When…, tap the selected rhythm chip to release it, choose Anytime, and Set. Watch BOTH devices.</t>
+          <t>Open the Ours capture and open the door.</t>
         </is>
       </c>
       <c r="F338" s="9" t="inlineStr">
         <is>
-          <t>The row goes plain and stays UN-ticked on both. It must not come back done. A repeat's ticks live per-date in a completion log and the row's own done flag stays false; the moment the recurrence goes, the merge would read that same log as a one-off's tick and mark the row finished, for both people, with a doneAt from whenever it was last ticked. Try it for a DATED ending too (release the rhythm, pick a day): that path feels least like an ending and is the easiest to get wrong.</t>
+          <t>The When row reads Anytime / Today / Tomorrow / Pick a date, with Anytime selected. The Add button says just 'Add'. Choosing Today makes it read 'Add . Today', because that is the notable case: it will appear on both your days.</t>
         </is>
       </c>
       <c r="G338" s="7" t="inlineStr">
@@ -14254,7 +14254,7 @@
     <row r="339">
       <c r="A339" s="6" t="inlineStr">
         <is>
-          <t>OUR-114</t>
+          <t>OUR-112</t>
         </is>
       </c>
       <c r="B339" s="7" t="inlineStr">
@@ -14262,24 +14262,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C339" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C339" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D339" s="9" t="inlineStr">
         <is>
-          <t>The day zone changes its question when a rhythm is alive</t>
+          <t>A shared row's WHEN can be changed, and cleared</t>
         </is>
       </c>
       <c r="E339" s="9" t="inlineStr">
         <is>
-          <t>In the room, hold a row and open When…. With no rhythm selected, read the label above the day chips. Now tap Daily. Read it again. Then tap Anytime.</t>
+          <t>In the room, hold a row. The door reads 'When…' with the row's current answer beside it. Open it. Set a date, Set. Reopen, pick a different date, Set. Reopen, tap Anytime, Set.</t>
         </is>
       </c>
       <c r="F339" s="9" t="inlineStr">
         <is>
-          <t>It reads 'A day' with no rhythm, and relabels to 'Starting' the moment one is selected, in the accent colour. The same chips now mean 'from when' rather than 'which day'. Anytime stays available throughout, and ONE tap on it ends the rhythm: the label goes back to 'A day' and the summary says 'The rhythm ends.' before anything commits. Tapping the selected rhythm chip releases it too, for anyone who finds that natural, and both routes land in exactly the same place.</t>
+          <t>All three land: date set, date CHANGED, and back to plain. Changing a date and getting back to a plain row were both impossible before this; remove-and-recreate was the only way out, and on a repeat that ends the series for both people. The button always names the outcome ('Set . Thu 20 Aug', 'Set . Anytime'), never 'Save'.</t>
         </is>
       </c>
       <c r="G339" s="7" t="inlineStr">
@@ -14294,7 +14294,7 @@
     <row r="340">
       <c r="A340" s="6" t="inlineStr">
         <is>
-          <t>OUR-115</t>
+          <t>OUR-113</t>
         </is>
       </c>
       <c r="B340" s="7" t="inlineStr">
@@ -14302,24 +14302,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C340" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C340" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D340" s="9" t="inlineStr">
         <is>
-          <t>Setting a shared row to Today actually reaches both Todays</t>
+          <t>Ending a rhythm does NOT mark the row done for both people</t>
         </is>
       </c>
       <c r="E340" s="9" t="inlineStr">
         <is>
-          <t>In the room, hold a plain row, open When…, tap Today, and Set. Check BOTH Todays (look away and back on each).</t>
+          <t>Make a shared row repeat weekly and tick it on one of its days, on either device. Then hold it, open When…, tap the selected rhythm chip to release it, choose Anytime, and Set. Watch BOTH devices.</t>
         </is>
       </c>
       <c r="F340" s="9" t="inlineStr">
         <is>
-          <t>It appears under DUE TODAY on both. The line in the sheet reads 'Today . &lt;the date&gt;' on purpose: a shared row with no date reaches nobody, so Today has to write a real date rather than 'no date', which is the same bug that once shipped on the shared capture bar above this sheet.</t>
+          <t>The row goes plain and stays UN-ticked on both. It must not come back done. A repeat's ticks live per-date in a completion log and the row's own done flag stays false; the moment the recurrence goes, the merge would read that same log as a one-off's tick and mark the row finished, for both people, with a doneAt from whenever it was last ticked. Try it for a DATED ending too (release the rhythm, pick a day): that path feels least like an ending and is the easiest to get wrong.</t>
         </is>
       </c>
       <c r="G340" s="7" t="inlineStr">
@@ -14334,7 +14334,7 @@
     <row r="341">
       <c r="A341" s="6" t="inlineStr">
         <is>
-          <t>OUR-116</t>
+          <t>OUR-114</t>
         </is>
       </c>
       <c r="B341" s="7" t="inlineStr">
@@ -14342,24 +14342,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C341" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C341" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D341" s="9" t="inlineStr">
         <is>
-          <t>An idle Set does not wash the row on the other device</t>
+          <t>The day zone changes its question when a rhythm is alive</t>
         </is>
       </c>
       <c r="E341" s="9" t="inlineStr">
         <is>
-          <t>On A, hold a row, open When…, change nothing, and tap Set. On B, leave the room and come back.</t>
+          <t>In the room, hold a row and open When…. With no rhythm selected, read the label above the day chips. Now tap Daily. Read it again. Then tap Anytime.</t>
         </is>
       </c>
       <c r="F341" s="9" t="inlineStr">
         <is>
-          <t>No 'changed since you looked' mark on B. Every write stamps the row, and a fresh stamp is exactly what the other person's screen reads as a change, so a Set that altered nothing would send them hunting for something nobody did.</t>
+          <t>It reads 'A day' with no rhythm, and relabels to 'Starting' the moment one is selected, in the accent colour. The same chips now mean 'from when' rather than 'which day'. Anytime stays available throughout, and ONE tap on it ends the rhythm: the label goes back to 'A day' and the summary says 'The rhythm ends.' before anything commits. Tapping the selected rhythm chip releases it too, for anyone who finds that natural, and both routes land in exactly the same place.</t>
         </is>
       </c>
       <c r="G341" s="7" t="inlineStr">
@@ -14374,7 +14374,7 @@
     <row r="342">
       <c r="A342" s="6" t="inlineStr">
         <is>
-          <t>OUR-118</t>
+          <t>OUR-115</t>
         </is>
       </c>
       <c r="B342" s="7" t="inlineStr">
@@ -14382,24 +14382,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C342" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C342" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D342" s="9" t="inlineStr">
         <is>
-          <t>A repeat you have already done today keeps its held card</t>
+          <t>Setting a shared row to Today actually reaches both Todays</t>
         </is>
       </c>
       <c r="E342" s="9" t="inlineStr">
         <is>
-          <t>In the room, make a row repeat on TODAY's weekday, then tick it. Now hold it.</t>
+          <t>In the room, hold a plain row, open When…, tap Today, and Set. Check BOTH Todays (look away and back on each).</t>
         </is>
       </c>
       <c r="F342" s="9" t="inlineStr">
         <is>
-          <t>The card still offers When… with its rhythm beside it, and it does NOT say 'Done is done.' A repeat is not a finished thing: it comes back, so the day you did it is exactly a day you might want to move it. Before this, ticking a repeat took its whole held card away until the next day, which put the When editor out of reach on the rows most likely to need it. A finished ONE-OFF still gets the minimal card, which is correct.</t>
+          <t>It appears under DUE TODAY on both. The line in the sheet reads 'Today . &lt;the date&gt;' on purpose: a shared row with no date reaches nobody, so Today has to write a real date rather than 'no date', which is the same bug that once shipped on the shared capture bar above this sheet.</t>
         </is>
       </c>
       <c r="G342" s="7" t="inlineStr">
@@ -14414,7 +14414,7 @@
     <row r="343">
       <c r="A343" s="6" t="inlineStr">
         <is>
-          <t>OUR-117</t>
+          <t>OUR-116</t>
         </is>
       </c>
       <c r="B343" s="7" t="inlineStr">
@@ -14422,24 +14422,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C343" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C343" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D343" s="9" t="inlineStr">
         <is>
-          <t>The Repeating drawer is untouched by the When editor</t>
+          <t>An idle Set does not wash the row on the other device</t>
         </is>
       </c>
       <c r="E343" s="9" t="inlineStr">
         <is>
-          <t>Menu -&gt; Repeating -&gt; Edit on any series. Compare with before.</t>
+          <t>On A, hold a row, open When…, change nothing, and tap Set. On B, leave the room and come back.</t>
         </is>
       </c>
       <c r="F343" s="9" t="inlineStr">
         <is>
-          <t>Same sheet as always: title, the four cadence chips (Daily / Weekly / Every few days / Monthly), weekday toggles or the stepper or the 1-31 grid, 'Starting from' with its date, and a commit button naming the cadence. NO Anytime chip, NO day zone, and tapping the selected cadence chip does NOT release it. 'No rhythm' there would mean the entry should not exist, which is removal, and removal stays in the drawer.</t>
+          <t>No 'changed since you looked' mark on B. Every write stamps the row, and a fresh stamp is exactly what the other person's screen reads as a change, so a Set that altered nothing would send them hunting for something nobody did.</t>
         </is>
       </c>
       <c r="G343" s="7" t="inlineStr">
@@ -14454,7 +14454,7 @@
     <row r="344">
       <c r="A344" s="6" t="inlineStr">
         <is>
-          <t>OUR-119</t>
+          <t>OUR-118</t>
         </is>
       </c>
       <c r="B344" s="7" t="inlineStr">
@@ -14462,24 +14462,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C344" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C344" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D344" s="9" t="inlineStr">
         <is>
-          <t>Monthly works on a shared row, and an out-of-date partner still sees the rhythm</t>
+          <t>A repeat you have already done today keeps its held card</t>
         </is>
       </c>
       <c r="E344" s="9" t="inlineStr">
         <is>
-          <t>On Ours, hold a row and tap 'Repeat…'. Choose Monthly and a day. Read the summary, commit, then look at the row and at both Todays on that day. If a partner is on an older build (1.3.1 or earlier), have them look at the same row.</t>
+          <t>In the room, make a row repeat on TODAY's weekday, then tick it. Now hold it.</t>
         </is>
       </c>
       <c r="F344" s="9" t="inlineStr">
         <is>
-          <t>Monthly is the fourth rhythm chip here too, from the same sheet the personal drawer uses, so a shared monthly row and a personal one are identical in shape. The summary reads 'Every month on the 15th · from {start}' and the commit button names it. The row lands on BOTH Todays on that day. A partner whose build predates monthly cannot compute the days, so their app shows the row with the plain-English line the writing client left alongside the rhythm rather than showing a repeating row with no rhythm at all. What it must never do is HIDE the row: one person seeing a task the other does not is the invisible disagreement this whole feature exists to prevent.</t>
+          <t>The card still offers When… with its rhythm beside it, and it does NOT say 'Done is done.' A repeat is not a finished thing: it comes back, so the day you did it is exactly a day you might want to move it. Before this, ticking a repeat took its whole held card away until the next day, which put the When editor out of reach on the rows most likely to need it. A finished ONE-OFF still gets the minimal card, which is correct.</t>
         </is>
       </c>
       <c r="G344" s="7" t="inlineStr">
@@ -14494,7 +14494,7 @@
     <row r="345">
       <c r="A345" s="6" t="inlineStr">
         <is>
-          <t>OUR-111</t>
+          <t>OUR-117</t>
         </is>
       </c>
       <c r="B345" s="7" t="inlineStr">
@@ -14502,24 +14502,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C345" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C345" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D345" s="9" t="inlineStr">
         <is>
-          <t>A finished dated shared row leaves both Todays the next day</t>
+          <t>The Repeating drawer is untouched by the When editor</t>
         </is>
       </c>
       <c r="E345" s="9" t="inlineStr">
         <is>
-          <t>Give a shared row today's date so it appears under DUE TODAY on both phones. Tick it on either phone. Look at both Todays now, then again tomorrow (or move a device's clock forward a day and reopen).</t>
+          <t>Menu -&gt; Repeating -&gt; Edit on any series. Compare with before.</t>
         </is>
       </c>
       <c r="F345" s="9" t="inlineStr">
         <is>
-          <t>Today: still there on BOTH, struck through, and un-tickable again, because ticking is the reversible act on this list. Tomorrow: gone from both. It must not accumulate. Before this rule the strip kept every dated row either of you had ever ticked, for good, on a screen excluded from the weight gauge and the close-the-day count, whose whole premise is that a day is finite. Check the other half too: an UNFINISHED row with a past date is still there tomorrow, which is correct and is not shaming.</t>
+          <t>Same sheet as always: title, the four cadence chips (Daily / Weekly / Every few days / Monthly), weekday toggles or the stepper or the 1-31 grid, 'Starting from' with its date, and a commit button naming the cadence. NO Anytime chip, NO day zone, and tapping the selected cadence chip does NOT release it. 'No rhythm' there would mean the entry should not exist, which is removal, and removal stays in the drawer.</t>
         </is>
       </c>
       <c r="G345" s="7" t="inlineStr">
@@ -14534,7 +14534,7 @@
     <row r="346">
       <c r="A346" s="6" t="inlineStr">
         <is>
-          <t>OUR-72</t>
+          <t>OUR-119</t>
         </is>
       </c>
       <c r="B346" s="7" t="inlineStr">
@@ -14549,17 +14549,17 @@
       </c>
       <c r="D346" s="9" t="inlineStr">
         <is>
-          <t>A repeat supersedes the day rather than joining it</t>
+          <t>Monthly works on a shared row, and an out-of-date partner still sees the rhythm</t>
         </is>
       </c>
       <c r="E346" s="9" t="inlineStr">
         <is>
-          <t>On the Ours capture, set a Daily repeat with When left on Anytime.</t>
+          <t>On Ours, hold a row and tap 'Repeat…'. Choose Monthly and a day. Read the summary, commit, then look at the row and at both Todays on that day. If a partner is on an older build (1.3.1 or earlier), have them look at the same row.</t>
         </is>
       </c>
       <c r="F346" s="9" t="inlineStr">
         <is>
-          <t>The door summary reads 'Daily', not 'Anytime . Daily'. On Today's own capture it still reads 'Today . Daily', where the when genuinely IS the repeat's start.</t>
+          <t>Monthly is the fourth rhythm chip here too, from the same sheet the personal drawer uses, so a shared monthly row and a personal one are identical in shape. The summary reads 'Every month on the 15th · from {start}' and the commit button names it. The row lands on BOTH Todays on that day. A partner whose build predates monthly cannot compute the days, so their app shows the row with the plain-English line the writing client left alongside the rhythm rather than showing a repeating row with no rhythm at all. What it must never do is HIDE the row: one person seeing a task the other does not is the invisible disagreement this whole feature exists to prevent.</t>
         </is>
       </c>
       <c r="G346" s="7" t="inlineStr">
@@ -14574,7 +14574,7 @@
     <row r="347">
       <c r="A347" s="6" t="inlineStr">
         <is>
-          <t>OUR-73</t>
+          <t>OUR-111</t>
         </is>
       </c>
       <c r="B347" s="7" t="inlineStr">
@@ -14582,24 +14582,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C347" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C347" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D347" s="9" t="inlineStr">
         <is>
-          <t>An unreadable cadence is never placed on a day</t>
+          <t>A finished dated shared row leaves both Todays the next day</t>
         </is>
       </c>
       <c r="E347" s="9" t="inlineStr">
         <is>
-          <t>Have a newer build write a cadence this build cannot parse, then open Today.</t>
+          <t>Give a shared row today's date so it appears under DUE TODAY on both phones. Tick it on either phone. Look at both Todays now, then again tomorrow (or move a device's clock forward a day and reopen).</t>
         </is>
       </c>
       <c r="F347" s="9" t="inlineStr">
         <is>
-          <t>It shows in the room (never invisible to the person who set it) and appears on NO Today. This build cannot know which days it means, and a wrong day on a shared surface is a thing the other person has to puzzle over.</t>
+          <t>Today: still there on BOTH, struck through, and un-tickable again, because ticking is the reversible act on this list. Tomorrow: gone from both. It must not accumulate. Before this rule the strip kept every dated row either of you had ever ticked, for good, on a screen excluded from the weight gauge and the close-the-day count, whose whole premise is that a day is finite. Check the other half too: an UNFINISHED row with a past date is still there tomorrow, which is correct and is not shaming.</t>
         </is>
       </c>
       <c r="G347" s="7" t="inlineStr">
@@ -14614,7 +14614,7 @@
     <row r="348">
       <c r="A348" s="6" t="inlineStr">
         <is>
-          <t>OUR-74</t>
+          <t>OUR-72</t>
         </is>
       </c>
       <c r="B348" s="7" t="inlineStr">
@@ -14622,24 +14622,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C348" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C348" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D348" s="9" t="inlineStr">
         <is>
-          <t>The door says what changed since you looked, and clears when you look</t>
+          <t>A repeat supersedes the day rather than joining it</t>
         </is>
       </c>
       <c r="E348" s="9" t="inlineStr">
         <is>
-          <t>Device B changes something on the shared list. On device A, open Today WITHOUT visiting Ours. Then tap through to Ours and come back.</t>
+          <t>On the Ours capture, set a Daily repeat with When left on Anytime.</t>
         </is>
       </c>
       <c r="F348" s="9" t="inlineStr">
         <is>
-          <t>The Ours door reads '1 since you looked'. After visiting, it is gone. The number is bounded by your own attention, not by the list's length, so it can never sit there climbing at you.</t>
+          <t>The door summary reads 'Daily', not 'Anytime . Daily'. On Today's own capture it still reads 'Today . Daily', where the when genuinely IS the repeat's start.</t>
         </is>
       </c>
       <c r="G348" s="7" t="inlineStr">
@@ -14654,7 +14654,7 @@
     <row r="349">
       <c r="A349" s="6" t="inlineStr">
         <is>
-          <t>OUR-75</t>
+          <t>OUR-73</t>
         </is>
       </c>
       <c r="B349" s="7" t="inlineStr">
@@ -14662,24 +14662,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C349" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C349" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D349" s="9" t="inlineStr">
         <is>
-          <t>Your OWN changes never appear in that count</t>
+          <t>An unreadable cadence is never placed on a day</t>
         </is>
       </c>
       <c r="E349" s="9" t="inlineStr">
         <is>
-          <t>On device A, add or tick several shared rows. Go to Today on the SAME device.</t>
+          <t>Have a newer build write a cadence this build cannot parse, then open Today.</t>
         </is>
       </c>
       <c r="F349" s="9" t="inlineStr">
         <is>
-          <t>No count on the door. It uses the room's own wash arithmetic, so the door and the room always agree about whose change it was.</t>
+          <t>It shows in the room (never invisible to the person who set it) and appears on NO Today. This build cannot know which days it means, and a wrong day on a shared surface is a thing the other person has to puzzle over.</t>
         </is>
       </c>
       <c r="G349" s="7" t="inlineStr">
@@ -14694,7 +14694,7 @@
     <row r="350">
       <c r="A350" s="6" t="inlineStr">
         <is>
-          <t>OUR-76</t>
+          <t>OUR-74</t>
         </is>
       </c>
       <c r="B350" s="7" t="inlineStr">
@@ -14702,24 +14702,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C350" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C350" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D350" s="9" t="inlineStr">
         <is>
-          <t>A first-ever visit counts nothing</t>
+          <t>The door says what changed since you looked, and clears when you look</t>
         </is>
       </c>
       <c r="E350" s="9" t="inlineStr">
         <is>
-          <t>Pair two accounts, put rows on the list from device B, and open Today on a device A that has never opened the room.</t>
+          <t>Device B changes something on the shared list. On device A, open Today WITHOUT visiting Ours. Then tap through to Ours and come back.</t>
         </is>
       </c>
       <c r="F350" s="9" t="inlineStr">
         <is>
-          <t>No count. There is no 'last looked' to measure against, and inventing one would open the app with a number already on it.</t>
+          <t>The Ours door reads '1 since you looked'. After visiting, it is gone. The number is bounded by your own attention, not by the list's length, so it can never sit there climbing at you.</t>
         </is>
       </c>
       <c r="G350" s="7" t="inlineStr">
@@ -14734,7 +14734,7 @@
     <row r="351">
       <c r="A351" s="6" t="inlineStr">
         <is>
-          <t>OUR-77</t>
+          <t>OUR-75</t>
         </is>
       </c>
       <c r="B351" s="7" t="inlineStr">
@@ -14742,24 +14742,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C351" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C351" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D351" s="9" t="inlineStr">
         <is>
-          <t>The capture's AI note names only what that surface HAS</t>
+          <t>Your OWN changes never appear in that count</t>
         </is>
       </c>
       <c r="E351" s="9" t="inlineStr">
         <is>
-          <t>Type into the Ours capture, then into Today's, and read the line under the buttons.</t>
+          <t>On device A, add or tick several shared rows. Go to Today on the SAME device.</t>
         </is>
       </c>
       <c r="F351" s="9" t="inlineStr">
         <is>
-          <t>Ours says Scan sends your photo. Today says Sort for me, Break it down and Scan send what you type or photograph. Ours must NEVER name Sort for me or Break it down: neither button is there, and a false claim about where your data goes teaches people the disclosure is decorative.</t>
+          <t>No count on the door. It uses the room's own wash arithmetic, so the door and the room always agree about whose change it was.</t>
         </is>
       </c>
       <c r="G351" s="7" t="inlineStr">
@@ -14774,7 +14774,7 @@
     <row r="352">
       <c r="A352" s="6" t="inlineStr">
         <is>
-          <t>OUR-78</t>
+          <t>OUR-76</t>
         </is>
       </c>
       <c r="B352" s="7" t="inlineStr">
@@ -14782,24 +14782,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C352" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C352" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D352" s="9" t="inlineStr">
         <is>
-          <t>Scan discloses on every path that can reach a camera</t>
+          <t>A first-ever visit counts nothing</t>
         </is>
       </c>
       <c r="E352" s="9" t="inlineStr">
         <is>
-          <t>Open Scan on web (gallery picker) and on Android with the camera already allowed.</t>
+          <t>Pair two accounts, put rows on the list from device B, and open Today on a device A that has never opened the room.</t>
         </is>
       </c>
       <c r="F352" s="9" t="inlineStr">
         <is>
-          <t>Both show the egress line. It used to appear only on the Android permission screen, so the two paths a person can reach WITHOUT a prompt sent a photograph having said nothing.</t>
+          <t>No count. There is no 'last looked' to measure against, and inventing one would open the app with a number already on it.</t>
         </is>
       </c>
       <c r="G352" s="7" t="inlineStr">
@@ -14814,7 +14814,7 @@
     <row r="353">
       <c r="A353" s="6" t="inlineStr">
         <is>
-          <t>OUR-79</t>
+          <t>OUR-77</t>
         </is>
       </c>
       <c r="B353" s="7" t="inlineStr">
@@ -14829,17 +14829,17 @@
       </c>
       <c r="D353" s="9" t="inlineStr">
         <is>
-          <t>Press and hold a From Ours row on Today</t>
+          <t>The capture's AI note names only what that surface HAS</t>
         </is>
       </c>
       <c r="E353" s="9" t="inlineStr">
         <is>
-          <t>Hold a row in the From Ours strip.</t>
+          <t>Type into the Ours capture, then into Today's, and read the line under the buttons.</t>
         </is>
       </c>
       <c r="F353" s="9" t="inlineStr">
         <is>
-          <t>The held card opens with Pin and, on a non-repeating row, Move to. Choosing either TAKES THE ROW ON as your own copy: it leaves the strip and joins your day, where the ordinary reorder and the rest of the held card already work.</t>
+          <t>Ours says Scan sends your photo. Today says Sort for me, Break it down and Scan send what you type or photograph. Ours must NEVER name Sort for me or Break it down: neither button is there, and a false claim about where your data goes teaches people the disclosure is decorative.</t>
         </is>
       </c>
       <c r="G353" s="7" t="inlineStr">
@@ -14854,7 +14854,7 @@
     <row r="354">
       <c r="A354" s="6" t="inlineStr">
         <is>
-          <t>OUR-80</t>
+          <t>OUR-78</t>
         </is>
       </c>
       <c r="B354" s="7" t="inlineStr">
@@ -14869,17 +14869,17 @@
       </c>
       <c r="D354" s="9" t="inlineStr">
         <is>
-          <t>Pin and Move-to never rearrange the other person's day</t>
+          <t>Scan discloses on every path that can reach a camera</t>
         </is>
       </c>
       <c r="E354" s="9" t="inlineStr">
         <is>
-          <t>Move a shared row to tomorrow from your Today. Check the other device.</t>
+          <t>Open Scan on web (gallery picker) and on Android with the camera already allowed.</t>
         </is>
       </c>
       <c r="F354" s="9" t="inlineStr">
         <is>
-          <t>YOUR copy moves to tomorrow. The shared row is untouched and still on her day. Applied to the shared row itself this would silently take it off her Wednesday too, on a thing she may have planned around.</t>
+          <t>Both show the egress line. It used to appear only on the Android permission screen, so the two paths a person can reach WITHOUT a prompt sent a photograph having said nothing.</t>
         </is>
       </c>
       <c r="G354" s="7" t="inlineStr">
@@ -14894,7 +14894,7 @@
     <row r="355">
       <c r="A355" s="6" t="inlineStr">
         <is>
-          <t>OUR-81</t>
+          <t>OUR-79</t>
         </is>
       </c>
       <c r="B355" s="7" t="inlineStr">
@@ -14902,24 +14902,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C355" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C355" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D355" s="9" t="inlineStr">
         <is>
-          <t>A taken-on row is never on screen twice</t>
+          <t>Press and hold a From Ours row on Today</t>
         </is>
       </c>
       <c r="E355" s="9" t="inlineStr">
         <is>
-          <t>Take a shared row on (Pin it, or Bring it from the room). Look at Today.</t>
+          <t>Hold a row in the From Ours strip.</t>
         </is>
       </c>
       <c r="F355" s="9" t="inlineStr">
         <is>
-          <t>It appears once, as your task, and NOT also in the From Ours strip. Still true once it is ticked: a finished copy and its finished origin must not both render.</t>
+          <t>The held card opens with Pin and, on a non-repeating row, Move to. Choosing either TAKES THE ROW ON as your own copy: it leaves the strip and joins your day, where the ordinary reorder and the rest of the held card already work.</t>
         </is>
       </c>
       <c r="G355" s="7" t="inlineStr">
@@ -14934,7 +14934,7 @@
     <row r="356">
       <c r="A356" s="6" t="inlineStr">
         <is>
-          <t>OUR-82</t>
+          <t>OUR-80</t>
         </is>
       </c>
       <c r="B356" s="7" t="inlineStr">
@@ -14942,24 +14942,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C356" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C356" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D356" s="9" t="inlineStr">
         <is>
-          <t>Move-to is not offered on a repeating shared row</t>
+          <t>Pin and Move-to never rearrange the other person's day</t>
         </is>
       </c>
       <c r="E356" s="9" t="inlineStr">
         <is>
-          <t>Hold a repeating row in the From Ours strip.</t>
+          <t>Move a shared row to tomorrow from your Today. Check the other device.</t>
         </is>
       </c>
       <c r="F356" s="9" t="inlineStr">
         <is>
-          <t>Pin is there, Move to is not. A date and a rhythm are alternatives, and rescheduling a series is a question for the room's cadence sheet, not a one-tap action on a day.</t>
+          <t>YOUR copy moves to tomorrow. The shared row is untouched and still on her day. Applied to the shared row itself this would silently take it off her Wednesday too, on a thing she may have planned around.</t>
         </is>
       </c>
       <c r="G356" s="7" t="inlineStr">
@@ -14974,7 +14974,7 @@
     <row r="357">
       <c r="A357" s="6" t="inlineStr">
         <is>
-          <t>OUR-83</t>
+          <t>OUR-81</t>
         </is>
       </c>
       <c r="B357" s="7" t="inlineStr">
@@ -14982,24 +14982,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C357" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C357" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D357" s="9" t="inlineStr">
         <is>
-          <t>One shared row, one route onto your day</t>
+          <t>A taken-on row is never on screen twice</t>
         </is>
       </c>
       <c r="E357" s="9" t="inlineStr">
         <is>
-          <t>In the room, hold an UNDATED row, then hold a repeating or dated one.</t>
+          <t>Take a shared row on (Pin it, or Bring it from the room). Look at Today.</t>
         </is>
       </c>
       <c r="F357" s="9" t="inlineStr">
         <is>
-          <t>The undated row offers 'Bring to my Today'. The dated or repeating one does NOT: it already arrives by itself. Two routes landing in two different places (a copy in your list, or the strip) was the confusion Melroy hit twice.</t>
+          <t>It appears once, as your task, and NOT also in the From Ours strip. Still true once it is ticked: a finished copy and its finished origin must not both render.</t>
         </is>
       </c>
       <c r="G357" s="7" t="inlineStr">
@@ -15014,7 +15014,7 @@
     <row r="358">
       <c r="A358" s="6" t="inlineStr">
         <is>
-          <t>OUR-84</t>
+          <t>OUR-82</t>
         </is>
       </c>
       <c r="B358" s="7" t="inlineStr">
@@ -15022,24 +15022,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C358" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C358" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D358" s="9" t="inlineStr">
         <is>
-          <t>Take a From Ours row on, and it becomes an ordinary task</t>
+          <t>Move-to is not offered on a repeating shared row</t>
         </is>
       </c>
       <c r="E358" s="9" t="inlineStr">
         <is>
-          <t>Hold a row in the From Just Us strip and choose 'Take this on today'.</t>
+          <t>Hold a repeating row in the From Ours strip.</t>
         </is>
       </c>
       <c r="F358" s="9" t="inlineStr">
         <is>
-          <t>It leaves the strip and joins your list tagged '. Ours'. Holding it now gives the FULL held card: Break it down, Make tiny, Steps, Nudge, reorder, everything. That visible move IS the message: you have taken it on.</t>
+          <t>Pin is there, Move to is not. A date and a rhythm are alternatives, and rescheduling a series is a question for the room's cadence sheet, not a one-tap action on a day.</t>
         </is>
       </c>
       <c r="G358" s="7" t="inlineStr">
@@ -15054,7 +15054,7 @@
     <row r="359">
       <c r="A359" s="6" t="inlineStr">
         <is>
-          <t>OUR-85</t>
+          <t>OUR-83</t>
         </is>
       </c>
       <c r="B359" s="7" t="inlineStr">
@@ -15062,24 +15062,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C359" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C359" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D359" s="9" t="inlineStr">
         <is>
-          <t>Break it down works once taken on, and never touches the shared list</t>
+          <t>One shared row, one route onto your day</t>
         </is>
       </c>
       <c r="E359" s="9" t="inlineStr">
         <is>
-          <t>Take a shared row on, then Break it down.</t>
+          <t>In the room, hold an UNDATED row, then hold a repeating or dated one.</t>
         </is>
       </c>
       <c r="F359" s="9" t="inlineStr">
         <is>
-          <t>The steps land on YOUR copy, on your day. The shared list is unchanged and your person sees nothing new. Breaking down was blocked on the shared row because a model authoring steps onto a list another person reads is a decision about them; on your own copy that objection is gone.</t>
+          <t>The undated row offers 'Bring to my Today'. The dated or repeating one does NOT: it already arrives by itself. Two routes landing in two different places (a copy in your list, or the strip) was the confusion Melroy hit twice.</t>
         </is>
       </c>
       <c r="G359" s="7" t="inlineStr">
@@ -15094,7 +15094,7 @@
     <row r="360">
       <c r="A360" s="6" t="inlineStr">
         <is>
-          <t>OUR-86</t>
+          <t>OUR-84</t>
         </is>
       </c>
       <c r="B360" s="7" t="inlineStr">
@@ -15109,17 +15109,17 @@
       </c>
       <c r="D360" s="9" t="inlineStr">
         <is>
-          <t>Select several rows in the room and tick them together</t>
+          <t>Take a From Ours row on, and it becomes an ordinary task</t>
         </is>
       </c>
       <c r="E360" s="9" t="inlineStr">
         <is>
-          <t>Hold a row, choose Select more, tap a few more, then Done.</t>
+          <t>Hold a row in the From Just Us strip and choose 'Take this on today'.</t>
         </is>
       </c>
       <c r="F360" s="9" t="inlineStr">
         <is>
-          <t>All of them tick at once and reach the other device. This is the trip-to-the-shops case: six things bought, six taps was a tax that stops people keeping the list.</t>
+          <t>It leaves the strip and joins your list tagged '. Ours'. Holding it now gives the FULL held card: Break it down, Make tiny, Steps, Nudge, reorder, everything. That visible move IS the message: you have taken it on.</t>
         </is>
       </c>
       <c r="G360" s="7" t="inlineStr">
@@ -15134,7 +15134,7 @@
     <row r="361">
       <c r="A361" s="6" t="inlineStr">
         <is>
-          <t>OUR-87</t>
+          <t>OUR-85</t>
         </is>
       </c>
       <c r="B361" s="7" t="inlineStr">
@@ -15142,24 +15142,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C361" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C361" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D361" s="9" t="inlineStr">
         <is>
-          <t>Bulk tick never UN-ticks</t>
+          <t>Break it down works once taken on, and never touches the shared list</t>
         </is>
       </c>
       <c r="E361" s="9" t="inlineStr">
         <is>
-          <t>Select a mix of done and not-done rows and tap Done.</t>
+          <t>Take a shared row on, then Break it down.</t>
         </is>
       </c>
       <c r="F361" s="9" t="inlineStr">
         <is>
-          <t>The not-done ones tick. The already-done ones are untouched. A bulk toggle would silently undo somebody's finished work on a mixed selection.</t>
+          <t>The steps land on YOUR copy, on your day. The shared list is unchanged and your person sees nothing new. Breaking down was blocked on the shared row because a model authoring steps onto a list another person reads is a decision about them; on your own copy that objection is gone.</t>
         </is>
       </c>
       <c r="G361" s="7" t="inlineStr">
@@ -15174,7 +15174,7 @@
     <row r="362">
       <c r="A362" s="6" t="inlineStr">
         <is>
-          <t>OUR-88</t>
+          <t>OUR-86</t>
         </is>
       </c>
       <c r="B362" s="7" t="inlineStr">
@@ -15189,17 +15189,17 @@
       </c>
       <c r="D362" s="9" t="inlineStr">
         <is>
-          <t>Bulk remove warns BEFORE the tap when a repeat is selected</t>
+          <t>Select several rows in the room and tick them together</t>
         </is>
       </c>
       <c r="E362" s="9" t="inlineStr">
         <is>
-          <t>Select a repeating row along with others. Read the shelf.</t>
+          <t>Hold a row, choose Select more, tap a few more, then Done.</t>
         </is>
       </c>
       <c r="F362" s="9" t="inlineStr">
         <is>
-          <t>A line says removing a repeat here ends it for both of you. A shared list has no per-day skip, so this is not a thing to learn from the consequence.</t>
+          <t>All of them tick at once and reach the other device. This is the trip-to-the-shops case: six things bought, six taps was a tax that stops people keeping the list.</t>
         </is>
       </c>
       <c r="G362" s="7" t="inlineStr">
@@ -15214,7 +15214,7 @@
     <row r="363">
       <c r="A363" s="6" t="inlineStr">
         <is>
-          <t>OUR-89</t>
+          <t>OUR-87</t>
         </is>
       </c>
       <c r="B363" s="7" t="inlineStr">
@@ -15222,24 +15222,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C363" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C363" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D363" s="9" t="inlineStr">
         <is>
-          <t>The select shelf takes the capture bar's seat</t>
+          <t>Bulk tick never UN-ticks</t>
         </is>
       </c>
       <c r="E363" s="9" t="inlineStr">
         <is>
-          <t>Enter select mode in the room.</t>
+          <t>Select a mix of done and not-done rows and tap Done.</t>
         </is>
       </c>
       <c r="F363" s="9" t="inlineStr">
         <is>
-          <t>The capture bar is gone while selecting, and back when you cancel. Two bottom-anchored surfaces competing for the thumb is how a calm screen stops being one, and you are not adding things while you are clearing things.</t>
+          <t>The not-done ones tick. The already-done ones are untouched. A bulk toggle would silently undo somebody's finished work on a mixed selection.</t>
         </is>
       </c>
       <c r="G363" s="7" t="inlineStr">
@@ -15254,7 +15254,7 @@
     <row r="364">
       <c r="A364" s="6" t="inlineStr">
         <is>
-          <t>OUR-90</t>
+          <t>OUR-88</t>
         </is>
       </c>
       <c r="B364" s="7" t="inlineStr">
@@ -15262,24 +15262,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C364" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C364" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D364" s="9" t="inlineStr">
         <is>
-          <t>No select mode on a closed list</t>
+          <t>Bulk remove warns BEFORE the tap when a repeat is selected</t>
         </is>
       </c>
       <c r="E364" s="9" t="inlineStr">
         <is>
-          <t>Open an archived list and hold a row.</t>
+          <t>Select a repeating row along with others. Read the shelf.</t>
         </is>
       </c>
       <c r="F364" s="9" t="inlineStr">
         <is>
-          <t>No Select more. A closed list is readable and nothing else, and the server would refuse the write anyway.</t>
+          <t>A line says removing a repeat here ends it for both of you. A shared list has no per-day skip, so this is not a thing to learn from the consequence.</t>
         </is>
       </c>
       <c r="G364" s="7" t="inlineStr">
@@ -15294,7 +15294,7 @@
     <row r="365">
       <c r="A365" s="6" t="inlineStr">
         <is>
-          <t>OUR-91</t>
+          <t>OUR-89</t>
         </is>
       </c>
       <c r="B365" s="7" t="inlineStr">
@@ -15302,24 +15302,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C365" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C365" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D365" s="9" t="inlineStr">
         <is>
-          <t>A copy says when its shared row was taken off the list</t>
+          <t>The select shelf takes the capture bar's seat</t>
         </is>
       </c>
       <c r="E365" s="9" t="inlineStr">
         <is>
-          <t>Device B removes a row from Ours. On device A, look at the brought copy on Today.</t>
+          <t>Enter select mode in the room.</t>
         </is>
       </c>
       <c r="F365" s="9" t="inlineStr">
         <is>
-          <t>The copy STAYS (it is your task now) and carries a faint line: 'no longer on &lt;list name&gt;'. The deciding case is wasted effort: she removed milk because she already bought it, and a silent copy sends you to the shop.</t>
+          <t>The capture bar is gone while selecting, and back when you cancel. Two bottom-anchored surfaces competing for the thumb is how a calm screen stops being one, and you are not adding things while you are clearing things.</t>
         </is>
       </c>
       <c r="G365" s="7" t="inlineStr">
@@ -15334,7 +15334,7 @@
     <row r="366">
       <c r="A366" s="6" t="inlineStr">
         <is>
-          <t>OUR-92</t>
+          <t>OUR-90</t>
         </is>
       </c>
       <c r="B366" s="7" t="inlineStr">
@@ -15342,24 +15342,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C366" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C366" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D366" s="9" t="inlineStr">
         <is>
-          <t>That line never says who, and never says why</t>
+          <t>No select mode on a closed list</t>
         </is>
       </c>
       <c r="E366" s="9" t="inlineStr">
         <is>
-          <t>Read the line closely.</t>
+          <t>Open an archived list and hold a row.</t>
         </is>
       </c>
       <c r="F366" s="9" t="inlineStr">
         <is>
-          <t>It states the fact only. Not who removed it (no such data exists anywhere in this feature, and a bridge is where that temptation returns) and not why (removal could be done, not-needed or tidying, and the app cannot tell them apart).</t>
+          <t>No Select more. A closed list is readable and nothing else, and the server would refuse the write anyway.</t>
         </is>
       </c>
       <c r="G366" s="7" t="inlineStr">
@@ -15374,7 +15374,7 @@
     <row r="367">
       <c r="A367" s="6" t="inlineStr">
         <is>
-          <t>OUR-93</t>
+          <t>OUR-91</t>
         </is>
       </c>
       <c r="B367" s="7" t="inlineStr">
@@ -15382,24 +15382,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C367" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C367" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D367" s="9" t="inlineStr">
         <is>
-          <t>No line on a copy you already finished or removed</t>
+          <t>A copy says when its shared row was taken off the list</t>
         </is>
       </c>
       <c r="E367" s="9" t="inlineStr">
         <is>
-          <t>Finish your copy, then have B remove the shared row. Then try it with a copy you removed yourself.</t>
+          <t>Device B removes a row from Ours. On device A, look at the brought copy on Today.</t>
         </is>
       </c>
       <c r="F367" s="9" t="inlineStr">
         <is>
-          <t>No line in either case. You did the thing, so its origin's fate is not news, and a note there would read as a correction.</t>
+          <t>The copy STAYS (it is your task now) and carries a faint line: 'no longer on &lt;list name&gt;'. The deciding case is wasted effort: she removed milk because she already bought it, and a silent copy sends you to the shop.</t>
         </is>
       </c>
       <c r="G367" s="7" t="inlineStr">
@@ -15414,7 +15414,7 @@
     <row r="368">
       <c r="A368" s="6" t="inlineStr">
         <is>
-          <t>OUR-94</t>
+          <t>OUR-92</t>
         </is>
       </c>
       <c r="B368" s="7" t="inlineStr">
@@ -15422,24 +15422,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C368" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C368" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D368" s="9" t="inlineStr">
         <is>
-          <t>The line goes quiet after the tombstone sweep, rather than guessing</t>
+          <t>That line never says who, and never says why</t>
         </is>
       </c>
       <c r="E368" s="9" t="inlineStr">
         <is>
-          <t>More than seven days after a removal (or with the tombstone swept), check the copy.</t>
+          <t>Read the line closely.</t>
         </is>
       </c>
       <c r="F368" s="9" t="inlineStr">
         <is>
-          <t>No line. A swept origin is indistinguishable from one never pulled, and keeping a permanent record of a deletion so the app can keep mentioning it is its own kind of creepy. Accepted limit, not a bug.</t>
+          <t>It states the fact only. Not who removed it (no such data exists anywhere in this feature, and a bridge is where that temptation returns) and not why (removal could be done, not-needed or tidying, and the app cannot tell them apart).</t>
         </is>
       </c>
       <c r="G368" s="7" t="inlineStr">
@@ -15454,7 +15454,7 @@
     <row r="369">
       <c r="A369" s="6" t="inlineStr">
         <is>
-          <t>OUR-95</t>
+          <t>OUR-93</t>
         </is>
       </c>
       <c r="B369" s="7" t="inlineStr">
@@ -15462,24 +15462,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C369" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C369" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D369" s="9" t="inlineStr">
         <is>
-          <t>A row's note is VISIBLE, not only spoken</t>
+          <t>No line on a copy you already finished or removed</t>
         </is>
       </c>
       <c r="E369" s="9" t="inlineStr">
         <is>
-          <t>Trigger any row note: have B change a row (the room's wash) or remove a shared row you hold a copy of (Today).</t>
+          <t>Finish your copy, then have B remove the shared row. Then try it with a copy you removed yourself.</t>
         </is>
       </c>
       <c r="F369" s="9" t="inlineStr">
         <is>
-          <t>The words appear as a quiet second line under the title. Before 2026-08-12 the note prop reached only the accessibility label, so every one of these lines was spoken to screen readers and shown to nobody, for as long as the prop had existed.</t>
+          <t>No line in either case. You did the thing, so its origin's fate is not news, and a note there would read as a correction.</t>
         </is>
       </c>
       <c r="G369" s="7" t="inlineStr">
@@ -15494,7 +15494,7 @@
     <row r="370">
       <c r="A370" s="6" t="inlineStr">
         <is>
-          <t>OUR-96</t>
+          <t>OUR-94</t>
         </is>
       </c>
       <c r="B370" s="7" t="inlineStr">
@@ -15502,24 +15502,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C370" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C370" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D370" s="9" t="inlineStr">
         <is>
-          <t>Rows WITHOUT a note are unchanged</t>
+          <t>The line goes quiet after the tombstone sweep, rather than guessing</t>
         </is>
       </c>
       <c r="E370" s="9" t="inlineStr">
         <is>
-          <t>Compare a plain row, a 'big' row and a repeating row against a build before the note landed.</t>
+          <t>More than seven days after a removal (or with the tombstone swept), check the copy.</t>
         </is>
       </c>
       <c r="F370" s="9" t="inlineStr">
         <is>
-          <t>Same height to within a pixel. The note gave TaskRow a second line, and a row that has no note must not gain one, shift, or reflow.</t>
+          <t>No line. A swept origin is indistinguishable from one never pulled, and keeping a permanent record of a deletion so the app can keep mentioning it is its own kind of creepy. Accepted limit, not a bug.</t>
         </is>
       </c>
       <c r="G370" s="7" t="inlineStr">
@@ -15534,7 +15534,7 @@
     <row r="371">
       <c r="A371" s="6" t="inlineStr">
         <is>
-          <t>OUR-97</t>
+          <t>OUR-95</t>
         </is>
       </c>
       <c r="B371" s="7" t="inlineStr">
@@ -15549,17 +15549,17 @@
       </c>
       <c r="D371" s="9" t="inlineStr">
         <is>
-          <t>A tick after midnight lands on the RIGHT day</t>
+          <t>A row's note is VISIBLE, not only spoken</t>
         </is>
       </c>
       <c r="E371" s="9" t="inlineStr">
         <is>
-          <t>Open the room at 23:58 and leave it open. Tick a row at 00:02. Check the partner's device.</t>
+          <t>Trigger any row note: have B change a row (the room's wash) or remove a shared row you hold a copy of (Today).</t>
         </is>
       </c>
       <c r="F371" s="9" t="inlineStr">
         <is>
-          <t>Done on both, dated today. The room's date used to freeze at mount, so the completion log took yesterday's key and the partner's phone, asking about today, got false. Permanently: the merge is per-date.</t>
+          <t>The words appear as a quiet second line under the title. Before 2026-08-12 the note prop reached only the accessibility label, so every one of these lines was spoken to screen readers and shown to nobody, for as long as the prop had existed.</t>
         </is>
       </c>
       <c r="G371" s="7" t="inlineStr">
@@ -15574,7 +15574,7 @@
     <row r="372">
       <c r="A372" s="6" t="inlineStr">
         <is>
-          <t>OUR-98</t>
+          <t>OUR-96</t>
         </is>
       </c>
       <c r="B372" s="7" t="inlineStr">
@@ -15582,24 +15582,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C372" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C372" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D372" s="9" t="inlineStr">
         <is>
-          <t>A tick made during a background sync is not undone</t>
+          <t>Rows WITHOUT a note are unchanged</t>
         </is>
       </c>
       <c r="E372" s="9" t="inlineStr">
         <is>
-          <t>Background and reopen the app (which triggers a settle), then immediately tick a row in the From Ours strip.</t>
+          <t>Compare a plain row, a 'big' row and a repeating row against a build before the note landed.</t>
         </is>
       </c>
       <c r="F372" s="9" t="inlineStr">
         <is>
-          <t>It stays ticked. The settle now refuses to save a merge that predates any local write made while it was on the wire.</t>
+          <t>Same height to within a pixel. The note gave TaskRow a second line, and a row that has no note must not gain one, shift, or reflow.</t>
         </is>
       </c>
       <c r="G372" s="7" t="inlineStr">
@@ -15614,7 +15614,7 @@
     <row r="373">
       <c r="A373" s="6" t="inlineStr">
         <is>
-          <t>OUR-99</t>
+          <t>OUR-97</t>
         </is>
       </c>
       <c r="B373" s="7" t="inlineStr">
@@ -15629,17 +15629,17 @@
       </c>
       <c r="D373" s="9" t="inlineStr">
         <is>
-          <t>A tick survives a device that has never opened the room</t>
+          <t>A tick after midnight lands on the RIGHT day</t>
         </is>
       </c>
       <c r="E373" s="9" t="inlineStr">
         <is>
-          <t>On a device with no Ours cache, go offline, tick a brought copy, come back online, reopen the app.</t>
+          <t>Open the room at 23:58 and leave it open. Tick a row at 00:02. Check the partner's device.</t>
         </is>
       </c>
       <c r="F373" s="9" t="inlineStr">
         <is>
-          <t>The tick reaches the shared list. It used to be lost forever: the only carrier pulled before writing, and nothing retried. The settle now carries it, with the copy's OWN completion time, so a deliberate un-tick on the other side still wins.</t>
+          <t>Done on both, dated today. The room's date used to freeze at mount, so the completion log took yesterday's key and the partner's phone, asking about today, got false. Permanently: the merge is per-date.</t>
         </is>
       </c>
       <c r="G373" s="7" t="inlineStr">
@@ -15654,7 +15654,7 @@
     <row r="374">
       <c r="A374" s="6" t="inlineStr">
         <is>
-          <t>OUR-100</t>
+          <t>OUR-98</t>
         </is>
       </c>
       <c r="B374" s="7" t="inlineStr">
@@ -15669,17 +15669,17 @@
       </c>
       <c r="D374" s="9" t="inlineStr">
         <is>
-          <t>A repeat is visible in the room EVERY day, tickable only on its own</t>
+          <t>A tick made during a background sync is not undone</t>
         </is>
       </c>
       <c r="E374" s="9" t="inlineStr">
         <is>
-          <t>Make a weekly shared repeat. Open the room on a day it is not due.</t>
+          <t>Background and reopen the app (which triggers a settle), then immediately tick a row in the From Ours strip.</t>
         </is>
       </c>
       <c r="F374" s="9" t="inlineStr">
         <is>
-          <t>The row is there, with its rhythm in words, and its checkbox is inert with 'you can tick this on its day'. It used to vanish six days a week: unreachable to edit or remove, and a list of only repeats said 'Nothing here yet'.</t>
+          <t>It stays ticked. The settle now refuses to save a merge that predates any local write made while it was on the wire.</t>
         </is>
       </c>
       <c r="G374" s="7" t="inlineStr">
@@ -15694,7 +15694,7 @@
     <row r="375">
       <c r="A375" s="6" t="inlineStr">
         <is>
-          <t>OUR-101</t>
+          <t>OUR-99</t>
         </is>
       </c>
       <c r="B375" s="7" t="inlineStr">
@@ -15702,24 +15702,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C375" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C375" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D375" s="9" t="inlineStr">
         <is>
-          <t>A closed list stops promising it keeps trying</t>
+          <t>A tick survives a device that has never opened the room</t>
         </is>
       </c>
       <c r="E375" s="9" t="inlineStr">
         <is>
-          <t>Open an archived list that has unpushed local changes.</t>
+          <t>On a device with no Ours cache, go offline, tick a brought copy, come back online, reopen the app.</t>
         </is>
       </c>
       <c r="F375" s="9" t="inlineStr">
         <is>
-          <t>It says the list is closed, not 'Saved here, not there'. On a list where the write can never succeed, the second is a false hope on a screen a separated or bereaved person may keep for years.</t>
+          <t>The tick reaches the shared list. It used to be lost forever: the only carrier pulled before writing, and nothing retried. The settle now carries it, with the copy's OWN completion time, so a deliberate un-tick on the other side still wins.</t>
         </is>
       </c>
       <c r="G375" s="7" t="inlineStr">
@@ -15734,7 +15734,7 @@
     <row r="376">
       <c r="A376" s="6" t="inlineStr">
         <is>
-          <t>OUR-102</t>
+          <t>OUR-100</t>
         </is>
       </c>
       <c r="B376" s="7" t="inlineStr">
@@ -15742,24 +15742,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C376" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C376" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D376" s="9" t="inlineStr">
         <is>
-          <t>Setting a rhythm clears any date the row was carrying</t>
+          <t>A repeat is visible in the room EVERY day, tickable only on its own</t>
         </is>
       </c>
       <c r="E376" s="9" t="inlineStr">
         <is>
-          <t>Give a DATED shared row a weekly rhythm, then read the row.</t>
+          <t>Make a weekly shared repeat. Open the room on a day it is not due.</t>
         </is>
       </c>
       <c r="F376" s="9" t="inlineStr">
         <is>
-          <t>One schedule, not two. The date is gone. Leaving it made the row answer differently depending on which code asked.</t>
+          <t>The row is there, with its rhythm in words, and its checkbox is inert with 'you can tick this on its day'. It used to vanish six days a week: unreachable to edit or remove, and a list of only repeats said 'Nothing here yet'.</t>
         </is>
       </c>
       <c r="G376" s="7" t="inlineStr">
@@ -15774,7 +15774,7 @@
     <row r="377">
       <c r="A377" s="6" t="inlineStr">
         <is>
-          <t>OUR-103</t>
+          <t>OUR-101</t>
         </is>
       </c>
       <c r="B377" s="7" t="inlineStr">
@@ -15789,17 +15789,17 @@
       </c>
       <c r="D377" s="9" t="inlineStr">
         <is>
-          <t>Renaming inside the cadence sheet warns about the 500-character cap</t>
+          <t>A closed list stops promising it keeps trying</t>
         </is>
       </c>
       <c r="E377" s="9" t="inlineStr">
         <is>
-          <t>Open a row's rhythm sheet, paste a title over 500 characters, save.</t>
+          <t>Open an archived list that has unpushed local changes.</t>
         </is>
       </c>
       <c r="F377" s="9" t="inlineStr">
         <is>
-          <t>The trim notice appears BEFORE the save, the same as renaming on the row. It used to save silently and the server clamped it, so the words vanished a second later.</t>
+          <t>It says the list is closed, not 'Saved here, not there'. On a list where the write can never succeed, the second is a false hope on a screen a separated or bereaved person may keep for years.</t>
         </is>
       </c>
       <c r="G377" s="7" t="inlineStr">
@@ -15814,7 +15814,7 @@
     <row r="378">
       <c r="A378" s="6" t="inlineStr">
         <is>
-          <t>OUR-104</t>
+          <t>OUR-102</t>
         </is>
       </c>
       <c r="B378" s="7" t="inlineStr">
@@ -15822,24 +15822,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C378" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C378" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D378" s="9" t="inlineStr">
         <is>
-          <t>No dead reorder rail on shared rows</t>
+          <t>Setting a rhythm clears any date the row was carrying</t>
         </is>
       </c>
       <c r="E378" s="9" t="inlineStr">
         <is>
-          <t>Hold a row in the room and in the From Ours strip.</t>
+          <t>Give a DATED shared row a weekly rhythm, then read the row.</t>
         </is>
       </c>
       <c r="F378" s="9" t="inlineStr">
         <is>
-          <t>No up/down rail. Neither surface supplies those handlers, so it was two permanently inert controls on the screen briefed to be plainer than Today. Dim-in-place is for a control that is sometimes live.</t>
+          <t>One schedule, not two. The date is gone. Leaving it made the row answer differently depending on which code asked.</t>
         </is>
       </c>
       <c r="G378" s="7" t="inlineStr">
@@ -15854,7 +15854,7 @@
     <row r="379">
       <c r="A379" s="6" t="inlineStr">
         <is>
-          <t>OUR-105</t>
+          <t>OUR-103</t>
         </is>
       </c>
       <c r="B379" s="7" t="inlineStr">
@@ -15862,24 +15862,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C379" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C379" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D379" s="9" t="inlineStr">
         <is>
-          <t>First run introduces the shared list</t>
+          <t>Renaming inside the cadence sheet warns about the 500-character cap</t>
         </is>
       </c>
       <c r="E379" s="9" t="inlineStr">
         <is>
-          <t>Reset onboarding (Settings, replay the first run) and step through it.</t>
+          <t>Open a row's rhythm sheet, paste a title over 500 characters, save.</t>
         </is>
       </c>
       <c r="F379" s="9" t="inlineStr">
         <is>
-          <t>An eighth step sits between 'keep' and 'premium', headed 'A list the two of you keep.' It says what arrives by itself, what deliberately does NOT, and that nothing keeps score. Its position matters: a FREE feature read immediately before the premium screen would be mistaken for part of the paid list.</t>
+          <t>The trim notice appears BEFORE the save, the same as renaming on the row. It used to save silently and the server clamped it, so the words vanished a second later.</t>
         </is>
       </c>
       <c r="G379" s="7" t="inlineStr">
@@ -15894,7 +15894,7 @@
     <row r="380">
       <c r="A380" s="6" t="inlineStr">
         <is>
-          <t>OUR-106</t>
+          <t>OUR-104</t>
         </is>
       </c>
       <c r="B380" s="7" t="inlineStr">
@@ -15902,24 +15902,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C380" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C380" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D380" s="9" t="inlineStr">
         <is>
-          <t>Anyone can start a shared list, not just an allowlisted address</t>
+          <t>No dead reorder rail on shared rows</t>
         </is>
       </c>
       <c r="E380" s="9" t="inlineStr">
         <is>
-          <t>With supabase/ours-open.sql applied, sign in as an account that was never in ours_allowlist and create an invite.</t>
+          <t>Hold a row in the room and in the From Ours strip.</t>
         </is>
       </c>
       <c r="F380" s="9" t="inlineStr">
         <is>
-          <t>It works. Before that migration only JOINING was open; STARTING was gated, so the refusal hit exactly the person a store listing brings you.</t>
+          <t>No up/down rail. Neither surface supplies those handlers, so it was two permanently inert controls on the screen briefed to be plainer than Today. Dim-in-place is for a control that is sometimes live.</t>
         </is>
       </c>
       <c r="G380" s="7" t="inlineStr">
@@ -15934,7 +15934,7 @@
     <row r="381">
       <c r="A381" s="6" t="inlineStr">
         <is>
-          <t>OUR-107</t>
+          <t>OUR-105</t>
         </is>
       </c>
       <c r="B381" s="7" t="inlineStr">
@@ -15949,17 +15949,17 @@
       </c>
       <c r="D381" s="9" t="inlineStr">
         <is>
-          <t>The shared-list onboarding step can actually be REACHED</t>
+          <t>First run introduces the shared list</t>
         </is>
       </c>
       <c r="E381" s="9" t="inlineStr">
         <is>
-          <t>Replay the first run and press the primary button through every step without skipping.</t>
+          <t>Reset onboarding (Settings, replay the first run) and step through it.</t>
         </is>
       </c>
       <c r="F381" s="9" t="inlineStr">
         <is>
-          <t>The shared-list screen appears as the sixth of eight, between 'What you finish, you keep' and the premium screen. It shipped once as a step that existed, was translated into five languages, and could not be arrived at: the flow advanced by a hand-written map that still went keep -&gt; premium.</t>
+          <t>An eighth step sits between 'keep' and 'premium', headed 'A list the two of you keep.' It says what arrives by itself, what deliberately does NOT, and that nothing keeps score. Its position matters: a FREE feature read immediately before the premium screen would be mistaken for part of the paid list.</t>
         </is>
       </c>
       <c r="G381" s="7" t="inlineStr">
@@ -15974,7 +15974,7 @@
     <row r="382">
       <c r="A382" s="6" t="inlineStr">
         <is>
-          <t>OUR-108</t>
+          <t>OUR-106</t>
         </is>
       </c>
       <c r="B382" s="7" t="inlineStr">
@@ -15982,24 +15982,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C382" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C382" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D382" s="9" t="inlineStr">
         <is>
-          <t>ONE person, TWO devices: does your own edit wash on your other phone?</t>
+          <t>Anyone can start a shared list, not just an allowlisted address</t>
         </is>
       </c>
       <c r="E382" s="9" t="inlineStr">
         <is>
-          <t>Sign in to the same account on two devices (an iPhone and an Android, say). Change a row in Ours on the FIRST. Open Ours on the SECOND.</t>
+          <t>With supabase/ours-open.sql applied, sign in as an account that was never in ours_allowlist and create an invite.</t>
         </is>
       </c>
       <c r="F382" s="9" t="inlineStr">
         <is>
-          <t>OPEN QUESTION, not a known-good expectation. The 'this edit was mine' record is stored PER DEVICE (noteOursMine writes to local storage), so the second device has no idea the first one did it and will most likely tint the row as changed-since-you-looked. It breaks none of the three laws, since the wording never names a person, but it may still read wrong: your own edit wearing the mark that means 'your person did something'. Only reachable when one person holds two phones, which nobody did until 2026-08-13. If it tints, the fix is to key `mine` on the account rather than the device.</t>
+          <t>It works. Before that migration only JOINING was open; STARTING was gated, so the refusal hit exactly the person a store listing brings you.</t>
         </is>
       </c>
       <c r="G382" s="7" t="inlineStr">
@@ -16014,7 +16014,7 @@
     <row r="383">
       <c r="A383" s="6" t="inlineStr">
         <is>
-          <t>OUR-109</t>
+          <t>OUR-107</t>
         </is>
       </c>
       <c r="B383" s="7" t="inlineStr">
@@ -16029,17 +16029,17 @@
       </c>
       <c r="D383" s="9" t="inlineStr">
         <is>
-          <t>A repeat's rhythm sits INSIDE its own card and reads as a rhythm</t>
+          <t>The shared-list onboarding step can actually be REACHED</t>
         </is>
       </c>
       <c r="E383" s="9" t="inlineStr">
         <is>
-          <t>Give a shared task a weekly repeat on a weekday that is not today. Look at it in the room.</t>
+          <t>Replay the first run and press the primary button through every step without skipping.</t>
         </is>
       </c>
       <c r="F383" s="9" t="inlineStr">
         <is>
-          <t>The line is indented under that row's title, inside the card, and reads 'Every Thu' rather than a bare 'Thu'. It used to be drawn BELOW the card, so it floated between two rows belonging to neither, and said only the weekday.</t>
+          <t>The shared-list screen appears as the sixth of eight, between 'What you finish, you keep' and the premium screen. It shipped once as a step that existed, was translated into five languages, and could not be arrived at: the flow advanced by a hand-written map that still went keep -&gt; premium.</t>
         </is>
       </c>
       <c r="G383" s="7" t="inlineStr">
@@ -16054,7 +16054,7 @@
     <row r="384">
       <c r="A384" s="6" t="inlineStr">
         <is>
-          <t>OUR-110</t>
+          <t>OUR-108</t>
         </is>
       </c>
       <c r="B384" s="7" t="inlineStr">
@@ -16062,24 +16062,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C384" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C384" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D384" s="9" t="inlineStr">
         <is>
-          <t>A circle you cannot tick LOOKS like one you cannot tick</t>
+          <t>ONE person, TWO devices: does your own edit wash on your other phone?</t>
         </is>
       </c>
       <c r="E384" s="9" t="inlineStr">
         <is>
-          <t>Find that same repeat on a day it is not due, or open any row on a closed list.</t>
+          <t>Sign in to the same account on two devices (an iPhone and an Android, say). Change a row in Ours on the FIRST. Open Ours on the SECOND.</t>
         </is>
       </c>
       <c r="F384" s="9" t="inlineStr">
         <is>
-          <t>The circle is visibly faded. It used to render identically to a live one, so the row offered a control that looked tappable and did nothing, which is the exact failure the 'quiet-unavailable' rule was written to prevent.</t>
+          <t>OPEN QUESTION, not a known-good expectation. The 'this edit was mine' record is stored PER DEVICE (noteOursMine writes to local storage), so the second device has no idea the first one did it and will most likely tint the row as changed-since-you-looked. It breaks none of the three laws, since the wording never names a person, but it may still read wrong: your own edit wearing the mark that means 'your person did something'. Only reachable when one person holds two phones, which nobody did until 2026-08-13. If it tints, the fix is to key `mine` on the account rather than the device.</t>
         </is>
       </c>
       <c r="G384" s="7" t="inlineStr">
@@ -16094,12 +16094,12 @@
     <row r="385">
       <c r="A385" s="6" t="inlineStr">
         <is>
-          <t>UPD-01</t>
+          <t>OUR-109</t>
         </is>
       </c>
       <c r="B385" s="7" t="inlineStr">
         <is>
-          <t>Updates</t>
+          <t>Ours</t>
         </is>
       </c>
       <c r="C385" s="8" t="inlineStr">
@@ -16109,17 +16109,17 @@
       </c>
       <c r="D385" s="9" t="inlineStr">
         <is>
-          <t>Settings states the version, and up-to-date is a fact</t>
+          <t>A repeat's rhythm sits INSIDE its own card and reads as a rhythm</t>
         </is>
       </c>
       <c r="E385" s="9" t="inlineStr">
         <is>
-          <t>Open Settings and scroll to the foot.</t>
+          <t>Give a shared task a weekly repeat on a weekday that is not today. Look at it in the room.</t>
         </is>
       </c>
       <c r="F385" s="9" t="inlineStr">
         <is>
-          <t>One line: 'v1.2.0 (11)  ·  Up to date'. It is a sage FACT, not a control. Nothing is offered when there is nothing to offer.</t>
+          <t>The line is indented under that row's title, inside the card, and reads 'Every Thu' rather than a bare 'Thu'. It used to be drawn BELOW the card, so it floated between two rows belonging to neither, and said only the weekday.</t>
         </is>
       </c>
       <c r="G385" s="7" t="inlineStr">
@@ -16134,12 +16134,12 @@
     <row r="386">
       <c r="A386" s="6" t="inlineStr">
         <is>
-          <t>UPD-02</t>
+          <t>OUR-110</t>
         </is>
       </c>
       <c r="B386" s="7" t="inlineStr">
         <is>
-          <t>Updates</t>
+          <t>Ours</t>
         </is>
       </c>
       <c r="C386" s="8" t="inlineStr">
@@ -16149,22 +16149,22 @@
       </c>
       <c r="D386" s="9" t="inlineStr">
         <is>
-          <t>Web offers a reload, and says drafts are kept</t>
+          <t>A circle you cannot tick LOOKS like one you cannot tick</t>
         </is>
       </c>
       <c r="E386" s="9" t="inlineStr">
         <is>
-          <t>With doubledone.app/version.json's "web" set ahead of the running build, open Settings on the web.</t>
+          <t>Find that same repeat on a day it is not due, or open any row on a closed list.</t>
         </is>
       </c>
       <c r="F386" s="9" t="inlineStr">
         <is>
-          <t>'A newer version is ready.' + 'Reload to get it' + 'Anything you were typing is kept.' Type something into the capture box first and confirm it survives the reload.</t>
+          <t>The circle is visibly faded. It used to render identically to a live one, so the row offered a control that looked tappable and did nothing, which is the exact failure the 'quiet-unavailable' rule was written to prevent.</t>
         </is>
       </c>
       <c r="G386" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H386" s="7" t="inlineStr"/>
@@ -16174,7 +16174,7 @@
     <row r="387">
       <c r="A387" s="6" t="inlineStr">
         <is>
-          <t>UPD-03</t>
+          <t>UPD-01</t>
         </is>
       </c>
       <c r="B387" s="7" t="inlineStr">
@@ -16189,22 +16189,22 @@
       </c>
       <c r="D387" s="9" t="inlineStr">
         <is>
-          <t>Native points at the store, and says lists are untouched</t>
+          <t>Settings states the version, and up-to-date is a fact</t>
         </is>
       </c>
       <c r="E387" s="9" t="inlineStr">
         <is>
-          <t>With version.json's "ios" / "android" set ahead of the installed build, open Settings on a device.</t>
+          <t>Open Settings and scroll to the foot.</t>
         </is>
       </c>
       <c r="F387" s="9" t="inlineStr">
         <is>
-          <t>'This build is getting old.' + 'Open the store' + 'Your lists stay exactly as they are.' The button opens the correct store listing.</t>
+          <t>One line: 'v1.2.0 (11)  ·  Up to date'. It is a sage FACT, not a control. Nothing is offered when there is nothing to offer.</t>
         </is>
       </c>
       <c r="G387" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H387" s="7" t="inlineStr"/>
@@ -16214,7 +16214,7 @@
     <row r="388">
       <c r="A388" s="6" t="inlineStr">
         <is>
-          <t>UPD-04</t>
+          <t>UPD-02</t>
         </is>
       </c>
       <c r="B388" s="7" t="inlineStr">
@@ -16222,29 +16222,29 @@
           <t>Updates</t>
         </is>
       </c>
-      <c r="C388" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C388" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D388" s="9" t="inlineStr">
         <is>
-          <t>Unreachable server says NOTHING, never 'up to date'</t>
+          <t>Web offers a reload, and says drafts are kept</t>
         </is>
       </c>
       <c r="E388" s="9" t="inlineStr">
         <is>
-          <t>Put the device in aeroplane mode and open Settings. Then, online, confirm doubledone.app/version.json returns JSON rather than the app's HTML (the SPA fallback would break it silently).</t>
+          <t>With doubledone.app/version.json's "web" set ahead of the running build, open Settings on the web.</t>
         </is>
       </c>
       <c r="F388" s="9" t="inlineStr">
         <is>
-          <t>No update line at all, and no 'Up to date' either: it cannot tell, so it says nothing. No spinner and no error.</t>
+          <t>'A newer version is ready.' + 'Reload to get it' + 'Anything you were typing is kept.' Type something into the capture box first and confirm it survives the reload.</t>
         </is>
       </c>
       <c r="G388" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H388" s="7" t="inlineStr"/>
@@ -16254,7 +16254,7 @@
     <row r="389">
       <c r="A389" s="6" t="inlineStr">
         <is>
-          <t>UPD-05</t>
+          <t>UPD-03</t>
         </is>
       </c>
       <c r="B389" s="7" t="inlineStr">
@@ -16262,29 +16262,29 @@
           <t>Updates</t>
         </is>
       </c>
-      <c r="C389" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C389" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D389" s="9" t="inlineStr">
         <is>
-          <t>The goodnight mention is rare, and framed for the other person</t>
+          <t>Native points at the store, and says lists are untouched</t>
         </is>
       </c>
       <c r="E389" s="9" t="inlineStr">
         <is>
-          <t>Clear the day with a build two minor versions behind, and reach the rested screen.</t>
+          <t>With version.json's "ios" / "android" set ahead of the installed build, open Settings on a device.</t>
         </is>
       </c>
       <c r="F389" s="9" t="inlineStr">
         <is>
-          <t>At most ONE offer shows. If it is the update one it reads 'The newer one can read everything your person sets, rhythms included.' 'Not now' dismisses it and it does not return for a fortnight. It never displaces the reminder, widget or scrapbook offer.</t>
+          <t>'This build is getting old.' + 'Open the store' + 'Your lists stay exactly as they are.' The button opens the correct store listing.</t>
         </is>
       </c>
       <c r="G389" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H389" s="7" t="inlineStr"/>
@@ -16294,32 +16294,32 @@
     <row r="390">
       <c r="A390" s="6" t="inlineStr">
         <is>
-          <t>OUR-12</t>
+          <t>UPD-04</t>
         </is>
       </c>
       <c r="B390" s="7" t="inlineStr">
         <is>
-          <t>Ours</t>
-        </is>
-      </c>
-      <c r="C390" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>Updates</t>
+        </is>
+      </c>
+      <c r="C390" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D390" s="9" t="inlineStr">
         <is>
-          <t>Unnamed lists read in each person's language</t>
+          <t>Unreachable server says NOTHING, never 'up to date'</t>
         </is>
       </c>
       <c r="E390" s="9" t="inlineStr">
         <is>
-          <t>Create a list WITHOUT naming it. Set the two accounts' devices to different languages (e.g. English and Italian).</t>
+          <t>Put the device in aeroplane mode and open Settings. Then, online, confirm doubledone.app/version.json returns JSON rather than the app's HTML (the SPA fallback would break it silently).</t>
         </is>
       </c>
       <c r="F390" s="9" t="inlineStr">
         <is>
-          <t>Each person sees the app's own word for a shared list in their own language, not the other person's.</t>
+          <t>No update line at all, and no 'Up to date' either: it cannot tell, so it says nothing. No spinner and no error.</t>
         </is>
       </c>
       <c r="G390" s="7" t="inlineStr">
@@ -16331,9 +16331,89 @@
       <c r="I390" s="9" t="inlineStr"/>
       <c r="J390" s="7" t="inlineStr"/>
     </row>
+    <row r="391">
+      <c r="A391" s="6" t="inlineStr">
+        <is>
+          <t>UPD-05</t>
+        </is>
+      </c>
+      <c r="B391" s="7" t="inlineStr">
+        <is>
+          <t>Updates</t>
+        </is>
+      </c>
+      <c r="C391" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D391" s="9" t="inlineStr">
+        <is>
+          <t>The goodnight mention is rare, and framed for the other person</t>
+        </is>
+      </c>
+      <c r="E391" s="9" t="inlineStr">
+        <is>
+          <t>Clear the day with a build two minor versions behind, and reach the rested screen.</t>
+        </is>
+      </c>
+      <c r="F391" s="9" t="inlineStr">
+        <is>
+          <t>At most ONE offer shows. If it is the update one it reads 'The newer one can read everything your person sets, rhythms included.' 'Not now' dismisses it and it does not return for a fortnight. It never displaces the reminder, widget or scrapbook offer.</t>
+        </is>
+      </c>
+      <c r="G391" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H391" s="7" t="inlineStr"/>
+      <c r="I391" s="9" t="inlineStr"/>
+      <c r="J391" s="7" t="inlineStr"/>
+    </row>
+    <row r="392">
+      <c r="A392" s="6" t="inlineStr">
+        <is>
+          <t>OUR-12</t>
+        </is>
+      </c>
+      <c r="B392" s="7" t="inlineStr">
+        <is>
+          <t>Ours</t>
+        </is>
+      </c>
+      <c r="C392" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D392" s="9" t="inlineStr">
+        <is>
+          <t>Unnamed lists read in each person's language</t>
+        </is>
+      </c>
+      <c r="E392" s="9" t="inlineStr">
+        <is>
+          <t>Create a list WITHOUT naming it. Set the two accounts' devices to different languages (e.g. English and Italian).</t>
+        </is>
+      </c>
+      <c r="F392" s="9" t="inlineStr">
+        <is>
+          <t>Each person sees the app's own word for a shared list in their own language, not the other person's.</t>
+        </is>
+      </c>
+      <c r="G392" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H392" s="7" t="inlineStr"/>
+      <c r="I392" s="9" t="inlineStr"/>
+      <c r="J392" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J390"/>
-  <conditionalFormatting sqref="H2:H390">
+  <autoFilter ref="A1:J392"/>
+  <conditionalFormatting sqref="H2:H392">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -16345,7 +16425,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H390" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H392" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -16381,7 +16461,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>389</t>
+          <t>391</t>
         </is>
       </c>
     </row>
@@ -16392,7 +16472,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$390,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$392,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -16403,7 +16483,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$390,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$392,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -16414,7 +16494,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$390,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$392,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -16425,7 +16505,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$390,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$392,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -16436,7 +16516,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>389-COUNTA('Test Suite'!$H$2:$H$390)</f>
+        <f>391-COUNTA('Test Suite'!$H$2:$H$392)</f>
         <v/>
       </c>
     </row>
@@ -16447,7 +16527,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$390,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$392,"P1")</f>
         <v/>
       </c>
     </row>
@@ -16458,7 +16538,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$390,"P1",'Test Suite'!$H$2:$H$390,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$392,"P1",'Test Suite'!$H$2:$H$392,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(ours): a waiting pair gets its bridge line on the shared list
Melroy's C6 check: with a pair minted but unjoined, the Menu lands on
the list, whose header seat rendered nothing, a dead end hiding the
waiting screen and its re-mint. The seat now reads "Waiting for your
person - Get a new code" and links to the pairing screen. Existing
strings, so all five locales ride free.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -11909,17 +11909,17 @@
       </c>
       <c r="D280" s="9" t="inlineStr">
         <is>
-          <t>Waiting-with-no-code says so, and the re-mint is a real button</t>
+          <t>Waiting-with-no-code is reachable, says so, and the re-mint is a real button</t>
         </is>
       </c>
       <c r="E280" s="9" t="inlineStr">
         <is>
-          <t>Mint a code, leave Ours entirely (back to Today), then come back to Ours before anyone joins.</t>
+          <t>Mint a code, leave Ours entirely (back to Today), then come back via the MENU's Ours row before anyone joins.</t>
         </is>
       </c>
       <c r="F280" s="9" t="inlineStr">
         <is>
-          <t>The screen is titled 'Waiting for your person', NOT 'Read this to your person' over an empty space (the code renders exactly once; the server keeps only a hash, so it can never be re-shown). 'Get a new code' is a full primary button in this state, not a quiet text link (the 2026-09-13 field report walked right past the link: 'no easy way to... regenerate the code'). While the code IS still on screen, the title and the quiet link stay as they were.</t>
+          <t>The Menu lands on the shared LIST (usable solo while waiting), and the list's header line reads 'Waiting for your person - Get a new code' where 'Kept with {name}' will later sit; tapping it opens the pairing screen (both Melroy's C6 check and the field report hit this as a dead end before 2026-09-20). That screen is titled 'Waiting for your person', NOT 'Read this to your person' over an empty space (the code renders exactly once; the server keeps only a hash, so it can never be re-shown), and 'Get a new code' is a full primary button there, not a quiet text link. While the code IS still on screen, the old title and quiet link stay as they were.</t>
         </is>
       </c>
       <c r="G280" s="7" t="inlineStr">

</xml_diff>

<commit_message>
fix(capture): When and Add clear Safari's floating address label on iPhone
Melroy's iPhone screenshot: with the keyboard up in Safari, the panel sat
correctly on the keyboard (the visualViewport lift works), but Safari's
small floating address label ("today-v3.doubledone.pages.dev") lay right
over When and Add. The label is Safari's chrome drawn inside the visual
viewport and in no safe-area inset, so the page cannot measure it.

The panel's foot keeps 44pt clear of it, only where it exists: iPhone
Safari in a tab, with the keyboard up. Not the home-screen app (no browser
chrome), not Chrome, Firefox, Edge, Opera, the Google app or in-app web
views, not iPad, not Android. The detection is pure and unit-tested in
lib/safari-chrome. The panel's floor includes the extra room, so the fixed
rows still fit.

CAP-13 now covers iPhone Safari and the home-screen app (platform Both).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -1246,12 +1246,12 @@
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>On a real Android phone (app and browser separately), tap the + pill, then tap the box, and watch the panel as the keyboard rises. Type a line, tap the When chip, pick Weekly, tap the box again, Add. Repeat at a large font-size setting, and on an iPhone.</t>
+          <t>On a real Android phone (app and browser separately), tap the + pill, then tap the box, and watch the panel as the keyboard rises. Type a line, tap the When chip, pick Weekly, tap the box again, Add. Repeat at a large font-size setting, on an iPhone in Safari (a normal tab), and in the iPhone home-screen app.</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>The panel sits on top of the keyboard: its heading and Close, the box (shrunk to its minimum first), the tools row, When and Add all stay in view, so you can see what you type and reach Add without dismissing the keyboard. Opening When puts the keyboard away and shows the choices; tapping the box brings the keyboard back and folds When to its chip. REGRESSION GUARD: a tester's v19 screenshots showed only 'ADD / Close' with everything else under the keyboard, because edge-to-edge Android ignores adjustResize and Chrome 108+ overlays the keyboard by default; the fix is the panel's own keyboard lift (native) + interactive-widget=resizes-content (web).</t>
+          <t>The panel sits on top of the keyboard: its heading and Close, the box (shrunk to its minimum first), the tools row, When and Add all stay in view, so you can see what you type and reach Add without dismissing the keyboard. Opening When puts the keyboard away and shows the choices; tapping the box brings the keyboard back and folds When to its chip. In iPhone Safari, Safari's own small address label floats just above the keyboard: When and Add sit clear above it, never under it (Melroy's screenshot, 2026-09-27, before lib/safari-chrome). REGRESSION GUARD: a tester's v19 screenshots showed only 'ADD / Close' with everything else under the keyboard, because edge-to-edge Android ignores adjustResize and Chrome 108+ overlays the keyboard by default; the fix is the panel's own keyboard lift (native) + interactive-widget=resizes-content (web).</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">

</xml_diff>

<commit_message>
fix(android): MainActivity back to singleTask, because singleTop broke sharing
Device test 8g: with singleTop every share from Chrome opened a new
DoubleDone inside Chrome's task, so recents filled with copies and later
shares broke. Back to expo-share-intent's default, the fallback decided in
advance. The accepted cost is RevenueCat's warning that a purchase which
detours through a bank app can come back as cancelled in the sheet; Google
still completes it and the webhook still records it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -11923,7 +11923,7 @@
       </c>
       <c r="F280" s="9" t="inlineStr">
         <is>
-          <t>Every share lands in Today's capture box. There is only ever ONE DoubleDone (the launcher does not open a second copy on top), and Back from DoubleDone returns to Chrome. The purchase sheet survives the app switch and completes. If it does not (RevenueCat's singleTask warning), the pre-decided fallback is to go back to singleTask and accept the warning: record what happened and tell Claude before any production upload.</t>
+          <t>Every share lands in Today's capture box. There is only ever ONE DoubleDone (the launcher does not open a second copy on top), and Back from DoubleDone returns to Chrome. The purchase sheet survives the app switch and completes. The build is singleTask (singleTop failed this case on 2026-10-03, opening a copy per share). If the purchase sheet comes back as cancelled after a bank-app detour, that is RevenueCat's known singleTask cost: Premium must still appear within a minute or two (the webhook records Google's completed purchase), and nothing is charged twice.</t>
         </is>
       </c>
       <c r="G280" s="7" t="inlineStr">
@@ -12083,7 +12083,7 @@
       </c>
       <c r="F284" s="9" t="inlineStr">
         <is>
-          <t>com.android.billingclient IS in the AAB (react-native-purchases now autolinks: the old expo.autolinking.android.exclude is gone from client/package.json). The merged manifest gains com.android.vending.BILLING and nothing else new; in particular there is NO com.google.android.gms.permission.AD_ID (if it appears, block it in app.json and rebuild before any upload). MainActivity's launchMode is singleTop, not singleTask (the expo-share-intent option in app.json). This is the regression guard on Path A's build config.</t>
+          <t>com.android.billingclient IS in the AAB (react-native-purchases now autolinks: the old expo.autolinking.android.exclude is gone from client/package.json). The merged manifest gains com.android.vending.BILLING and nothing else new; in particular there is NO com.google.android.gms.permission.AD_ID (if it appears, block it in app.json and rebuild before any upload). MainActivity's launchMode is singleTask, the expo-share-intent default (singleTop was tried and FAILED PREM-57 on 2026-10-03: every share opened another copy of the app). This is the regression guard on Path A's build config.</t>
         </is>
       </c>
       <c r="G284" s="7" t="inlineStr">

</xml_diff>

<commit_message>
fix(left-off): the line field rises above the keyboard, and the mark sits on the first line
Two things Melroy saw on the 1.8.0 TestFlight build. A task low on Today opened its
editor with the line field under the keyboard: iOS reserved the room
(automaticallyAdjustKeyboardInsets) but nothing scrolled the field into it, the step the
handoff's keyboard plan asked for and the first build left out. Today now measures the
open card's line field once the keyboard is up and scrolls the list by the overlap only,
so a card already in view never moves. And the dog-ear sat about 6px high beside the
field's placeholder: it was pinned to the row's top while the words start below the
field's own padding. It now centres on the first line of the words, in the editor and
on the card, so a wrapped line keeps its mark beside its first words.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -19399,7 +19399,7 @@
       </c>
       <c r="F467" s="9" t="inlineStr">
         <is>
-          <t>'Noted.' shows in the affirm line, once. The card stays open and shows the dog-ear, the words and today's calendar date (e.g. 'Sun, 4 Oct', never 'today') directly under the title. Shut the card: the Today row shows the dog-ear straight after the title and nothing else; the row is the same height as before. A screen reader hears the row label end ', has a note'. Return on the title field moves to the line field rather than closing.</t>
+          <t>'Noted.' shows in the affirm line, once. The card stays open and shows the dog-ear (level with the FIRST line of the words, in the editor and on the card, never above it), the words and today's calendar date (e.g. 'Sun, 4 Oct', never 'today') directly under the title. Shut the card: the Today row shows the dog-ear straight after the title and nothing else; the row is the same height as before. A screen reader hears the row label end ', has a note'. Return on the title field moves to the line field rather than closing.</t>
         </is>
       </c>
       <c r="G467" s="7" t="inlineStr">
@@ -19759,7 +19759,7 @@
       </c>
       <c r="F476" s="9" t="inlineStr">
         <is>
-          <t>On Android and iOS the focused field stays above the keyboard (the list can scroll far enough). In Focus the slip stays visible above the keyboard, and Done and Choose another stay reachable by scrolling. On Android Chrome the page resizes rather than hiding the field.</t>
+          <t>On Android and iOS the list scrolls BY ITSELF so the line field sits just above the keyboard, the moment the keyboard is up (Melroy's iPhone, 2026-10-05: before the fix it hid under it); a card already clear of the keyboard does not move at all. In Focus the slip stays visible above the keyboard, and Done and Choose another stay reachable by scrolling. On Android Chrome the page resizes rather than hiding the field.</t>
         </is>
       </c>
       <c r="G476" s="7" t="inlineStr">

</xml_diff>

<commit_message>
feat(left-off): the held card shows the empty line under the title, so the note is findable
Melroy on the first TestFlight build: it was not obvious, until he tapped the title, that
a task could carry a note. An eligible task with no line now shows the field at rest on
the held card (the mark and 'Where you left off, for next time', over a hairline, or
Quiet's filled slip so the soft ink still clears 4.5:1), and a tap opens the editor on
the line. Today's rows are unchanged ('ONLY when you tap and hold'). This reverses the
handoff's empty-card rule; the cost is one 44pt row on those cards. New string
leftOff.addA11y in all five languages.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -19394,7 +19394,7 @@
       </c>
       <c r="E467" s="9" t="inlineStr">
         <is>
-          <t>Hold a one-off task on Today and tap its title. Under the title a second field appears, led by a dog-ear mark: 'Where you left off, for next time'. Type 'Called, ref 4471, ring back Thu' and press the keyboard's done key.</t>
+          <t>Hold a one-off task with no line on Today. Under the title, BEFORE anything is tapped, the card shows the dog-ear and 'Where you left off, for next time' (a hairline under it; a filled slip on Quiet); Today's rows show nothing new. Tap that line: the editor opens with the line field focused. Type 'Called, ref 4471, ring back Thu' and press the keyboard's done key. (Tapping the title also opens the same editor.)</t>
         </is>
       </c>
       <c r="F467" s="9" t="inlineStr">
@@ -19599,7 +19599,7 @@
       </c>
       <c r="F472" s="9" t="inlineStr">
         <is>
-          <t>The repeating card keeps today's single-field title editor and shows no mark or line. The Ours list rows have no line field. The shared row created from a task with a line carries NO line (the partner never sees it). Your '· Ours' copy on Today can carry a line of its own: the dog-ear sits after the title, before '· Ours', and the partner's devices never show it. A ticked (done) task shows no line or mark, and gets it back unchanged if un-ticked.</t>
+          <t>The repeating card keeps today's single-field title editor and shows no mark, no line and no empty line under its title (nor does a done card). The Ours list rows have no line field. The shared row created from a task with a line carries NO line (the partner never sees it). Your '· Ours' copy on Today can carry a line of its own: the dog-ear sits after the title, before '· Ours', and the partner's devices never show it. A ticked (done) task shows no line or mark, and gets it back unchanged if un-ticked.</t>
         </is>
       </c>
       <c r="G472" s="7" t="inlineStr">

</xml_diff>

<commit_message>
fix(web): the landing review's 26 confirmed findings, and two more privacy-policy fixes
Six reviewers and a skeptic per finding confirmed 26 problems. The three
majors: the policy said no record exists of who added a shared item (the
server does note it; Melroy approved the correction and a matching line in
Your control), and the page painted 8px wider until the app bundle reset the
body margin, then jumped.

Also: the hero trust line now says the list lives on your device (AI starts
on); Turn AI off and the consent card stop claiming more than the switch
does; the welcome's Ours promise is corrected; one App Store badge per
layout; Android credited; badge names match the printed badges; lists keep
their role for VoiceOver; the laptop column is the board's 640; a calm
no-JavaScript note; CI runs the shipped boot; the capture script refuses a
crop past the viewport and records the size of the file it wrote.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -6131,7 +6131,7 @@
       </c>
       <c r="F135" s="9" t="inlineStr">
         <is>
-          <t>Each picture is that language's own screen (German words on the German page, never English), and switches with the theme: Close the day at rest ('A quiet day, and that's allowed.'), Here's the plan for Do my taxes with five steps carrying minutes and a day, the top of Today on a Low day, Settle with the guide's first word, the shared list 'Just us' with Bin night every Sunday and the parcel today, and the Calendar on Sunday 18 October with Do my taxes as the big one. No picture is stretched or cut mid-row, and the page does not jump as they load.</t>
+          <t>Each picture is that language's own screen (German words on the German page, never English), and switches with the theme: Close the day at rest ('A quiet day, and that's allowed.'), Here's the plan for Do my taxes with four steps carrying minutes and a day, the top of Today on a Low day, Settle with the guide's first word, the shared list 'Just us' with Bin night every Sunday and the parcel today, and the Calendar on Sunday 18 October with Do my taxes as the big one. No picture is stretched or cut mid-row, and the page does not jump as they load.</t>
         </is>
       </c>
       <c r="G135" s="7" t="inlineStr">
@@ -9291,7 +9291,7 @@
       </c>
       <c r="F214" s="9" t="inlineStr">
         <is>
-          <t>Turning off is instant with a warm line ('AI is off. Nothing you write goes to an AI.'). Every AI affordance then disappears: Sort for me / Tidy this / Scan in capture; Break it down / Make it tiny / Combine / Plan my day on Today, including the per-task Break-down and Make-tiny; the 'Chart a course' menu entry (and the screen redirects away); and Calendar's scrapbook + weekly reflection. On-device Speak stays. Nothing calls the AI backend and the calm to-do loop still works fully.</t>
+          <t>Turning off is instant with a warm line ('AI is off. The app's AI features send nothing you write.', and when signed in, a second line that a connected AI assistant keeps its access until Disconnect AI connectors). Every AI affordance then disappears: Sort for me / Tidy this / Scan in capture; Break it down / Make it tiny / Combine / Plan my day on Today, including the per-task Break-down and Make-tiny; the 'Chart a course' menu entry (and the screen redirects away); and Calendar's scrapbook + weekly reflection. On-device Speak stays. Nothing calls the AI backend and the calm to-do loop still works fully.</t>
         </is>
       </c>
       <c r="G214" s="7" t="inlineStr">
@@ -9331,7 +9331,7 @@
       </c>
       <c r="F215" s="9" t="inlineStr">
         <is>
-          <t>Turning ON asks first: a card naming exactly what is sent and to whom ('sends the text you choose... to Anthropic's Claude... Nothing else ever leaves your device.'). 'Not now' cancels with no change. 'Turn on AI' restores every AI affordance across the app. The asymmetry is deliberate: off is one instant tap, on is a clear informed tap.</t>
+          <t>Turning ON asks first: a card naming exactly what is sent and to whom ('sends the text you choose... to Anthropic's Claude... Nothing else goes to an AI.'). 'Not now' cancels with no change. 'Turn on AI' restores every AI affordance across the app. The asymmetry is deliberate: off is one instant tap, on is a clear informed tap.</t>
         </is>
       </c>
       <c r="G215" s="7" t="inlineStr">

</xml_diff>

<commit_message>
fix(mcp,api): never write a task that is already removed
MCP update_task's plain field change and delete_task, and REST DELETE,
were the only writes on either surface without deleted_at=is.null (the
server map's finding 4). So a rename of a removed task answered
"Updated." for a task nobody could see, and a second removal re-stamped
the tombstone's time. The app's repair reads that time to recognise a
task folded by Combine and to keep Remove's Undo on offer, so moving it
could unpick both.

All three are now pinned to a live row. A removed task answers "No
matching task found." over MCP. REST DELETE still answers 204 when
nothing matched, so a retried delete stays harmless (a 404 there would
make a retry read as a failure, and the route never returned one).

MCP-14 now removes twice and renames the removed task. Server tests 872
(2 new).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -8606,12 +8606,12 @@
       </c>
       <c r="E197" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent to remove a task by id. PREREQ: MCP-01.</t>
+          <t>Ask the agent to remove a task by id. Then ask it to remove the same id again, and to rename it. PREREQ: MCP-01.</t>
         </is>
       </c>
       <c r="F197" s="9" t="inlineStr">
         <is>
-          <t>The task disappears from the app (hidden), confirmed 'Removed.' It is soft-deleted (deleted_at set), never hard-deleted; the tombstone syncs across devices.</t>
+          <t>The task disappears from the app (hidden), confirmed 'Removed.' It is soft-deleted (deleted_at set), never hard-deleted; the tombstone syncs across devices. The second removal and the rename each answer 'No matching task found.' and change nothing (the removal's time stays as it was, so the app's Undo still finds it).</t>
         </is>
       </c>
       <c r="G197" s="7" t="inlineStr">

</xml_diff>

<commit_message>
docs(release): a failed VoiceOver check cuts the App Review notes' claim too
The cut table said a failed A11Y-07 removes the "With VoiceOver on" sentence
from the five Apple blocks. The App Review notes make the same claim on their
own ("gives VoiceOver an Options action on every task"), the table never named
them, and DEP-05 diffed What's New only. A failed check would have left the
reviewer reading about a VoiceOver feature that does not work.

The A11Y-07 row now names the notes, and a line under the table says what
their paragraph becomes and that their count drops from 2646 to 2594. DEP-05
diffs the notes against App Review Information too, and step (14) pastes them
after the cut table. The suite is regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -11086,12 +11086,12 @@
       </c>
       <c r="E259" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: the 1.9.0 version in App Store Connect with its seven localisations added (slice 8), the 1.9.0 Play release drafted, and the device checks A11Y-07, A11Y-08 and I18N-02 already run. In App Store Connect open each localisation in turn (the primary English, the second English, German, French, Italian, Spanish (Mexico), Spanish (Spain)) and read its What's New. In Play Console read the release notes in each language. Print each block from docs/release-notes/1.9.0.md and diff it against what the console shows.</t>
+          <t>PREREQ: the 1.9.0 version in App Store Connect with its seven localisations added (slice 8), the 1.9.0 Play release drafted, and the device checks A11Y-07, A11Y-08 and I18N-02 already run. In App Store Connect open each localisation in turn (the primary English, the second English, German, French, Italian, Spanish (Mexico), Spanish (Spain)) and read its What's New. In Play Console read the release notes in each language. Print each block from docs/release-notes/1.9.0.md and diff it against what the console shows. Then open App Review Information on the 1.9.0 version and diff its Notes against the file's App Review notes block.</t>
         </is>
       </c>
       <c r="F259" s="9" t="inlineStr">
         <is>
-          <t>All seven App Store localisations show What's New in their own language (the same English in both English ones, the same neutral Spanish in both Spanish ones). None is empty and none carries another language's text, because nothing inherits it. Play shows six languages, en-AU, de-DE, es-419, es-ES, fr-FR and it-IT, with es-419 and es-ES identical. Every diff is empty: the French keeps its no-break spaces and every language its accents. Neither store's notes mention the rating card, a price, a trial or Premium. A sentence the file's cut table names for a failed device check is gone from every block that table lists.</t>
+          <t>All seven App Store localisations show What's New in their own language (the same English in both English ones, the same neutral Spanish in both Spanish ones). None is empty and none carries another language's text, because nothing inherits it. Play shows six languages, en-AU, de-DE, es-419, es-ES, fr-FR and it-IT, with es-419 and es-ES identical. Every diff is empty: the French keeps its no-break spaces and every language its accents. Neither store's notes mention the rating card, a price, a trial or Premium. A sentence the file's cut table names for a failed device check is gone from every block that table lists, the App Review notes included: after a failed A11Y-07 they no longer mention VoiceOver.</t>
         </is>
       </c>
       <c r="G259" s="7" t="inlineStr">

</xml_diff>

<commit_message>
fix(terms): the iPhone's Premium paragraph names the App Store's price, never ours
On an iPhone the in-app Terms said Premium costs A$5 or A$50 on our
website: the same wrong-currency figure the welcome no longer shows, and a
website price inside the iPhone app. The iPhone now gets its own paragraph,
the way Android has one: sold through the App Store, at the price it shows
before you buy, in your own currency, cancelled in Apple ID settings. Melroy
approved the wording (2026-10-19). The web Terms keep the Stripe figures.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$525</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$526</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J525"/>
+  <dimension ref="A1:J526"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -17534,12 +17534,12 @@
     <row r="421">
       <c r="A421" s="6" t="inlineStr">
         <is>
-          <t>OUR-42</t>
+          <t>LEG-07</t>
         </is>
       </c>
       <c r="B421" s="7" t="inlineStr">
         <is>
-          <t>Ours</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="C421" s="8" t="inlineStr">
@@ -17549,22 +17549,22 @@
       </c>
       <c r="D421" s="9" t="inlineStr">
         <is>
-          <t>A change on one phone appears on the other WITHOUT touching it</t>
+          <t>The iPhone's Terms name no price of ours and no website price</t>
         </is>
       </c>
       <c r="E421" s="9" t="inlineStr">
         <is>
-          <t>Both sit on the shared list. One adds a task. Do not touch the other device.</t>
+          <t>On an iPhone (the 1.9.0 App Store or TestFlight build), open Settings &gt; Terms and read 'Premium and billing'. Then open doubledone.app/terms in a browser.</t>
         </is>
       </c>
       <c r="F421" s="9" t="inlineStr">
         <is>
-          <t>It appears within about 15 seconds. (The poll never fired once before 2026-08-09: setPair rebuilt the pair object every sync, which restarted the interval before it could tick.)</t>
+          <t>The iPhone says Premium is sold through the App Store, at the price the App Store shows before you buy, in your own currency, charged to your Apple ID monthly or yearly, renewing until you cancel in your Apple ID subscription settings. It mentions the free 30 days with no card, and how to cancel a Stripe or Google Play subscription, but shows no A$ figure and no website price anywhere on the screen. The website's Terms still show A$5 a month or A$50 a year (Stripe sells there).</t>
         </is>
       </c>
       <c r="G421" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>iOS + Web</t>
         </is>
       </c>
       <c r="H421" s="7" t="inlineStr"/>
@@ -17574,7 +17574,7 @@
     <row r="422">
       <c r="A422" s="6" t="inlineStr">
         <is>
-          <t>OUR-43</t>
+          <t>OUR-42</t>
         </is>
       </c>
       <c r="B422" s="7" t="inlineStr">
@@ -17589,17 +17589,17 @@
       </c>
       <c r="D422" s="9" t="inlineStr">
         <is>
-          <t>Opening your own list does not bounce you back</t>
+          <t>A change on one phone appears on the other WITHOUT touching it</t>
         </is>
       </c>
       <c r="E422" s="9" t="inlineStr">
         <is>
-          <t>With a live list, tap Ours then 'Open the list'. Also try /ours-list directly in a cold tab.</t>
+          <t>Both sit on the shared list. One adds a task. Do not touch the other device.</t>
         </is>
       </c>
       <c r="F422" s="9" t="inlineStr">
         <is>
-          <t>You land on the list and stay. (useSession returns null while hydrating; the room used to read that as signed-out and redirect, making the button an endless loop.)</t>
+          <t>It appears within about 15 seconds. (The poll never fired once before 2026-08-09: setPair rebuilt the pair object every sync, which restarted the interval before it could tick.)</t>
         </is>
       </c>
       <c r="G422" s="7" t="inlineStr">
@@ -17614,7 +17614,7 @@
     <row r="423">
       <c r="A423" s="6" t="inlineStr">
         <is>
-          <t>OUR-44</t>
+          <t>OUR-43</t>
         </is>
       </c>
       <c r="B423" s="7" t="inlineStr">
@@ -17622,24 +17622,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C423" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C423" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D423" s="9" t="inlineStr">
         <is>
-          <t>The pairing screen offers a way INTO the list</t>
+          <t>Opening your own list does not bounce you back</t>
         </is>
       </c>
       <c r="E423" s="9" t="inlineStr">
         <is>
-          <t>Finish pairing, then look at the pairing screen.</t>
+          <t>With a live list, tap Ours then 'Open the list'. Also try /ours-list directly in a cold tab.</t>
         </is>
       </c>
       <c r="F423" s="9" t="inlineStr">
         <is>
-          <t>There is an 'Open the list' button. (It used to dead-end: the only route to the room was Today's door or the Menu, which a new pair has no reason to know about.)</t>
+          <t>You land on the list and stay. (useSession returns null while hydrating; the room used to read that as signed-out and redirect, making the button an endless loop.)</t>
         </is>
       </c>
       <c r="G423" s="7" t="inlineStr">
@@ -17654,7 +17654,7 @@
     <row r="424">
       <c r="A424" s="6" t="inlineStr">
         <is>
-          <t>OUR-45</t>
+          <t>OUR-44</t>
         </is>
       </c>
       <c r="B424" s="7" t="inlineStr">
@@ -17669,17 +17669,17 @@
       </c>
       <c r="D424" s="9" t="inlineStr">
         <is>
-          <t>The quiet wash appears and then takes itself away</t>
+          <t>The pairing screen offers a way INTO the list</t>
         </is>
       </c>
       <c r="E424" s="9" t="inlineStr">
         <is>
-          <t>Have the other account change a row while you are elsewhere, then open the list.</t>
+          <t>Finish pairing, then look at the pairing screen.</t>
         </is>
       </c>
       <c r="F424" s="9" t="inlineStr">
         <is>
-          <t>The changed row carries ONE warmed border, on the card itself, never a second ring around it. It clears itself after about 8 seconds without animating. It does not return on the next visit, even if the other phone's clock runs ahead.</t>
+          <t>There is an 'Open the list' button. (It used to dead-end: the only route to the room was Today's door or the Menu, which a new pair has no reason to know about.)</t>
         </is>
       </c>
       <c r="G424" s="7" t="inlineStr">
@@ -17694,7 +17694,7 @@
     <row r="425">
       <c r="A425" s="6" t="inlineStr">
         <is>
-          <t>OUR-47</t>
+          <t>OUR-45</t>
         </is>
       </c>
       <c r="B425" s="7" t="inlineStr">
@@ -17702,24 +17702,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C425" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C425" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D425" s="9" t="inlineStr">
         <is>
-          <t>Ours lives in Today's heading (Today v3)</t>
+          <t>The quiet wash appears and then takes itself away</t>
         </is>
       </c>
       <c r="E425" s="9" t="inlineStr">
         <is>
-          <t>With a live list, look at the top of Today. Then leave the list (or sign out) and look again. With a screen reader, move through the heading.</t>
+          <t>Have the other account change a row while you are elsewhere, then open the list.</t>
         </is>
       </c>
       <c r="F425" s="9" t="inlineStr">
         <is>
-          <t>With a live list the heading reads 'Today' and the list's name side by side (its own name when it has one, else 'Ours'), 'Today' underlined as the current tab. With no live list there is only 'Today', and no empty space where Ours would be. A screen reader hears them as tabs, 'Today, selected' and '{name}'. The old Ours door card under the list is gone.</t>
+          <t>The changed row carries ONE warmed border, on the card itself, never a second ring around it. It clears itself after about 8 seconds without animating. It does not return on the next visit, even if the other phone's clock runs ahead.</t>
         </is>
       </c>
       <c r="G425" s="7" t="inlineStr">
@@ -17734,7 +17734,7 @@
     <row r="426">
       <c r="A426" s="6" t="inlineStr">
         <is>
-          <t>OUR-48</t>
+          <t>OUR-47</t>
         </is>
       </c>
       <c r="B426" s="7" t="inlineStr">
@@ -17749,17 +17749,17 @@
       </c>
       <c r="D426" s="9" t="inlineStr">
         <is>
-          <t>Their tick marks your copy DONE and leaves it on your day</t>
+          <t>Ours lives in Today's heading (Today v3)</t>
         </is>
       </c>
       <c r="E426" s="9" t="inlineStr">
         <is>
-          <t>A has an open brought copy on Today. B ticks that row in Ours. A backgrounds the app and returns to Today WITHOUT navigating.</t>
+          <t>With a live list, look at the top of Today. Then leave the list (or sign out) and look again. With a screen reader, move through the heading.</t>
         </is>
       </c>
       <c r="F426" s="9" t="inlineStr">
         <is>
-          <t>The copy is still there, ticked, NOT gone. It appears in A's Lookback. Nothing anywhere says which of them did it. (Before 2026-08-11 it was tombstoned and replaced by a note, and for three rounds it vanished outright because it was marked done with no completion date.)</t>
+          <t>With a live list the heading reads 'Today' and the list's name side by side (its own name when it has one, else 'Ours'), 'Today' underlined as the current tab. With no live list there is only 'Today', and no empty space where Ours would be. A screen reader hears them as tabs, 'Today, selected' and '{name}'. The old Ours door card under the list is gone.</t>
         </is>
       </c>
       <c r="G426" s="7" t="inlineStr">
@@ -17774,7 +17774,7 @@
     <row r="427">
       <c r="A427" s="6" t="inlineStr">
         <is>
-          <t>OUR-49</t>
+          <t>OUR-48</t>
         </is>
       </c>
       <c r="B427" s="7" t="inlineStr">
@@ -17789,17 +17789,17 @@
       </c>
       <c r="D427" s="9" t="inlineStr">
         <is>
-          <t>A settled copy carries a completion DATE, not just a done flag</t>
+          <t>Their tick marks your copy DONE and leaves it on your day</t>
         </is>
       </c>
       <c r="E427" s="9" t="inlineStr">
         <is>
-          <t>After OUR-48, open Today with ?debug=1 and read the `copy` line for that task.</t>
+          <t>A has an open brought copy on Today. B ticks that row in Ours. A backgrounds the app and returns to Today WITHOUT navigating.</t>
         </is>
       </c>
       <c r="F427" s="9" t="inlineStr">
         <is>
-          <t>done=true, doneDay = today's date, showsToday=true. A done task with doneDay=none is invisible on Today AND absent from Lookback: tasksForToday places a finished task by its completion day.</t>
+          <t>The copy is still there, ticked, NOT gone. It appears in A's Lookback. Nothing anywhere says which of them did it. (Before 2026-08-11 it was tombstoned and replaced by a note, and for three rounds it vanished outright because it was marked done with no completion date.)</t>
         </is>
       </c>
       <c r="G427" s="7" t="inlineStr">
@@ -17814,7 +17814,7 @@
     <row r="428">
       <c r="A428" s="6" t="inlineStr">
         <is>
-          <t>OUR-50</t>
+          <t>OUR-49</t>
         </is>
       </c>
       <c r="B428" s="7" t="inlineStr">
@@ -17822,24 +17822,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C428" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C428" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D428" s="9" t="inlineStr">
         <is>
-          <t>A finished copy can be brought over again</t>
+          <t>A settled copy carries a completion DATE, not just a done flag</t>
         </is>
       </c>
       <c r="E428" s="9" t="inlineStr">
         <is>
-          <t>After OUR-48, hold that row in Ours.</t>
+          <t>After OUR-48, open Today with ?debug=1 and read the `copy` line for that task.</t>
         </is>
       </c>
       <c r="F428" s="9" t="inlineStr">
         <is>
-          <t>'Bring to my Today' is offered again, not 'Already on your Today'. (A done copy is not on your plate; while only tombstones were skipped you had a task you could neither see nor re-add.)</t>
+          <t>done=true, doneDay = today's date, showsToday=true. A done task with doneDay=none is invisible on Today AND absent from Lookback: tasksForToday places a finished task by its completion day.</t>
         </is>
       </c>
       <c r="G428" s="7" t="inlineStr">
@@ -17854,7 +17854,7 @@
     <row r="429">
       <c r="A429" s="6" t="inlineStr">
         <is>
-          <t>OUR-51</t>
+          <t>OUR-50</t>
         </is>
       </c>
       <c r="B429" s="7" t="inlineStr">
@@ -17862,24 +17862,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C429" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C429" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D429" s="9" t="inlineStr">
         <is>
-          <t>Your own edit never highlights; their later edit always does</t>
+          <t>A finished copy can be brought over again</t>
         </is>
       </c>
       <c r="E429" s="9" t="inlineStr">
         <is>
-          <t>B ticks a row (A highlights). A un-ticks it. B ticks it again. Watch both screens throughout.</t>
+          <t>After OUR-48, hold that row in Ours.</t>
         </is>
       </c>
       <c r="F429" s="9" t="inlineStr">
         <is>
-          <t>Each side lights up for the OTHER's change every time, including repeatedly on the same row, and never for its own. (`mine` records WHEN you wrote a row, not merely that you did; as a plain id set, one touch made that row permanently dark on that device.)</t>
+          <t>'Bring to my Today' is offered again, not 'Already on your Today'. (A done copy is not on your plate; while only tombstones were skipped you had a task you could neither see nor re-add.)</t>
         </is>
       </c>
       <c r="G429" s="7" t="inlineStr">
@@ -17894,7 +17894,7 @@
     <row r="430">
       <c r="A430" s="6" t="inlineStr">
         <is>
-          <t>OUR-52</t>
+          <t>OUR-51</t>
         </is>
       </c>
       <c r="B430" s="7" t="inlineStr">
@@ -17902,24 +17902,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C430" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C430" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D430" s="9" t="inlineStr">
         <is>
-          <t>The highlight arrives at once and fades away</t>
+          <t>Your own edit never highlights; their later edit always does</t>
         </is>
       </c>
       <c r="E430" s="9" t="inlineStr">
         <is>
-          <t>Have B change a row while A is on the list.</t>
+          <t>B ticks a row (A highlights). A un-ticks it. B ticks it again. Watch both screens throughout.</t>
         </is>
       </c>
       <c r="F430" s="9" t="inlineStr">
         <is>
-          <t>A's row warms immediately, holds about 8 seconds, then fades over roughly 700ms. It does not snap off, does not strobe, and does not return on the next poll for the same change. Reduce-motion gets an instant disappearance instead of a fade.</t>
+          <t>Each side lights up for the OTHER's change every time, including repeatedly on the same row, and never for its own. (`mine` records WHEN you wrote a row, not merely that you did; as a plain id set, one touch made that row permanently dark on that device.)</t>
         </is>
       </c>
       <c r="G430" s="7" t="inlineStr">
@@ -17934,7 +17934,7 @@
     <row r="431">
       <c r="A431" s="6" t="inlineStr">
         <is>
-          <t>OUR-53</t>
+          <t>OUR-52</t>
         </is>
       </c>
       <c r="B431" s="7" t="inlineStr">
@@ -17949,17 +17949,17 @@
       </c>
       <c r="D431" s="9" t="inlineStr">
         <is>
-          <t>Two devices share ONE clock</t>
+          <t>The highlight arrives at once and fades away</t>
         </is>
       </c>
       <c r="E431" s="9" t="inlineStr">
         <is>
-          <t>Open the list on both devices with ?debug=1 and read `skew` on the wash line.</t>
+          <t>Have B change a row while A is on the list.</t>
         </is>
       </c>
       <c r="F431" s="9" t="inlineStr">
         <is>
-          <t>A small value in seconds, not minutes, on both. Every stamp (completion log, last-look, last-write-wins) is compared against server time via server_now(). A device whose clock ran ahead used to stamp its own last-look into the future and could never highlight anything again.</t>
+          <t>A's row warms immediately, holds about 8 seconds, then fades over roughly 700ms. It does not snap off, does not strobe, and does not return on the next poll for the same change. Reduce-motion gets an instant disappearance instead of a fade.</t>
         </is>
       </c>
       <c r="G431" s="7" t="inlineStr">
@@ -17974,7 +17974,7 @@
     <row r="432">
       <c r="A432" s="6" t="inlineStr">
         <is>
-          <t>OUR-54</t>
+          <t>OUR-53</t>
         </is>
       </c>
       <c r="B432" s="7" t="inlineStr">
@@ -17982,24 +17982,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C432" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C432" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D432" s="9" t="inlineStr">
         <is>
-          <t>The debug panel is opt-in and carries no task text</t>
+          <t>Two devices share ONE clock</t>
         </is>
       </c>
       <c r="E432" s="9" t="inlineStr">
         <is>
-          <t>Open /ours-list?debug=1 and /today?debug=1, then the same URLs without the flag.</t>
+          <t>Open the list on both devices with ?debug=1 and read `skew` on the wash line.</t>
         </is>
       </c>
       <c r="F432" s="9" t="inlineStr">
         <is>
-          <t>A small log appears only with the flag, at the top of Today and the foot of the list. Every line is counts, ids and flags. NO task title ever appears in it: these get screenshotted and pasted, and a shared list is two people's words.</t>
+          <t>A small value in seconds, not minutes, on both. Every stamp (completion log, last-look, last-write-wins) is compared against server time via server_now(). A device whose clock ran ahead used to stamp its own last-look into the future and could never highlight anything again.</t>
         </is>
       </c>
       <c r="G432" s="7" t="inlineStr">
@@ -18014,7 +18014,7 @@
     <row r="433">
       <c r="A433" s="6" t="inlineStr">
         <is>
-          <t>OUR-55</t>
+          <t>OUR-54</t>
         </is>
       </c>
       <c r="B433" s="7" t="inlineStr">
@@ -18022,24 +18022,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C433" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C433" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D433" s="9" t="inlineStr">
         <is>
-          <t>Capture on Ours IS Today's capture</t>
+          <t>The debug panel is opt-in and carries no task text</t>
         </is>
       </c>
       <c r="E433" s="9" t="inlineStr">
         <is>
-          <t>Open a shared list and tap the + pill at the foot of the screen.</t>
+          <t>Open /ours-list?debug=1 and /today?debug=1, then the same URLs without the flag.</t>
         </is>
       </c>
       <c r="F433" s="9" t="inlineStr">
         <is>
-          <t>The same pill and the same panel Today has, headed 'Add to {name}': the same box, the same Speak button (web), the same When chip and door, the same Add button naming its own consequence. Not a lookalike, the same component, so the two can never drift apart.</t>
+          <t>A small log appears only with the flag, at the top of Today and the foot of the list. Every line is counts, ids and flags. NO task title ever appears in it: these get screenshotted and pasted, and a shared list is two people's words.</t>
         </is>
       </c>
       <c r="G433" s="7" t="inlineStr">
@@ -18054,7 +18054,7 @@
     <row r="434">
       <c r="A434" s="6" t="inlineStr">
         <is>
-          <t>OUR-56</t>
+          <t>OUR-55</t>
         </is>
       </c>
       <c r="B434" s="7" t="inlineStr">
@@ -18069,17 +18069,17 @@
       </c>
       <c r="D434" s="9" t="inlineStr">
         <is>
-          <t>Repeating can be set AT capture, without knowing a gesture</t>
+          <t>Capture on Ours IS Today's capture</t>
         </is>
       </c>
       <c r="E434" s="9" t="inlineStr">
         <is>
-          <t>In that panel, open the door and choose Daily (or Weekly, or Every N days), then Add.</t>
+          <t>Open a shared list and tap the + pill at the foot of the screen.</t>
         </is>
       </c>
       <c r="F434" s="9" t="inlineStr">
         <is>
-          <t>The button reads 'Add · Daily' before the tap, and the row lands already repeating, visible to both of you. (Before this, the only way to make a repeating shared task was to add it and then somehow know to long-press it. Melroy: 'there is no way to add Repeating Tasks.')</t>
+          <t>The same pill and the same panel Today has, headed 'Add to {name}': the same box, the same Speak button (web), the same When chip and door, the same Add button naming its own consequence. Not a lookalike, the same component, so the two can never drift apart.</t>
         </is>
       </c>
       <c r="G434" s="7" t="inlineStr">
@@ -18094,7 +18094,7 @@
     <row r="435">
       <c r="A435" s="6" t="inlineStr">
         <is>
-          <t>OUR-57</t>
+          <t>OUR-56</t>
         </is>
       </c>
       <c r="B435" s="7" t="inlineStr">
@@ -18102,24 +18102,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C435" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C435" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D435" s="9" t="inlineStr">
         <is>
-          <t>A dump becomes several shared rows, in the order typed</t>
+          <t>Repeating can be set AT capture, without knowing a gesture</t>
         </is>
       </c>
       <c r="E435" s="9" t="inlineStr">
         <is>
-          <t>Type three lines into the Ours capture and Add.</t>
+          <t>In that panel, open the door and choose Daily (or Weekly, or Every N days), then Add.</t>
         </is>
       </c>
       <c r="F435" s="9" t="inlineStr">
         <is>
-          <t>The button reads 'Add 3' and three rows land, in the typed order, on both devices. With a cadence set, all three carry it.</t>
+          <t>The button reads 'Add · Daily' before the tap, and the row lands already repeating, visible to both of you. (Before this, the only way to make a repeating shared task was to add it and then somehow know to long-press it. Melroy: 'there is no way to add Repeating Tasks.')</t>
         </is>
       </c>
       <c r="G435" s="7" t="inlineStr">
@@ -18134,7 +18134,7 @@
     <row r="436">
       <c r="A436" s="6" t="inlineStr">
         <is>
-          <t>OUR-58</t>
+          <t>OUR-57</t>
         </is>
       </c>
       <c r="B436" s="7" t="inlineStr">
@@ -18142,24 +18142,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C436" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C436" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D436" s="9" t="inlineStr">
         <is>
-          <t>The shared door offers When and Repeating, never Steps</t>
+          <t>A dump becomes several shared rows, in the order typed</t>
         </is>
       </c>
       <c r="E436" s="9" t="inlineStr">
         <is>
-          <t>Open the door on Ours and compare it with the door on Today.</t>
+          <t>Type three lines into the Ours capture and Add.</t>
         </is>
       </c>
       <c r="F436" s="9" t="inlineStr">
         <is>
-          <t>Ours shows a When row and a Repeating row, and NO Steps row (a shared row has no slices field, and breaking a thing down is personal). The When row is deliberate: a dated or repeating shared row now reaches BOTH Todays, so a day here is a real act rather than a word that means nothing. See OUR-71 for what the When row rests on.</t>
+          <t>The button reads 'Add 3' and three rows land, in the typed order, on both devices. With a cadence set, all three carry it.</t>
         </is>
       </c>
       <c r="G436" s="7" t="inlineStr">
@@ -18174,7 +18174,7 @@
     <row r="437">
       <c r="A437" s="6" t="inlineStr">
         <is>
-          <t>OUR-59</t>
+          <t>OUR-58</t>
         </is>
       </c>
       <c r="B437" s="7" t="inlineStr">
@@ -18182,24 +18182,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C437" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C437" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D437" s="9" t="inlineStr">
         <is>
-          <t>Typed text survives the panel going</t>
+          <t>The shared door offers When and Repeating, never Steps</t>
         </is>
       </c>
       <c r="E437" s="9" t="inlineStr">
         <is>
-          <t>Type half a sentence into the Ours panel, Close it, tick something, then tap the pill again.</t>
+          <t>Open the door on Ours and compare it with the door on Today.</t>
         </is>
       </c>
       <c r="F437" s="9" t="inlineStr">
         <is>
-          <t>The pill shows '+' and three dots while words wait, and the half sentence is still there. The panel is always mounted, never unmounted. Only an Add resets the door; the words never reset on their own.</t>
+          <t>Ours shows a When row and a Repeating row, and NO Steps row (a shared row has no slices field, and breaking a thing down is personal). The When row is deliberate: a dated or repeating shared row now reaches BOTH Todays, so a day here is a real act rather than a word that means nothing. See OUR-71 for what the When row rests on.</t>
         </is>
       </c>
       <c r="G437" s="7" t="inlineStr">
@@ -18214,7 +18214,7 @@
     <row r="438">
       <c r="A438" s="6" t="inlineStr">
         <is>
-          <t>OUR-60</t>
+          <t>OUR-59</t>
         </is>
       </c>
       <c r="B438" s="7" t="inlineStr">
@@ -18229,22 +18229,22 @@
       </c>
       <c r="D438" s="9" t="inlineStr">
         <is>
-          <t>The Ours panel rides above the keyboard</t>
+          <t>Typed text survives the panel going</t>
         </is>
       </c>
       <c r="E438" s="9" t="inlineStr">
         <is>
-          <t>On a real Android device, tap the + pill on the Ours list, tap the box and start typing.</t>
+          <t>Type half a sentence into the Ours panel, Close it, tick something, then tap the pill again.</t>
         </is>
       </c>
       <c r="F438" s="9" t="inlineStr">
         <is>
-          <t>The panel and its Add button stay visible above the keyboard while you type. Nothing on this stack does this by itself (edge-to-edge Android ignores softwareKeyboardLayoutMode), so it is done by hand and must be re-checked on a device, never only in a browser.</t>
+          <t>The pill shows '+' and three dots while words wait, and the half sentence is still there. The panel is always mounted, never unmounted. Only an Add resets the door; the words never reset on their own.</t>
         </is>
       </c>
       <c r="G438" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H438" s="7" t="inlineStr"/>
@@ -18254,7 +18254,7 @@
     <row r="439">
       <c r="A439" s="6" t="inlineStr">
         <is>
-          <t>OUR-61</t>
+          <t>OUR-60</t>
         </is>
       </c>
       <c r="B439" s="7" t="inlineStr">
@@ -18262,29 +18262,29 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C439" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C439" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D439" s="9" t="inlineStr">
         <is>
-          <t>No AI on the shared capture</t>
+          <t>The Ours panel rides above the keyboard</t>
         </is>
       </c>
       <c r="E439" s="9" t="inlineStr">
         <is>
-          <t>Open the Ours capture panel with AI enabled in Settings, and type a long run-on line.</t>
+          <t>On a real Android device, tap the + pill on the Ours list, tap the box and start typing.</t>
         </is>
       </c>
       <c r="F439" s="9" t="inlineStr">
         <is>
-          <t>No 'Break it down', no 'Sort for me', and no 'Tidy this into tasks': steps or rewrites a model proposes would land on a list another person reads, and pointing a model at somebody else's screen is a decision about them. Speak stays (on-device dictation, not a server call) and so does Scan, which reads a photo INTO the box for you to edit rather than authoring anything, and is the one AI action that belongs here. See OUR-62.</t>
+          <t>The panel and its Add button stay visible above the keyboard while you type. Nothing on this stack does this by itself (edge-to-edge Android ignores softwareKeyboardLayoutMode), so it is done by hand and must be re-checked on a device, never only in a browser.</t>
         </is>
       </c>
       <c r="G439" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H439" s="7" t="inlineStr"/>
@@ -18294,7 +18294,7 @@
     <row r="440">
       <c r="A440" s="6" t="inlineStr">
         <is>
-          <t>OUR-62</t>
+          <t>OUR-61</t>
         </is>
       </c>
       <c r="B440" s="7" t="inlineStr">
@@ -18302,29 +18302,29 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C440" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C440" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D440" s="9" t="inlineStr">
         <is>
-          <t>Scan (premium) reaches the shared capture</t>
+          <t>No AI on the shared capture</t>
         </is>
       </c>
       <c r="E440" s="9" t="inlineStr">
         <is>
-          <t>Premium, AI enabled in Settings. Open the Ours capture on a phone. Tap Scan and photograph a handwritten shopping list.</t>
+          <t>Open the Ours capture panel with AI enabled in Settings, and type a long run-on line.</t>
         </is>
       </c>
       <c r="F440" s="9" t="inlineStr">
         <is>
-          <t>The panel rises with the words IN its box (keyboard down), not on the list. You read them, edit them, and Add them yourself. This is the surface Scan most belongs on: the most photographed list anybody owns is the one on the fridge, and that list is shared by definition.</t>
+          <t>No 'Break it down', no 'Sort for me', and no 'Tidy this into tasks': steps or rewrites a model proposes would land on a list another person reads, and pointing a model at somebody else's screen is a decision about them. Speak stays (on-device dictation, not a server call) and so does Scan, which reads a photo INTO the box for you to edit rather than authoring anything, and is the one AI action that belongs here. See OUR-62.</t>
         </is>
       </c>
       <c r="G440" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H440" s="7" t="inlineStr"/>
@@ -18334,7 +18334,7 @@
     <row r="441">
       <c r="A441" s="6" t="inlineStr">
         <is>
-          <t>OUR-63</t>
+          <t>OUR-62</t>
         </is>
       </c>
       <c r="B441" s="7" t="inlineStr">
@@ -18349,22 +18349,22 @@
       </c>
       <c r="D441" s="9" t="inlineStr">
         <is>
-          <t>Scan on Ours meets the paywall, tagged apart from Today's</t>
+          <t>Scan (premium) reaches the shared capture</t>
         </is>
       </c>
       <c r="E441" s="9" t="inlineStr">
         <is>
-          <t>Sign in as a NON-premium user, open the Ours capture, tap Scan.</t>
+          <t>Premium, AI enabled in Settings. Open the Ours capture on a phone. Tap Scan and photograph a handwritten shopping list.</t>
         </is>
       </c>
       <c r="F441" s="9" t="inlineStr">
         <is>
-          <t>The premium screen opens, the same one Today's Scan opens. Nothing is scanned and nothing is charged. The gate logs reason 'ocr_ours', not 'ocr': a paywall met on a surface a second person can see is a different moment from one met alone.</t>
+          <t>The panel rises with the words IN its box (keyboard down), not on the list. You read them, edit them, and Add them yourself. This is the surface Scan most belongs on: the most photographed list anybody owns is the one on the fridge, and that list is shared by definition.</t>
         </is>
       </c>
       <c r="G441" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H441" s="7" t="inlineStr"/>
@@ -18374,7 +18374,7 @@
     <row r="442">
       <c r="A442" s="6" t="inlineStr">
         <is>
-          <t>OUR-64</t>
+          <t>OUR-63</t>
         </is>
       </c>
       <c r="B442" s="7" t="inlineStr">
@@ -18382,24 +18382,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C442" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C442" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D442" s="9" t="inlineStr">
         <is>
-          <t>The photo never reaches the shared list</t>
+          <t>Scan on Ours meets the paywall, tagged apart from Today's</t>
         </is>
       </c>
       <c r="E442" s="9" t="inlineStr">
         <is>
-          <t>Scan something into Ours and Add it. Check the other device.</t>
+          <t>Sign in as a NON-premium user, open the Ours capture, tap Scan.</t>
         </is>
       </c>
       <c r="F442" s="9" t="inlineStr">
         <is>
-          <t>Your person sees the rows you added and nothing else, exactly as if you had typed them. No image is stored anywhere, shared or otherwise: it is sent to be read, then discarded.</t>
+          <t>The premium screen opens, the same one Today's Scan opens. Nothing is scanned and nothing is charged. The gate logs reason 'ocr_ours', not 'ocr': a paywall met on a surface a second person can see is a different moment from one met alone.</t>
         </is>
       </c>
       <c r="G442" s="7" t="inlineStr">
@@ -18414,7 +18414,7 @@
     <row r="443">
       <c r="A443" s="6" t="inlineStr">
         <is>
-          <t>OUR-65</t>
+          <t>OUR-64</t>
         </is>
       </c>
       <c r="B443" s="7" t="inlineStr">
@@ -18422,24 +18422,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C443" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C443" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D443" s="9" t="inlineStr">
         <is>
-          <t>Scan is absent when AI is off</t>
+          <t>The photo never reaches the shared list</t>
         </is>
       </c>
       <c r="E443" s="9" t="inlineStr">
         <is>
-          <t>Turn AI off in Settings, then open the Ours capture.</t>
+          <t>Scan something into Ours and Add it. Check the other device.</t>
         </is>
       </c>
       <c r="F443" s="9" t="inlineStr">
         <is>
-          <t>No Scan button, on either screen. Speak stays: it is on-device dictation, not a server call.</t>
+          <t>Your person sees the rows you added and nothing else, exactly as if you had typed them. No image is stored anywhere, shared or otherwise: it is sent to be read, then discarded.</t>
         </is>
       </c>
       <c r="G443" s="7" t="inlineStr">
@@ -18454,7 +18454,7 @@
     <row r="444">
       <c r="A444" s="6" t="inlineStr">
         <is>
-          <t>OUR-66</t>
+          <t>OUR-65</t>
         </is>
       </c>
       <c r="B444" s="7" t="inlineStr">
@@ -18462,24 +18462,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C444" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C444" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D444" s="9" t="inlineStr">
         <is>
-          <t>A repeating shared row appears on BOTH Todays on its day</t>
+          <t>Scan is absent when AI is off</t>
         </is>
       </c>
       <c r="E444" s="9" t="inlineStr">
         <is>
-          <t>Make a shared task repeat weekly on today's weekday. Open Today on both devices.</t>
+          <t>Turn AI off in Settings, then open the Ours capture.</t>
         </is>
       </c>
       <c r="F444" s="9" t="inlineStr">
         <is>
-          <t>It appears on each Today under a 'From Ours' heading, below the day's own tasks. Neither person had to fetch it. This is the answer to 'I do not want to manually decide what gets added to my list for today'.</t>
+          <t>No Scan button, on either screen. Speak stays: it is on-device dictation, not a server call.</t>
         </is>
       </c>
       <c r="G444" s="7" t="inlineStr">
@@ -18494,7 +18494,7 @@
     <row r="445">
       <c r="A445" s="6" t="inlineStr">
         <is>
-          <t>OUR-67</t>
+          <t>OUR-66</t>
         </is>
       </c>
       <c r="B445" s="7" t="inlineStr">
@@ -18509,17 +18509,17 @@
       </c>
       <c r="D445" s="9" t="inlineStr">
         <is>
-          <t>An UNDATED shared row never reaches Today</t>
+          <t>A repeating shared row appears on BOTH Todays on its day</t>
         </is>
       </c>
       <c r="E445" s="9" t="inlineStr">
         <is>
-          <t>Add an ordinary shared task with the door left on Anytime. Check Today on both devices.</t>
+          <t>Make a shared task repeat weekly on today's weekday. Open Today on both devices.</t>
         </is>
       </c>
       <c r="F445" s="9" t="inlineStr">
         <is>
-          <t>It is in the room and NOWHERE on Today. This is the load-bearing rule: without it, your person adding eight things to the shopping list makes your morning eight heavier without you agreeing to any of it.</t>
+          <t>It appears on each Today under a 'From Ours' heading, below the day's own tasks. Neither person had to fetch it. This is the answer to 'I do not want to manually decide what gets added to my list for today'.</t>
         </is>
       </c>
       <c r="G445" s="7" t="inlineStr">
@@ -18534,7 +18534,7 @@
     <row r="446">
       <c r="A446" s="6" t="inlineStr">
         <is>
-          <t>OUR-68</t>
+          <t>OUR-67</t>
         </is>
       </c>
       <c r="B446" s="7" t="inlineStr">
@@ -18549,17 +18549,17 @@
       </c>
       <c r="D446" s="9" t="inlineStr">
         <is>
-          <t>Shared rows never make the day look heavier</t>
+          <t>An UNDATED shared row never reaches Today</t>
         </is>
       </c>
       <c r="E446" s="9" t="inlineStr">
         <is>
-          <t>With several shared rows showing on Today, check the weight gauge, Plan my day, Lighten, and the close-the-day count.</t>
+          <t>Add an ordinary shared task with the door left on Anytime. Check Today on both devices.</t>
         </is>
       </c>
       <c r="F446" s="9" t="inlineStr">
         <is>
-          <t>All of them ignore the shared rows entirely. They are not in `tasks`, so they cannot reach any of it by construction. The day the app promises is finite stays finite.</t>
+          <t>It is in the room and NOWHERE on Today. This is the load-bearing rule: without it, your person adding eight things to the shopping list makes your morning eight heavier without you agreeing to any of it.</t>
         </is>
       </c>
       <c r="G446" s="7" t="inlineStr">
@@ -18574,7 +18574,7 @@
     <row r="447">
       <c r="A447" s="6" t="inlineStr">
         <is>
-          <t>OUR-69</t>
+          <t>OUR-68</t>
         </is>
       </c>
       <c r="B447" s="7" t="inlineStr">
@@ -18589,17 +18589,17 @@
       </c>
       <c r="D447" s="9" t="inlineStr">
         <is>
-          <t>Ticking a shared row from Today closes it for both</t>
+          <t>Shared rows never make the day look heavier</t>
         </is>
       </c>
       <c r="E447" s="9" t="inlineStr">
         <is>
-          <t>Tick a row in the From Ours strip on device A. Look at device B's Ours list and Today.</t>
+          <t>With several shared rows showing on Today, check the weight gauge, Plan my day, Lighten, and the close-the-day count.</t>
         </is>
       </c>
       <c r="F447" s="9" t="inlineStr">
         <is>
-          <t>Done on both, within a poll. Nothing anywhere says who did it, and neither room tints it as a stranger's change on the device that did it (noteOursMine).</t>
+          <t>All of them ignore the shared rows entirely. They are not in `tasks`, so they cannot reach any of it by construction. The day the app promises is finite stays finite.</t>
         </is>
       </c>
       <c r="G447" s="7" t="inlineStr">
@@ -18614,7 +18614,7 @@
     <row r="448">
       <c r="A448" s="6" t="inlineStr">
         <is>
-          <t>OUR-70</t>
+          <t>OUR-69</t>
         </is>
       </c>
       <c r="B448" s="7" t="inlineStr">
@@ -18622,24 +18622,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C448" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C448" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D448" s="9" t="inlineStr">
         <is>
-          <t>A dated shared row shows from its day onward, never before</t>
+          <t>Ticking a shared row from Today closes it for both</t>
         </is>
       </c>
       <c r="E448" s="9" t="inlineStr">
         <is>
-          <t>Add a shared task with the door set to a date two days out. Check Today now, then on the day.</t>
+          <t>Tick a row in the From Ours strip on device A. Look at device B's Ours list and Today.</t>
         </is>
       </c>
       <c r="F448" s="9" t="inlineStr">
         <is>
-          <t>Absent today, present on the day and on any day after (a shared thing nobody did does not stop being one). The room shows its date on the row all along, so it is never a surprise.</t>
+          <t>Done on both, within a poll. Nothing anywhere says who did it, and neither room tints it as a stranger's change on the device that did it (noteOursMine).</t>
         </is>
       </c>
       <c r="G448" s="7" t="inlineStr">
@@ -18654,7 +18654,7 @@
     <row r="449">
       <c r="A449" s="6" t="inlineStr">
         <is>
-          <t>OUR-71</t>
+          <t>OUR-70</t>
         </is>
       </c>
       <c r="B449" s="7" t="inlineStr">
@@ -18662,24 +18662,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C449" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C449" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D449" s="9" t="inlineStr">
         <is>
-          <t>The shared capture rests on Anytime, and says what a day means</t>
+          <t>A dated shared row shows from its day onward, never before</t>
         </is>
       </c>
       <c r="E449" s="9" t="inlineStr">
         <is>
-          <t>Tap the + pill on Ours and read the line beside the When chip. Open the door. Pick Today, then Tomorrow, then Daily, reading that line each time.</t>
+          <t>Add a shared task with the door set to a date two days out. Check Today now, then on the day.</t>
         </is>
       </c>
       <c r="F449" s="9" t="inlineStr">
         <is>
-          <t>The When row reads Anytime / Today / Tomorrow / Pick a date, with Anytime selected, and the Add button says just 'Add'. Choosing Today makes it read 'Add · Today', because that is the notable case: it will appear on both your days. The line beside the chip says, in plain words, what the current choice means on a shared list (no day lives here; a day reaches both Todays; a rhythm repeats for both of you), before you add.</t>
+          <t>Absent today, present on the day and on any day after (a shared thing nobody did does not stop being one). The room shows its date on the row all along, so it is never a surprise.</t>
         </is>
       </c>
       <c r="G449" s="7" t="inlineStr">
@@ -18694,7 +18694,7 @@
     <row r="450">
       <c r="A450" s="6" t="inlineStr">
         <is>
-          <t>OUR-112</t>
+          <t>OUR-71</t>
         </is>
       </c>
       <c r="B450" s="7" t="inlineStr">
@@ -18709,17 +18709,17 @@
       </c>
       <c r="D450" s="9" t="inlineStr">
         <is>
-          <t>A shared row's WHEN can be changed, and cleared</t>
+          <t>The shared capture rests on Anytime, and says what a day means</t>
         </is>
       </c>
       <c r="E450" s="9" t="inlineStr">
         <is>
-          <t>In the room, hold a row. The door reads 'When…' with the row's current answer beside it. Open it. Set a date, Set. Reopen, pick a different date, Set. Reopen, tap Anytime, Set.</t>
+          <t>Tap the + pill on Ours and read the line beside the When chip. Open the door. Pick Today, then Tomorrow, then Daily, reading that line each time.</t>
         </is>
       </c>
       <c r="F450" s="9" t="inlineStr">
         <is>
-          <t>All three land: date set, date CHANGED, and back to plain. Changing a date and getting back to a plain row were both impossible before this; remove-and-recreate was the only way out, and on a repeat that ends the series for both people. The button always names the outcome ('Set . Thu 20 Aug', 'Set . Anytime'), never 'Save'.</t>
+          <t>The When row reads Anytime / Today / Tomorrow / Pick a date, with Anytime selected, and the Add button says just 'Add'. Choosing Today makes it read 'Add · Today', because that is the notable case: it will appear on both your days. The line beside the chip says, in plain words, what the current choice means on a shared list (no day lives here; a day reaches both Todays; a rhythm repeats for both of you), before you add.</t>
         </is>
       </c>
       <c r="G450" s="7" t="inlineStr">
@@ -18734,7 +18734,7 @@
     <row r="451">
       <c r="A451" s="6" t="inlineStr">
         <is>
-          <t>OUR-113</t>
+          <t>OUR-112</t>
         </is>
       </c>
       <c r="B451" s="7" t="inlineStr">
@@ -18749,17 +18749,17 @@
       </c>
       <c r="D451" s="9" t="inlineStr">
         <is>
-          <t>Ending a rhythm does NOT mark the row done for both people</t>
+          <t>A shared row's WHEN can be changed, and cleared</t>
         </is>
       </c>
       <c r="E451" s="9" t="inlineStr">
         <is>
-          <t>Make a shared row repeat weekly and tick it on one of its days, on either device. Then hold it, open When…, tap the selected rhythm chip to release it, choose Anytime, and Set. Watch BOTH devices.</t>
+          <t>In the room, hold a row. The door reads 'When…' with the row's current answer beside it. Open it. Set a date, Set. Reopen, pick a different date, Set. Reopen, tap Anytime, Set.</t>
         </is>
       </c>
       <c r="F451" s="9" t="inlineStr">
         <is>
-          <t>The row goes plain and stays UN-ticked on both. It must not come back done. A repeat's ticks live per-date in a completion log and the row's own done flag stays false; the moment the recurrence goes, the merge would read that same log as a one-off's tick and mark the row finished, for both people, with a doneAt from whenever it was last ticked. Try it for a DATED ending too (release the rhythm, pick a day): that path feels least like an ending and is the easiest to get wrong.</t>
+          <t>All three land: date set, date CHANGED, and back to plain. Changing a date and getting back to a plain row were both impossible before this; remove-and-recreate was the only way out, and on a repeat that ends the series for both people. The button always names the outcome ('Set . Thu 20 Aug', 'Set . Anytime'), never 'Save'.</t>
         </is>
       </c>
       <c r="G451" s="7" t="inlineStr">
@@ -18774,7 +18774,7 @@
     <row r="452">
       <c r="A452" s="6" t="inlineStr">
         <is>
-          <t>OUR-114</t>
+          <t>OUR-113</t>
         </is>
       </c>
       <c r="B452" s="7" t="inlineStr">
@@ -18782,24 +18782,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C452" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C452" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D452" s="9" t="inlineStr">
         <is>
-          <t>The day zone changes its question when a rhythm is alive</t>
+          <t>Ending a rhythm does NOT mark the row done for both people</t>
         </is>
       </c>
       <c r="E452" s="9" t="inlineStr">
         <is>
-          <t>In the room, hold a row and open When…. With no rhythm selected, read the label above the day chips. Now tap Daily. Read it again. Then tap Anytime.</t>
+          <t>Make a shared row repeat weekly and tick it on one of its days, on either device. Then hold it, open When…, tap the selected rhythm chip to release it, choose Anytime, and Set. Watch BOTH devices.</t>
         </is>
       </c>
       <c r="F452" s="9" t="inlineStr">
         <is>
-          <t>It reads 'A day' with no rhythm, and relabels to 'Starting' the moment one is selected, in the accent colour. The same chips now mean 'from when' rather than 'which day'. Anytime stays available throughout, and ONE tap on it ends the rhythm: the label goes back to 'A day' and the summary says 'The rhythm ends.' before anything commits. Tapping the selected rhythm chip releases it too, for anyone who finds that natural, and both routes land in exactly the same place.</t>
+          <t>The row goes plain and stays UN-ticked on both. It must not come back done. A repeat's ticks live per-date in a completion log and the row's own done flag stays false; the moment the recurrence goes, the merge would read that same log as a one-off's tick and mark the row finished, for both people, with a doneAt from whenever it was last ticked. Try it for a DATED ending too (release the rhythm, pick a day): that path feels least like an ending and is the easiest to get wrong.</t>
         </is>
       </c>
       <c r="G452" s="7" t="inlineStr">
@@ -18814,7 +18814,7 @@
     <row r="453">
       <c r="A453" s="6" t="inlineStr">
         <is>
-          <t>OUR-115</t>
+          <t>OUR-114</t>
         </is>
       </c>
       <c r="B453" s="7" t="inlineStr">
@@ -18829,17 +18829,17 @@
       </c>
       <c r="D453" s="9" t="inlineStr">
         <is>
-          <t>Setting a shared row to Today actually reaches both Todays</t>
+          <t>The day zone changes its question when a rhythm is alive</t>
         </is>
       </c>
       <c r="E453" s="9" t="inlineStr">
         <is>
-          <t>In the room, hold a plain row, open When…, tap Today, and Set. Check BOTH Todays (look away and back on each).</t>
+          <t>In the room, hold a row and open When…. With no rhythm selected, read the label above the day chips. Now tap Daily. Read it again. Then tap Anytime.</t>
         </is>
       </c>
       <c r="F453" s="9" t="inlineStr">
         <is>
-          <t>It appears under DUE TODAY on both. The line in the sheet reads 'Today . &lt;the date&gt;' on purpose: a shared row with no date reaches nobody, so Today has to write a real date rather than 'no date', which is the same bug that once shipped on the shared capture bar above this sheet.</t>
+          <t>It reads 'A day' with no rhythm, and relabels to 'Starting' the moment one is selected, in the accent colour. The same chips now mean 'from when' rather than 'which day'. Anytime stays available throughout, and ONE tap on it ends the rhythm: the label goes back to 'A day' and the summary says 'The rhythm ends.' before anything commits. Tapping the selected rhythm chip releases it too, for anyone who finds that natural, and both routes land in exactly the same place.</t>
         </is>
       </c>
       <c r="G453" s="7" t="inlineStr">
@@ -18854,7 +18854,7 @@
     <row r="454">
       <c r="A454" s="6" t="inlineStr">
         <is>
-          <t>OUR-116</t>
+          <t>OUR-115</t>
         </is>
       </c>
       <c r="B454" s="7" t="inlineStr">
@@ -18862,24 +18862,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C454" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C454" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D454" s="9" t="inlineStr">
         <is>
-          <t>An idle Set does not wash the row on the other device</t>
+          <t>Setting a shared row to Today actually reaches both Todays</t>
         </is>
       </c>
       <c r="E454" s="9" t="inlineStr">
         <is>
-          <t>On A, hold a row, open When…, change nothing, and tap Set. On B, leave the room and come back.</t>
+          <t>In the room, hold a plain row, open When…, tap Today, and Set. Check BOTH Todays (look away and back on each).</t>
         </is>
       </c>
       <c r="F454" s="9" t="inlineStr">
         <is>
-          <t>No 'changed since you looked' mark on B. Every write stamps the row, and a fresh stamp is exactly what the other person's screen reads as a change, so a Set that altered nothing would send them hunting for something nobody did.</t>
+          <t>It appears under DUE TODAY on both. The line in the sheet reads 'Today . &lt;the date&gt;' on purpose: a shared row with no date reaches nobody, so Today has to write a real date rather than 'no date', which is the same bug that once shipped on the shared capture bar above this sheet.</t>
         </is>
       </c>
       <c r="G454" s="7" t="inlineStr">
@@ -18894,7 +18894,7 @@
     <row r="455">
       <c r="A455" s="6" t="inlineStr">
         <is>
-          <t>OUR-118</t>
+          <t>OUR-116</t>
         </is>
       </c>
       <c r="B455" s="7" t="inlineStr">
@@ -18902,24 +18902,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C455" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C455" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D455" s="9" t="inlineStr">
         <is>
-          <t>A repeat you have already done today keeps its held card</t>
+          <t>An idle Set does not wash the row on the other device</t>
         </is>
       </c>
       <c r="E455" s="9" t="inlineStr">
         <is>
-          <t>In the room, make a row repeat on TODAY's weekday, then tick it. Now hold it.</t>
+          <t>On A, hold a row, open When…, change nothing, and tap Set. On B, leave the room and come back.</t>
         </is>
       </c>
       <c r="F455" s="9" t="inlineStr">
         <is>
-          <t>The card still offers When… with its rhythm beside it, and it does NOT say 'Done is done.' A repeat is not a finished thing: it comes back, so the day you did it is exactly a day you might want to move it. Before this, ticking a repeat took its whole held card away until the next day, which put the When editor out of reach on the rows most likely to need it. A finished ONE-OFF still gets the minimal card, which is correct.</t>
+          <t>No 'changed since you looked' mark on B. Every write stamps the row, and a fresh stamp is exactly what the other person's screen reads as a change, so a Set that altered nothing would send them hunting for something nobody did.</t>
         </is>
       </c>
       <c r="G455" s="7" t="inlineStr">
@@ -18934,7 +18934,7 @@
     <row r="456">
       <c r="A456" s="6" t="inlineStr">
         <is>
-          <t>OUR-117</t>
+          <t>OUR-118</t>
         </is>
       </c>
       <c r="B456" s="7" t="inlineStr">
@@ -18942,24 +18942,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C456" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C456" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D456" s="9" t="inlineStr">
         <is>
-          <t>The Repeating room's Edit sheet is untouched by the When editor</t>
+          <t>A repeat you have already done today keeps its held card</t>
         </is>
       </c>
       <c r="E456" s="9" t="inlineStr">
         <is>
-          <t>Menu -&gt; Repeating -&gt; Edit on any series. Compare with before.</t>
+          <t>In the room, make a row repeat on TODAY's weekday, then tick it. Now hold it.</t>
         </is>
       </c>
       <c r="F456" s="9" t="inlineStr">
         <is>
-          <t>Same sheet as always: title, the four cadence chips (Daily / Weekly / Every few days / Monthly), weekday toggles or the stepper or the 1-31 grid, 'Starting from' with its date, and a commit button naming the cadence. NO Anytime chip, NO day zone, and tapping the selected cadence chip does NOT release it. 'No rhythm' there would mean the entry should not exist, which is removal, and removal stays in the Repeating room.</t>
+          <t>The card still offers When… with its rhythm beside it, and it does NOT say 'Done is done.' A repeat is not a finished thing: it comes back, so the day you did it is exactly a day you might want to move it. Before this, ticking a repeat took its whole held card away until the next day, which put the When editor out of reach on the rows most likely to need it. A finished ONE-OFF still gets the minimal card, which is correct.</t>
         </is>
       </c>
       <c r="G456" s="7" t="inlineStr">
@@ -18974,7 +18974,7 @@
     <row r="457">
       <c r="A457" s="6" t="inlineStr">
         <is>
-          <t>OUR-119</t>
+          <t>OUR-117</t>
         </is>
       </c>
       <c r="B457" s="7" t="inlineStr">
@@ -18989,17 +18989,17 @@
       </c>
       <c r="D457" s="9" t="inlineStr">
         <is>
-          <t>Monthly works on a shared row, and an out-of-date partner still sees the rhythm</t>
+          <t>The Repeating room's Edit sheet is untouched by the When editor</t>
         </is>
       </c>
       <c r="E457" s="9" t="inlineStr">
         <is>
-          <t>On Ours, hold a row and tap 'Repeat…'. Choose Monthly and a day. Read the summary, commit, then look at the row and at both Todays on that day. If a partner is on an older build (1.3.1 or earlier), have them look at the same row.</t>
+          <t>Menu -&gt; Repeating -&gt; Edit on any series. Compare with before.</t>
         </is>
       </c>
       <c r="F457" s="9" t="inlineStr">
         <is>
-          <t>Monthly is the fourth rhythm chip here too, from the same sheet the Repeating room uses, so a shared monthly row and a personal one are identical in shape. The summary reads 'Every month on the 15th · from {start}' and the commit button names it. The row lands on BOTH Todays on that day. A partner whose build predates monthly cannot compute the days, so their app shows the row with the plain-English line the writing client left alongside the rhythm rather than showing a repeating row with no rhythm at all. What it must never do is HIDE the row: one person seeing a task the other does not is the invisible disagreement this whole feature exists to prevent.</t>
+          <t>Same sheet as always: title, the four cadence chips (Daily / Weekly / Every few days / Monthly), weekday toggles or the stepper or the 1-31 grid, 'Starting from' with its date, and a commit button naming the cadence. NO Anytime chip, NO day zone, and tapping the selected cadence chip does NOT release it. 'No rhythm' there would mean the entry should not exist, which is removal, and removal stays in the Repeating room.</t>
         </is>
       </c>
       <c r="G457" s="7" t="inlineStr">
@@ -19014,7 +19014,7 @@
     <row r="458">
       <c r="A458" s="6" t="inlineStr">
         <is>
-          <t>OUR-111</t>
+          <t>OUR-119</t>
         </is>
       </c>
       <c r="B458" s="7" t="inlineStr">
@@ -19022,24 +19022,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C458" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C458" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D458" s="9" t="inlineStr">
         <is>
-          <t>A finished dated shared row leaves both Todays the next day</t>
+          <t>Monthly works on a shared row, and an out-of-date partner still sees the rhythm</t>
         </is>
       </c>
       <c r="E458" s="9" t="inlineStr">
         <is>
-          <t>Give a shared row today's date so it appears under DUE TODAY on both phones. Tick it on either phone. Look at both Todays now, then again tomorrow (or move a device's clock forward a day and reopen).</t>
+          <t>On Ours, hold a row and tap 'Repeat…'. Choose Monthly and a day. Read the summary, commit, then look at the row and at both Todays on that day. If a partner is on an older build (1.3.1 or earlier), have them look at the same row.</t>
         </is>
       </c>
       <c r="F458" s="9" t="inlineStr">
         <is>
-          <t>Today: still there on BOTH, ticked, and un-tickable again, because ticking is the reversible act on this list. Tomorrow: gone from both. It must not accumulate. Before this rule the strip kept every dated row either of you had ever ticked, for good, on a screen excluded from the weight gauge and the close-the-day count, whose whole premise is that a day is finite. Check the other half too: an UNFINISHED row with a past date is still there tomorrow, which is correct and is not shaming.</t>
+          <t>Monthly is the fourth rhythm chip here too, from the same sheet the Repeating room uses, so a shared monthly row and a personal one are identical in shape. The summary reads 'Every month on the 15th · from {start}' and the commit button names it. The row lands on BOTH Todays on that day. A partner whose build predates monthly cannot compute the days, so their app shows the row with the plain-English line the writing client left alongside the rhythm rather than showing a repeating row with no rhythm at all. What it must never do is HIDE the row: one person seeing a task the other does not is the invisible disagreement this whole feature exists to prevent.</t>
         </is>
       </c>
       <c r="G458" s="7" t="inlineStr">
@@ -19054,7 +19054,7 @@
     <row r="459">
       <c r="A459" s="6" t="inlineStr">
         <is>
-          <t>OUR-72</t>
+          <t>OUR-111</t>
         </is>
       </c>
       <c r="B459" s="7" t="inlineStr">
@@ -19062,24 +19062,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C459" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C459" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D459" s="9" t="inlineStr">
         <is>
-          <t>A repeat supersedes the day rather than joining it</t>
+          <t>A finished dated shared row leaves both Todays the next day</t>
         </is>
       </c>
       <c r="E459" s="9" t="inlineStr">
         <is>
-          <t>On the Ours capture, set a Daily repeat with When left on Anytime.</t>
+          <t>Give a shared row today's date so it appears under DUE TODAY on both phones. Tick it on either phone. Look at both Todays now, then again tomorrow (or move a device's clock forward a day and reopen).</t>
         </is>
       </c>
       <c r="F459" s="9" t="inlineStr">
         <is>
-          <t>The door summary reads 'Daily', not 'Anytime . Daily'. On Today's own capture it still reads 'Today . Daily', where the when genuinely IS the repeat's start.</t>
+          <t>Today: still there on BOTH, ticked, and un-tickable again, because ticking is the reversible act on this list. Tomorrow: gone from both. It must not accumulate. Before this rule the strip kept every dated row either of you had ever ticked, for good, on a screen excluded from the weight gauge and the close-the-day count, whose whole premise is that a day is finite. Check the other half too: an UNFINISHED row with a past date is still there tomorrow, which is correct and is not shaming.</t>
         </is>
       </c>
       <c r="G459" s="7" t="inlineStr">
@@ -19094,7 +19094,7 @@
     <row r="460">
       <c r="A460" s="6" t="inlineStr">
         <is>
-          <t>OUR-73</t>
+          <t>OUR-72</t>
         </is>
       </c>
       <c r="B460" s="7" t="inlineStr">
@@ -19102,24 +19102,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C460" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C460" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D460" s="9" t="inlineStr">
         <is>
-          <t>An unreadable cadence is never placed on a day</t>
+          <t>A repeat supersedes the day rather than joining it</t>
         </is>
       </c>
       <c r="E460" s="9" t="inlineStr">
         <is>
-          <t>Have a newer build write a cadence this build cannot parse, then open Today.</t>
+          <t>On the Ours capture, set a Daily repeat with When left on Anytime.</t>
         </is>
       </c>
       <c r="F460" s="9" t="inlineStr">
         <is>
-          <t>It shows in the room (never invisible to the person who set it) and appears on NO Today. This build cannot know which days it means, and a wrong day on a shared surface is a thing the other person has to puzzle over.</t>
+          <t>The door summary reads 'Daily', not 'Anytime . Daily'. On Today's own capture it still reads 'Today . Daily', where the when genuinely IS the repeat's start.</t>
         </is>
       </c>
       <c r="G460" s="7" t="inlineStr">
@@ -19134,7 +19134,7 @@
     <row r="461">
       <c r="A461" s="6" t="inlineStr">
         <is>
-          <t>OUR-74</t>
+          <t>OUR-73</t>
         </is>
       </c>
       <c r="B461" s="7" t="inlineStr">
@@ -19142,24 +19142,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C461" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C461" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D461" s="9" t="inlineStr">
         <is>
-          <t>The heading's '!' says something changed since you looked, and clears when you look</t>
+          <t>An unreadable cadence is never placed on a day</t>
         </is>
       </c>
       <c r="E461" s="9" t="inlineStr">
         <is>
-          <t>Device B changes something on the shared list. On device A, open Today WITHOUT visiting Ours. Then tap the list's name in the heading and come back. Also have device B delete a row and check again.</t>
+          <t>Have a newer build write a cadence this build cannot parse, then open Today.</t>
         </is>
       </c>
       <c r="F461" s="9" t="inlineStr">
         <is>
-          <t>A small tinted '!' sits beside the list's name in Today's heading, and a screen reader hears '{name}. 1 since you looked'. After visiting, it is gone. A deleted row never raises it. The mark is bounded by your own attention, not by the list's length, and it never shows a climbing number.</t>
+          <t>It shows in the room (never invisible to the person who set it) and appears on NO Today. This build cannot know which days it means, and a wrong day on a shared surface is a thing the other person has to puzzle over.</t>
         </is>
       </c>
       <c r="G461" s="7" t="inlineStr">
@@ -19174,7 +19174,7 @@
     <row r="462">
       <c r="A462" s="6" t="inlineStr">
         <is>
-          <t>OUR-75</t>
+          <t>OUR-74</t>
         </is>
       </c>
       <c r="B462" s="7" t="inlineStr">
@@ -19182,24 +19182,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C462" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C462" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D462" s="9" t="inlineStr">
         <is>
-          <t>Your OWN changes never raise the '!'</t>
+          <t>The heading's '!' says something changed since you looked, and clears when you look</t>
         </is>
       </c>
       <c r="E462" s="9" t="inlineStr">
         <is>
-          <t>On device A, add or tick several shared rows. Go to Today on the SAME device.</t>
+          <t>Device B changes something on the shared list. On device A, open Today WITHOUT visiting Ours. Then tap the list's name in the heading and come back. Also have device B delete a row and check again.</t>
         </is>
       </c>
       <c r="F462" s="9" t="inlineStr">
         <is>
-          <t>No '!' in the heading. It uses the room's own wash arithmetic, so the heading and the room always agree about whose change it was.</t>
+          <t>A small tinted '!' sits beside the list's name in Today's heading, and a screen reader hears '{name}. 1 since you looked'. After visiting, it is gone. A deleted row never raises it. The mark is bounded by your own attention, not by the list's length, and it never shows a climbing number.</t>
         </is>
       </c>
       <c r="G462" s="7" t="inlineStr">
@@ -19214,7 +19214,7 @@
     <row r="463">
       <c r="A463" s="6" t="inlineStr">
         <is>
-          <t>OUR-76</t>
+          <t>OUR-75</t>
         </is>
       </c>
       <c r="B463" s="7" t="inlineStr">
@@ -19229,17 +19229,17 @@
       </c>
       <c r="D463" s="9" t="inlineStr">
         <is>
-          <t>A first-ever visit raises nothing</t>
+          <t>Your OWN changes never raise the '!'</t>
         </is>
       </c>
       <c r="E463" s="9" t="inlineStr">
         <is>
-          <t>Pair two accounts, put rows on the list from device B, and open Today on a device A that has never opened the room.</t>
+          <t>On device A, add or tick several shared rows. Go to Today on the SAME device.</t>
         </is>
       </c>
       <c r="F463" s="9" t="inlineStr">
         <is>
-          <t>No '!'. There is no 'last looked' to measure against, and inventing one would open the app with a mark already on it.</t>
+          <t>No '!' in the heading. It uses the room's own wash arithmetic, so the heading and the room always agree about whose change it was.</t>
         </is>
       </c>
       <c r="G463" s="7" t="inlineStr">
@@ -19254,7 +19254,7 @@
     <row r="464">
       <c r="A464" s="6" t="inlineStr">
         <is>
-          <t>OUR-77</t>
+          <t>OUR-76</t>
         </is>
       </c>
       <c r="B464" s="7" t="inlineStr">
@@ -19262,24 +19262,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C464" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C464" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D464" s="9" t="inlineStr">
         <is>
-          <t>The capture's AI note names only what that surface HAS</t>
+          <t>A first-ever visit raises nothing</t>
         </is>
       </c>
       <c r="E464" s="9" t="inlineStr">
         <is>
-          <t>Type into the Ours capture, then into Today's, and read the line under the buttons.</t>
+          <t>Pair two accounts, put rows on the list from device B, and open Today on a device A that has never opened the room.</t>
         </is>
       </c>
       <c r="F464" s="9" t="inlineStr">
         <is>
-          <t>Ours says Scan sends your photo. Today says Sort for me, Break it down and Scan send what you type or photograph. Ours must NEVER name Sort for me or Break it down: neither button is there, and a false claim about where your data goes teaches people the disclosure is decorative.</t>
+          <t>No '!'. There is no 'last looked' to measure against, and inventing one would open the app with a mark already on it.</t>
         </is>
       </c>
       <c r="G464" s="7" t="inlineStr">
@@ -19294,7 +19294,7 @@
     <row r="465">
       <c r="A465" s="6" t="inlineStr">
         <is>
-          <t>OUR-78</t>
+          <t>OUR-77</t>
         </is>
       </c>
       <c r="B465" s="7" t="inlineStr">
@@ -19309,17 +19309,17 @@
       </c>
       <c r="D465" s="9" t="inlineStr">
         <is>
-          <t>Scan discloses on every path that can reach a camera</t>
+          <t>The capture's AI note names only what that surface HAS</t>
         </is>
       </c>
       <c r="E465" s="9" t="inlineStr">
         <is>
-          <t>Open Scan on web (gallery picker) and on Android with the camera already allowed.</t>
+          <t>Type into the Ours capture, then into Today's, and read the line under the buttons.</t>
         </is>
       </c>
       <c r="F465" s="9" t="inlineStr">
         <is>
-          <t>Both show the egress line. It used to appear only on the Android permission screen, so the two paths a person can reach WITHOUT a prompt sent a photograph having said nothing.</t>
+          <t>Ours says Scan sends your photo. Today says Sort for me, Break it down and Scan send what you type or photograph. Ours must NEVER name Sort for me or Break it down: neither button is there, and a false claim about where your data goes teaches people the disclosure is decorative.</t>
         </is>
       </c>
       <c r="G465" s="7" t="inlineStr">
@@ -19334,7 +19334,7 @@
     <row r="466">
       <c r="A466" s="6" t="inlineStr">
         <is>
-          <t>OUR-79</t>
+          <t>OUR-78</t>
         </is>
       </c>
       <c r="B466" s="7" t="inlineStr">
@@ -19349,17 +19349,17 @@
       </c>
       <c r="D466" s="9" t="inlineStr">
         <is>
-          <t>Press and hold a From Ours row on Today</t>
+          <t>Scan discloses on every path that can reach a camera</t>
         </is>
       </c>
       <c r="E466" s="9" t="inlineStr">
         <is>
-          <t>Hold a row in the From Ours strip.</t>
+          <t>Open Scan on web (gallery picker) and on Android with the camera already allowed.</t>
         </is>
       </c>
       <c r="F466" s="9" t="inlineStr">
         <is>
-          <t>The held card opens with Pin and, on a non-repeating row, Move to. Choosing either TAKES THE ROW ON as your own copy: it leaves the strip and joins your day, where the ordinary reorder and the rest of the held card already work.</t>
+          <t>Both show the egress line. It used to appear only on the Android permission screen, so the two paths a person can reach WITHOUT a prompt sent a photograph having said nothing.</t>
         </is>
       </c>
       <c r="G466" s="7" t="inlineStr">
@@ -19374,7 +19374,7 @@
     <row r="467">
       <c r="A467" s="6" t="inlineStr">
         <is>
-          <t>OUR-80</t>
+          <t>OUR-79</t>
         </is>
       </c>
       <c r="B467" s="7" t="inlineStr">
@@ -19389,17 +19389,17 @@
       </c>
       <c r="D467" s="9" t="inlineStr">
         <is>
-          <t>Pin and Move-to never rearrange the other person's day</t>
+          <t>Press and hold a From Ours row on Today</t>
         </is>
       </c>
       <c r="E467" s="9" t="inlineStr">
         <is>
-          <t>Move a shared row to tomorrow from your Today. Check the other device.</t>
+          <t>Hold a row in the From Ours strip.</t>
         </is>
       </c>
       <c r="F467" s="9" t="inlineStr">
         <is>
-          <t>YOUR copy moves to tomorrow. The shared row is untouched and still on her day. Applied to the shared row itself this would silently take it off her Wednesday too, on a thing she may have planned around.</t>
+          <t>The held card opens with Pin and, on a non-repeating row, Move to. Choosing either TAKES THE ROW ON as your own copy: it leaves the strip and joins your day, where the ordinary reorder and the rest of the held card already work.</t>
         </is>
       </c>
       <c r="G467" s="7" t="inlineStr">
@@ -19414,7 +19414,7 @@
     <row r="468">
       <c r="A468" s="6" t="inlineStr">
         <is>
-          <t>OUR-81</t>
+          <t>OUR-80</t>
         </is>
       </c>
       <c r="B468" s="7" t="inlineStr">
@@ -19422,24 +19422,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C468" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C468" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D468" s="9" t="inlineStr">
         <is>
-          <t>A taken-on row is never on screen twice</t>
+          <t>Pin and Move-to never rearrange the other person's day</t>
         </is>
       </c>
       <c r="E468" s="9" t="inlineStr">
         <is>
-          <t>Take a shared row on (Pin it, or Bring it from the room). Look at Today.</t>
+          <t>Move a shared row to tomorrow from your Today. Check the other device.</t>
         </is>
       </c>
       <c r="F468" s="9" t="inlineStr">
         <is>
-          <t>It appears once, as your task, and NOT also in the From Ours strip. Still true once it is ticked: a finished copy and its finished origin must not both render.</t>
+          <t>YOUR copy moves to tomorrow. The shared row is untouched and still on her day. Applied to the shared row itself this would silently take it off her Wednesday too, on a thing she may have planned around.</t>
         </is>
       </c>
       <c r="G468" s="7" t="inlineStr">
@@ -19454,7 +19454,7 @@
     <row r="469">
       <c r="A469" s="6" t="inlineStr">
         <is>
-          <t>OUR-82</t>
+          <t>OUR-81</t>
         </is>
       </c>
       <c r="B469" s="7" t="inlineStr">
@@ -19469,17 +19469,17 @@
       </c>
       <c r="D469" s="9" t="inlineStr">
         <is>
-          <t>Move-to is not offered on a repeating shared row</t>
+          <t>A taken-on row is never on screen twice</t>
         </is>
       </c>
       <c r="E469" s="9" t="inlineStr">
         <is>
-          <t>Hold a repeating row in the From Ours strip.</t>
+          <t>Take a shared row on (Pin it, or Bring it from the room). Look at Today.</t>
         </is>
       </c>
       <c r="F469" s="9" t="inlineStr">
         <is>
-          <t>Pin is there, Move to is not. A date and a rhythm are alternatives, and rescheduling a series is a question for the room's cadence sheet, not a one-tap action on a day.</t>
+          <t>It appears once, as your task, and NOT also in the From Ours strip. Still true once it is ticked: a finished copy and its finished origin must not both render.</t>
         </is>
       </c>
       <c r="G469" s="7" t="inlineStr">
@@ -19494,7 +19494,7 @@
     <row r="470">
       <c r="A470" s="6" t="inlineStr">
         <is>
-          <t>OUR-83</t>
+          <t>OUR-82</t>
         </is>
       </c>
       <c r="B470" s="7" t="inlineStr">
@@ -19502,24 +19502,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C470" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C470" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D470" s="9" t="inlineStr">
         <is>
-          <t>One shared row, one route onto your day</t>
+          <t>Move-to is not offered on a repeating shared row</t>
         </is>
       </c>
       <c r="E470" s="9" t="inlineStr">
         <is>
-          <t>In the room, hold an UNDATED row, then hold a repeating or dated one.</t>
+          <t>Hold a repeating row in the From Ours strip.</t>
         </is>
       </c>
       <c r="F470" s="9" t="inlineStr">
         <is>
-          <t>The undated row offers 'Bring to my Today'. The dated or repeating one does NOT: it already arrives by itself. Two routes landing in two different places (a copy in your list, or the strip) was the confusion Melroy hit twice.</t>
+          <t>Pin is there, Move to is not. A date and a rhythm are alternatives, and rescheduling a series is a question for the room's cadence sheet, not a one-tap action on a day.</t>
         </is>
       </c>
       <c r="G470" s="7" t="inlineStr">
@@ -19534,7 +19534,7 @@
     <row r="471">
       <c r="A471" s="6" t="inlineStr">
         <is>
-          <t>OUR-84</t>
+          <t>OUR-83</t>
         </is>
       </c>
       <c r="B471" s="7" t="inlineStr">
@@ -19549,17 +19549,17 @@
       </c>
       <c r="D471" s="9" t="inlineStr">
         <is>
-          <t>Take a From Ours row on, and it becomes an ordinary task</t>
+          <t>One shared row, one route onto your day</t>
         </is>
       </c>
       <c r="E471" s="9" t="inlineStr">
         <is>
-          <t>Hold a row in the From Just Us strip and choose 'Take this on today'.</t>
+          <t>In the room, hold an UNDATED row, then hold a repeating or dated one.</t>
         </is>
       </c>
       <c r="F471" s="9" t="inlineStr">
         <is>
-          <t>It leaves the strip and joins your list tagged '. Ours'. Holding it now gives the FULL held card: Break it down, Make tiny, Steps, Nudge, reorder, everything. That visible move IS the message: you have taken it on.</t>
+          <t>The undated row offers 'Bring to my Today'. The dated or repeating one does NOT: it already arrives by itself. Two routes landing in two different places (a copy in your list, or the strip) was the confusion Melroy hit twice.</t>
         </is>
       </c>
       <c r="G471" s="7" t="inlineStr">
@@ -19574,7 +19574,7 @@
     <row r="472">
       <c r="A472" s="6" t="inlineStr">
         <is>
-          <t>OUR-85</t>
+          <t>OUR-84</t>
         </is>
       </c>
       <c r="B472" s="7" t="inlineStr">
@@ -19582,24 +19582,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C472" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C472" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D472" s="9" t="inlineStr">
         <is>
-          <t>Break it down works once taken on, and never touches the shared list</t>
+          <t>Take a From Ours row on, and it becomes an ordinary task</t>
         </is>
       </c>
       <c r="E472" s="9" t="inlineStr">
         <is>
-          <t>Take a shared row on, then Break it down.</t>
+          <t>Hold a row in the From Just Us strip and choose 'Take this on today'.</t>
         </is>
       </c>
       <c r="F472" s="9" t="inlineStr">
         <is>
-          <t>The steps land on YOUR copy, on your day. The shared list is unchanged and your person sees nothing new. Breaking down was blocked on the shared row because a model authoring steps onto a list another person reads is a decision about them; on your own copy that objection is gone.</t>
+          <t>It leaves the strip and joins your list tagged '. Ours'. Holding it now gives the FULL held card: Break it down, Make tiny, Steps, Nudge, reorder, everything. That visible move IS the message: you have taken it on.</t>
         </is>
       </c>
       <c r="G472" s="7" t="inlineStr">
@@ -19614,7 +19614,7 @@
     <row r="473">
       <c r="A473" s="6" t="inlineStr">
         <is>
-          <t>OUR-86</t>
+          <t>OUR-85</t>
         </is>
       </c>
       <c r="B473" s="7" t="inlineStr">
@@ -19622,24 +19622,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C473" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C473" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D473" s="9" t="inlineStr">
         <is>
-          <t>Select several rows in the room and tick them together</t>
+          <t>Break it down works once taken on, and never touches the shared list</t>
         </is>
       </c>
       <c r="E473" s="9" t="inlineStr">
         <is>
-          <t>Hold a row, choose Select more, tap a few more, then Done.</t>
+          <t>Take a shared row on, then Break it down.</t>
         </is>
       </c>
       <c r="F473" s="9" t="inlineStr">
         <is>
-          <t>All of them tick at once and reach the other device. This is the trip-to-the-shops case: six things bought, six taps was a tax that stops people keeping the list.</t>
+          <t>The steps land on YOUR copy, on your day. The shared list is unchanged and your person sees nothing new. Breaking down was blocked on the shared row because a model authoring steps onto a list another person reads is a decision about them; on your own copy that objection is gone.</t>
         </is>
       </c>
       <c r="G473" s="7" t="inlineStr">
@@ -19654,7 +19654,7 @@
     <row r="474">
       <c r="A474" s="6" t="inlineStr">
         <is>
-          <t>OUR-87</t>
+          <t>OUR-86</t>
         </is>
       </c>
       <c r="B474" s="7" t="inlineStr">
@@ -19669,17 +19669,17 @@
       </c>
       <c r="D474" s="9" t="inlineStr">
         <is>
-          <t>Bulk tick never UN-ticks</t>
+          <t>Select several rows in the room and tick them together</t>
         </is>
       </c>
       <c r="E474" s="9" t="inlineStr">
         <is>
-          <t>Select a mix of done and not-done rows and tap Done.</t>
+          <t>Hold a row, choose Select more, tap a few more, then Done.</t>
         </is>
       </c>
       <c r="F474" s="9" t="inlineStr">
         <is>
-          <t>The not-done ones tick. The already-done ones are untouched. A bulk toggle would silently undo somebody's finished work on a mixed selection.</t>
+          <t>All of them tick at once and reach the other device. This is the trip-to-the-shops case: six things bought, six taps was a tax that stops people keeping the list.</t>
         </is>
       </c>
       <c r="G474" s="7" t="inlineStr">
@@ -19694,7 +19694,7 @@
     <row r="475">
       <c r="A475" s="6" t="inlineStr">
         <is>
-          <t>OUR-88</t>
+          <t>OUR-87</t>
         </is>
       </c>
       <c r="B475" s="7" t="inlineStr">
@@ -19709,17 +19709,17 @@
       </c>
       <c r="D475" s="9" t="inlineStr">
         <is>
-          <t>Bulk remove warns BEFORE the tap when a repeat is selected</t>
+          <t>Bulk tick never UN-ticks</t>
         </is>
       </c>
       <c r="E475" s="9" t="inlineStr">
         <is>
-          <t>Select a repeating row along with others. Read the shelf.</t>
+          <t>Select a mix of done and not-done rows and tap Done.</t>
         </is>
       </c>
       <c r="F475" s="9" t="inlineStr">
         <is>
-          <t>A line says removing a repeat here ends it for both of you. A shared list has no per-day skip, so this is not a thing to learn from the consequence.</t>
+          <t>The not-done ones tick. The already-done ones are untouched. A bulk toggle would silently undo somebody's finished work on a mixed selection.</t>
         </is>
       </c>
       <c r="G475" s="7" t="inlineStr">
@@ -19734,7 +19734,7 @@
     <row r="476">
       <c r="A476" s="6" t="inlineStr">
         <is>
-          <t>OUR-89</t>
+          <t>OUR-88</t>
         </is>
       </c>
       <c r="B476" s="7" t="inlineStr">
@@ -19742,24 +19742,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C476" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C476" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D476" s="9" t="inlineStr">
         <is>
-          <t>The pill steps aside for the select shelf</t>
+          <t>Bulk remove warns BEFORE the tap when a repeat is selected</t>
         </is>
       </c>
       <c r="E476" s="9" t="inlineStr">
         <is>
-          <t>Enter select mode in the room with a few words waiting in the capture panel.</t>
+          <t>Select a repeating row along with others. Read the shelf.</t>
         </is>
       </c>
       <c r="F476" s="9" t="inlineStr">
         <is>
-          <t>The pill is gone while selecting (the select shelf docks at the foot), and back when you cancel, still showing its waiting words. Two bottom-anchored surfaces competing for the thumb is how a calm screen stops being one, and you are not adding things while you are clearing things.</t>
+          <t>A line says removing a repeat here ends it for both of you. A shared list has no per-day skip, so this is not a thing to learn from the consequence.</t>
         </is>
       </c>
       <c r="G476" s="7" t="inlineStr">
@@ -19774,7 +19774,7 @@
     <row r="477">
       <c r="A477" s="6" t="inlineStr">
         <is>
-          <t>OUR-90</t>
+          <t>OUR-89</t>
         </is>
       </c>
       <c r="B477" s="7" t="inlineStr">
@@ -19782,24 +19782,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C477" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C477" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D477" s="9" t="inlineStr">
         <is>
-          <t>No select mode on a closed list</t>
+          <t>The pill steps aside for the select shelf</t>
         </is>
       </c>
       <c r="E477" s="9" t="inlineStr">
         <is>
-          <t>Open an archived list and hold a row.</t>
+          <t>Enter select mode in the room with a few words waiting in the capture panel.</t>
         </is>
       </c>
       <c r="F477" s="9" t="inlineStr">
         <is>
-          <t>No Select more. A closed list is readable and nothing else, and the server would refuse the write anyway.</t>
+          <t>The pill is gone while selecting (the select shelf docks at the foot), and back when you cancel, still showing its waiting words. Two bottom-anchored surfaces competing for the thumb is how a calm screen stops being one, and you are not adding things while you are clearing things.</t>
         </is>
       </c>
       <c r="G477" s="7" t="inlineStr">
@@ -19814,7 +19814,7 @@
     <row r="478">
       <c r="A478" s="6" t="inlineStr">
         <is>
-          <t>OUR-91</t>
+          <t>OUR-90</t>
         </is>
       </c>
       <c r="B478" s="7" t="inlineStr">
@@ -19822,24 +19822,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C478" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C478" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D478" s="9" t="inlineStr">
         <is>
-          <t>A copy says when its shared row was taken off the list</t>
+          <t>No select mode on a closed list</t>
         </is>
       </c>
       <c r="E478" s="9" t="inlineStr">
         <is>
-          <t>Device B removes a row from Ours. On device A, look at the brought copy on Today.</t>
+          <t>Open an archived list and hold a row.</t>
         </is>
       </c>
       <c r="F478" s="9" t="inlineStr">
         <is>
-          <t>The copy STAYS (it is your task now) and carries a faint line: 'no longer on &lt;list name&gt;'. The deciding case is wasted effort: she removed milk because she already bought it, and a silent copy sends you to the shop.</t>
+          <t>No Select more. A closed list is readable and nothing else, and the server would refuse the write anyway.</t>
         </is>
       </c>
       <c r="G478" s="7" t="inlineStr">
@@ -19854,7 +19854,7 @@
     <row r="479">
       <c r="A479" s="6" t="inlineStr">
         <is>
-          <t>OUR-92</t>
+          <t>OUR-91</t>
         </is>
       </c>
       <c r="B479" s="7" t="inlineStr">
@@ -19869,17 +19869,17 @@
       </c>
       <c r="D479" s="9" t="inlineStr">
         <is>
-          <t>That line never says who, and never says why</t>
+          <t>A copy says when its shared row was taken off the list</t>
         </is>
       </c>
       <c r="E479" s="9" t="inlineStr">
         <is>
-          <t>Read the line closely.</t>
+          <t>Device B removes a row from Ours. On device A, look at the brought copy on Today.</t>
         </is>
       </c>
       <c r="F479" s="9" t="inlineStr">
         <is>
-          <t>It states the fact only. Not who removed it (no such data exists anywhere in this feature, and a bridge is where that temptation returns) and not why (removal could be done, not-needed or tidying, and the app cannot tell them apart).</t>
+          <t>The copy STAYS (it is your task now) and carries a faint line: 'no longer on &lt;list name&gt;'. The deciding case is wasted effort: she removed milk because she already bought it, and a silent copy sends you to the shop.</t>
         </is>
       </c>
       <c r="G479" s="7" t="inlineStr">
@@ -19894,7 +19894,7 @@
     <row r="480">
       <c r="A480" s="6" t="inlineStr">
         <is>
-          <t>OUR-93</t>
+          <t>OUR-92</t>
         </is>
       </c>
       <c r="B480" s="7" t="inlineStr">
@@ -19902,24 +19902,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C480" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C480" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D480" s="9" t="inlineStr">
         <is>
-          <t>No line on a copy you already finished or removed</t>
+          <t>That line never says who, and never says why</t>
         </is>
       </c>
       <c r="E480" s="9" t="inlineStr">
         <is>
-          <t>Finish your copy, then have B remove the shared row. Then try it with a copy you removed yourself.</t>
+          <t>Read the line closely.</t>
         </is>
       </c>
       <c r="F480" s="9" t="inlineStr">
         <is>
-          <t>No line in either case. You did the thing, so its origin's fate is not news, and a note there would read as a correction.</t>
+          <t>It states the fact only. Not who removed it (no such data exists anywhere in this feature, and a bridge is where that temptation returns) and not why (removal could be done, not-needed or tidying, and the app cannot tell them apart).</t>
         </is>
       </c>
       <c r="G480" s="7" t="inlineStr">
@@ -19934,7 +19934,7 @@
     <row r="481">
       <c r="A481" s="6" t="inlineStr">
         <is>
-          <t>OUR-94</t>
+          <t>OUR-93</t>
         </is>
       </c>
       <c r="B481" s="7" t="inlineStr">
@@ -19942,24 +19942,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C481" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C481" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D481" s="9" t="inlineStr">
         <is>
-          <t>The line goes quiet after the tombstone sweep, rather than guessing</t>
+          <t>No line on a copy you already finished or removed</t>
         </is>
       </c>
       <c r="E481" s="9" t="inlineStr">
         <is>
-          <t>More than seven days after a removal (or with the tombstone swept), check the copy.</t>
+          <t>Finish your copy, then have B remove the shared row. Then try it with a copy you removed yourself.</t>
         </is>
       </c>
       <c r="F481" s="9" t="inlineStr">
         <is>
-          <t>No line. A swept origin is indistinguishable from one never pulled, and keeping a permanent record of a deletion so the app can keep mentioning it is its own kind of creepy. Accepted limit, not a bug.</t>
+          <t>No line in either case. You did the thing, so its origin's fate is not news, and a note there would read as a correction.</t>
         </is>
       </c>
       <c r="G481" s="7" t="inlineStr">
@@ -19974,7 +19974,7 @@
     <row r="482">
       <c r="A482" s="6" t="inlineStr">
         <is>
-          <t>OUR-95</t>
+          <t>OUR-94</t>
         </is>
       </c>
       <c r="B482" s="7" t="inlineStr">
@@ -19982,24 +19982,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C482" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C482" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D482" s="9" t="inlineStr">
         <is>
-          <t>A row's note is VISIBLE, not only spoken</t>
+          <t>The line goes quiet after the tombstone sweep, rather than guessing</t>
         </is>
       </c>
       <c r="E482" s="9" t="inlineStr">
         <is>
-          <t>Trigger any row note: have B change a row (the room's wash) or remove a shared row you hold a copy of (Today).</t>
+          <t>More than seven days after a removal (or with the tombstone swept), check the copy.</t>
         </is>
       </c>
       <c r="F482" s="9" t="inlineStr">
         <is>
-          <t>The words appear as a quiet second line under the title. Before 2026-08-12 the note prop reached only the accessibility label, so every one of these lines was spoken to screen readers and shown to nobody, for as long as the prop had existed.</t>
+          <t>No line. A swept origin is indistinguishable from one never pulled, and keeping a permanent record of a deletion so the app can keep mentioning it is its own kind of creepy. Accepted limit, not a bug.</t>
         </is>
       </c>
       <c r="G482" s="7" t="inlineStr">
@@ -20014,7 +20014,7 @@
     <row r="483">
       <c r="A483" s="6" t="inlineStr">
         <is>
-          <t>OUR-96</t>
+          <t>OUR-95</t>
         </is>
       </c>
       <c r="B483" s="7" t="inlineStr">
@@ -20022,24 +20022,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C483" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C483" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D483" s="9" t="inlineStr">
         <is>
-          <t>Rows WITHOUT a note are unchanged</t>
+          <t>A row's note is VISIBLE, not only spoken</t>
         </is>
       </c>
       <c r="E483" s="9" t="inlineStr">
         <is>
-          <t>Compare a plain row, a 'big' row and a repeating row against a build before the note landed.</t>
+          <t>Trigger any row note: have B change a row (the room's wash) or remove a shared row you hold a copy of (Today).</t>
         </is>
       </c>
       <c r="F483" s="9" t="inlineStr">
         <is>
-          <t>Same height to within a pixel. The note gave TaskRow a second line, and a row that has no note must not gain one, shift, or reflow.</t>
+          <t>The words appear as a quiet second line under the title. Before 2026-08-12 the note prop reached only the accessibility label, so every one of these lines was spoken to screen readers and shown to nobody, for as long as the prop had existed.</t>
         </is>
       </c>
       <c r="G483" s="7" t="inlineStr">
@@ -20054,7 +20054,7 @@
     <row r="484">
       <c r="A484" s="6" t="inlineStr">
         <is>
-          <t>OUR-97</t>
+          <t>OUR-96</t>
         </is>
       </c>
       <c r="B484" s="7" t="inlineStr">
@@ -20062,24 +20062,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C484" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C484" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D484" s="9" t="inlineStr">
         <is>
-          <t>A tick after midnight lands on the RIGHT day</t>
+          <t>Rows WITHOUT a note are unchanged</t>
         </is>
       </c>
       <c r="E484" s="9" t="inlineStr">
         <is>
-          <t>Open the room at 23:58 and leave it open. Tick a row at 00:02. Check the partner's device.</t>
+          <t>Compare a plain row, a 'big' row and a repeating row against a build before the note landed.</t>
         </is>
       </c>
       <c r="F484" s="9" t="inlineStr">
         <is>
-          <t>Done on both, dated today. The room's date used to freeze at mount, so the completion log took yesterday's key and the partner's phone, asking about today, got false. Permanently: the merge is per-date.</t>
+          <t>Same height to within a pixel. The note gave TaskRow a second line, and a row that has no note must not gain one, shift, or reflow.</t>
         </is>
       </c>
       <c r="G484" s="7" t="inlineStr">
@@ -20094,7 +20094,7 @@
     <row r="485">
       <c r="A485" s="6" t="inlineStr">
         <is>
-          <t>OUR-98</t>
+          <t>OUR-97</t>
         </is>
       </c>
       <c r="B485" s="7" t="inlineStr">
@@ -20109,17 +20109,17 @@
       </c>
       <c r="D485" s="9" t="inlineStr">
         <is>
-          <t>A tick made during a background sync is not undone</t>
+          <t>A tick after midnight lands on the RIGHT day</t>
         </is>
       </c>
       <c r="E485" s="9" t="inlineStr">
         <is>
-          <t>Background and reopen the app (which triggers a settle), then immediately tick a row in the From Ours strip.</t>
+          <t>Open the room at 23:58 and leave it open. Tick a row at 00:02. Check the partner's device.</t>
         </is>
       </c>
       <c r="F485" s="9" t="inlineStr">
         <is>
-          <t>It stays ticked. The settle now refuses to save a merge that predates any local write made while it was on the wire.</t>
+          <t>Done on both, dated today. The room's date used to freeze at mount, so the completion log took yesterday's key and the partner's phone, asking about today, got false. Permanently: the merge is per-date.</t>
         </is>
       </c>
       <c r="G485" s="7" t="inlineStr">
@@ -20134,7 +20134,7 @@
     <row r="486">
       <c r="A486" s="6" t="inlineStr">
         <is>
-          <t>OUR-99</t>
+          <t>OUR-98</t>
         </is>
       </c>
       <c r="B486" s="7" t="inlineStr">
@@ -20149,17 +20149,17 @@
       </c>
       <c r="D486" s="9" t="inlineStr">
         <is>
-          <t>A tick survives a device that has never opened the room</t>
+          <t>A tick made during a background sync is not undone</t>
         </is>
       </c>
       <c r="E486" s="9" t="inlineStr">
         <is>
-          <t>On a device with no Ours cache, go offline, tick a brought copy, come back online, reopen the app.</t>
+          <t>Background and reopen the app (which triggers a settle), then immediately tick a row in the From Ours strip.</t>
         </is>
       </c>
       <c r="F486" s="9" t="inlineStr">
         <is>
-          <t>The tick reaches the shared list. It used to be lost forever: the only carrier pulled before writing, and nothing retried. The settle now carries it, with the copy's OWN completion time, so a deliberate un-tick on the other side still wins.</t>
+          <t>It stays ticked. The settle now refuses to save a merge that predates any local write made while it was on the wire.</t>
         </is>
       </c>
       <c r="G486" s="7" t="inlineStr">
@@ -20174,7 +20174,7 @@
     <row r="487">
       <c r="A487" s="6" t="inlineStr">
         <is>
-          <t>OUR-100</t>
+          <t>OUR-99</t>
         </is>
       </c>
       <c r="B487" s="7" t="inlineStr">
@@ -20189,17 +20189,17 @@
       </c>
       <c r="D487" s="9" t="inlineStr">
         <is>
-          <t>A repeat is visible in the room EVERY day, tickable only on its own</t>
+          <t>A tick survives a device that has never opened the room</t>
         </is>
       </c>
       <c r="E487" s="9" t="inlineStr">
         <is>
-          <t>Make a weekly shared repeat. Open the room on a day it is not due.</t>
+          <t>On a device with no Ours cache, go offline, tick a brought copy, come back online, reopen the app.</t>
         </is>
       </c>
       <c r="F487" s="9" t="inlineStr">
         <is>
-          <t>The row is there, with its rhythm in words, and its checkbox is inert with 'you can tick this on its day'. It used to vanish six days a week: unreachable to edit or remove, and a list of only repeats said 'Nothing here yet'.</t>
+          <t>The tick reaches the shared list. It used to be lost forever: the only carrier pulled before writing, and nothing retried. The settle now carries it, with the copy's OWN completion time, so a deliberate un-tick on the other side still wins.</t>
         </is>
       </c>
       <c r="G487" s="7" t="inlineStr">
@@ -20214,7 +20214,7 @@
     <row r="488">
       <c r="A488" s="6" t="inlineStr">
         <is>
-          <t>OUR-101</t>
+          <t>OUR-100</t>
         </is>
       </c>
       <c r="B488" s="7" t="inlineStr">
@@ -20222,24 +20222,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C488" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C488" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D488" s="9" t="inlineStr">
         <is>
-          <t>A closed list stops promising it keeps trying</t>
+          <t>A repeat is visible in the room EVERY day, tickable only on its own</t>
         </is>
       </c>
       <c r="E488" s="9" t="inlineStr">
         <is>
-          <t>Open an archived list that has unpushed local changes.</t>
+          <t>Make a weekly shared repeat. Open the room on a day it is not due.</t>
         </is>
       </c>
       <c r="F488" s="9" t="inlineStr">
         <is>
-          <t>It says the list is closed, not 'Saved here, not there'. On a list where the write can never succeed, the second is a false hope on a screen a separated or bereaved person may keep for years.</t>
+          <t>The row is there, with its rhythm in words, and its checkbox is inert with 'you can tick this on its day'. It used to vanish six days a week: unreachable to edit or remove, and a list of only repeats said 'Nothing here yet'.</t>
         </is>
       </c>
       <c r="G488" s="7" t="inlineStr">
@@ -20254,7 +20254,7 @@
     <row r="489">
       <c r="A489" s="6" t="inlineStr">
         <is>
-          <t>OUR-102</t>
+          <t>OUR-101</t>
         </is>
       </c>
       <c r="B489" s="7" t="inlineStr">
@@ -20269,17 +20269,17 @@
       </c>
       <c r="D489" s="9" t="inlineStr">
         <is>
-          <t>Setting a rhythm clears any date the row was carrying</t>
+          <t>A closed list stops promising it keeps trying</t>
         </is>
       </c>
       <c r="E489" s="9" t="inlineStr">
         <is>
-          <t>Give a DATED shared row a weekly rhythm, then read the row.</t>
+          <t>Open an archived list that has unpushed local changes.</t>
         </is>
       </c>
       <c r="F489" s="9" t="inlineStr">
         <is>
-          <t>One schedule, not two. The date is gone. Leaving it made the row answer differently depending on which code asked.</t>
+          <t>It says the list is closed, not 'Saved here, not there'. On a list where the write can never succeed, the second is a false hope on a screen a separated or bereaved person may keep for years.</t>
         </is>
       </c>
       <c r="G489" s="7" t="inlineStr">
@@ -20294,7 +20294,7 @@
     <row r="490">
       <c r="A490" s="6" t="inlineStr">
         <is>
-          <t>OUR-103</t>
+          <t>OUR-102</t>
         </is>
       </c>
       <c r="B490" s="7" t="inlineStr">
@@ -20309,17 +20309,17 @@
       </c>
       <c r="D490" s="9" t="inlineStr">
         <is>
-          <t>Renaming inside the cadence sheet warns about the 500-character cap</t>
+          <t>Setting a rhythm clears any date the row was carrying</t>
         </is>
       </c>
       <c r="E490" s="9" t="inlineStr">
         <is>
-          <t>Open a row's rhythm sheet, paste a title over 500 characters, save.</t>
+          <t>Give a DATED shared row a weekly rhythm, then read the row.</t>
         </is>
       </c>
       <c r="F490" s="9" t="inlineStr">
         <is>
-          <t>The trim notice appears BEFORE the save, the same as renaming on the row. It used to save silently and the server clamped it, so the words vanished a second later.</t>
+          <t>One schedule, not two. The date is gone. Leaving it made the row answer differently depending on which code asked.</t>
         </is>
       </c>
       <c r="G490" s="7" t="inlineStr">
@@ -20334,7 +20334,7 @@
     <row r="491">
       <c r="A491" s="6" t="inlineStr">
         <is>
-          <t>OUR-104</t>
+          <t>OUR-103</t>
         </is>
       </c>
       <c r="B491" s="7" t="inlineStr">
@@ -20342,24 +20342,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C491" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C491" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D491" s="9" t="inlineStr">
         <is>
-          <t>No dead reorder rail on shared rows</t>
+          <t>Renaming inside the cadence sheet warns about the 500-character cap</t>
         </is>
       </c>
       <c r="E491" s="9" t="inlineStr">
         <is>
-          <t>Hold a row in the room and in the From Ours strip.</t>
+          <t>Open a row's rhythm sheet, paste a title over 500 characters, save.</t>
         </is>
       </c>
       <c r="F491" s="9" t="inlineStr">
         <is>
-          <t>No up/down rail. Neither surface supplies those handlers, so it was two permanently inert controls on the screen briefed to be plainer than Today. Dim-in-place is for a control that is sometimes live.</t>
+          <t>The trim notice appears BEFORE the save, the same as renaming on the row. It used to save silently and the server clamped it, so the words vanished a second later.</t>
         </is>
       </c>
       <c r="G491" s="7" t="inlineStr">
@@ -20374,7 +20374,7 @@
     <row r="492">
       <c r="A492" s="6" t="inlineStr">
         <is>
-          <t>OUR-105</t>
+          <t>OUR-104</t>
         </is>
       </c>
       <c r="B492" s="7" t="inlineStr">
@@ -20382,24 +20382,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C492" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C492" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D492" s="9" t="inlineStr">
         <is>
-          <t>First run introduces the shared list</t>
+          <t>No dead reorder rail on shared rows</t>
         </is>
       </c>
       <c r="E492" s="9" t="inlineStr">
         <is>
-          <t>Reset onboarding (Settings, replay the first run) and step through it.</t>
+          <t>Hold a row in the room and in the From Ours strip.</t>
         </is>
       </c>
       <c r="F492" s="9" t="inlineStr">
         <is>
-          <t>An eighth step sits between 'keep' and 'premium', headed 'A list the two of you keep.' It says what arrives by itself, what deliberately does NOT, and that nothing keeps score. Its position matters: a FREE feature read immediately before the premium screen would be mistaken for part of the paid list.</t>
+          <t>No up/down rail. Neither surface supplies those handlers, so it was two permanently inert controls on the screen briefed to be plainer than Today. Dim-in-place is for a control that is sometimes live.</t>
         </is>
       </c>
       <c r="G492" s="7" t="inlineStr">
@@ -20414,7 +20414,7 @@
     <row r="493">
       <c r="A493" s="6" t="inlineStr">
         <is>
-          <t>OUR-106</t>
+          <t>OUR-105</t>
         </is>
       </c>
       <c r="B493" s="7" t="inlineStr">
@@ -20429,17 +20429,17 @@
       </c>
       <c r="D493" s="9" t="inlineStr">
         <is>
-          <t>Anyone can start a shared list, not just an allowlisted address</t>
+          <t>First run introduces the shared list</t>
         </is>
       </c>
       <c r="E493" s="9" t="inlineStr">
         <is>
-          <t>With supabase/ours-open.sql applied, sign in as an account that was never in ours_allowlist and create an invite.</t>
+          <t>Reset onboarding (Settings, replay the first run) and step through it.</t>
         </is>
       </c>
       <c r="F493" s="9" t="inlineStr">
         <is>
-          <t>It works. Before that migration only JOINING was open; STARTING was gated, so the refusal hit exactly the person a store listing brings you.</t>
+          <t>An eighth step sits between 'keep' and 'premium', headed 'A list the two of you keep.' It says what arrives by itself, what deliberately does NOT, and that nothing keeps score. Its position matters: a FREE feature read immediately before the premium screen would be mistaken for part of the paid list.</t>
         </is>
       </c>
       <c r="G493" s="7" t="inlineStr">
@@ -20454,7 +20454,7 @@
     <row r="494">
       <c r="A494" s="6" t="inlineStr">
         <is>
-          <t>OUR-107</t>
+          <t>OUR-106</t>
         </is>
       </c>
       <c r="B494" s="7" t="inlineStr">
@@ -20469,17 +20469,17 @@
       </c>
       <c r="D494" s="9" t="inlineStr">
         <is>
-          <t>The shared-list onboarding step can actually be REACHED</t>
+          <t>Anyone can start a shared list, not just an allowlisted address</t>
         </is>
       </c>
       <c r="E494" s="9" t="inlineStr">
         <is>
-          <t>Replay the first run and press the primary button through every step without skipping.</t>
+          <t>With supabase/ours-open.sql applied, sign in as an account that was never in ours_allowlist and create an invite.</t>
         </is>
       </c>
       <c r="F494" s="9" t="inlineStr">
         <is>
-          <t>The shared-list screen appears as the sixth of eight, between 'What you finish, you keep' and the premium screen. It shipped once as a step that existed, was translated into five languages, and could not be arrived at: the flow advanced by a hand-written map that still went keep -&gt; premium.</t>
+          <t>It works. Before that migration only JOINING was open; STARTING was gated, so the refusal hit exactly the person a store listing brings you.</t>
         </is>
       </c>
       <c r="G494" s="7" t="inlineStr">
@@ -20494,7 +20494,7 @@
     <row r="495">
       <c r="A495" s="6" t="inlineStr">
         <is>
-          <t>OUR-108</t>
+          <t>OUR-107</t>
         </is>
       </c>
       <c r="B495" s="7" t="inlineStr">
@@ -20502,24 +20502,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C495" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C495" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D495" s="9" t="inlineStr">
         <is>
-          <t>ONE person, TWO devices: does your own edit wash on your other phone?</t>
+          <t>The shared-list onboarding step can actually be REACHED</t>
         </is>
       </c>
       <c r="E495" s="9" t="inlineStr">
         <is>
-          <t>Sign in to the same account on two devices (an iPhone and an Android, say). Change a row in Ours on the FIRST. Open Ours on the SECOND.</t>
+          <t>Replay the first run and press the primary button through every step without skipping.</t>
         </is>
       </c>
       <c r="F495" s="9" t="inlineStr">
         <is>
-          <t>OPEN QUESTION, not a known-good expectation. The 'this edit was mine' record is stored PER DEVICE (noteOursMine writes to local storage), so the second device has no idea the first one did it and will most likely tint the row as changed-since-you-looked. It breaks none of the three laws, since the wording never names a person, but it may still read wrong: your own edit wearing the mark that means 'your person did something'. Only reachable when one person holds two phones, which nobody did until 2026-08-13. If it tints, the fix is to key `mine` on the account rather than the device.</t>
+          <t>The shared-list screen appears as the sixth of eight, between 'What you finish, you keep' and the premium screen. It shipped once as a step that existed, was translated into five languages, and could not be arrived at: the flow advanced by a hand-written map that still went keep -&gt; premium.</t>
         </is>
       </c>
       <c r="G495" s="7" t="inlineStr">
@@ -20534,7 +20534,7 @@
     <row r="496">
       <c r="A496" s="6" t="inlineStr">
         <is>
-          <t>OUR-109</t>
+          <t>OUR-108</t>
         </is>
       </c>
       <c r="B496" s="7" t="inlineStr">
@@ -20542,24 +20542,24 @@
           <t>Ours</t>
         </is>
       </c>
-      <c r="C496" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C496" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D496" s="9" t="inlineStr">
         <is>
-          <t>A repeat's rhythm sits INSIDE its own card and reads as a rhythm</t>
+          <t>ONE person, TWO devices: does your own edit wash on your other phone?</t>
         </is>
       </c>
       <c r="E496" s="9" t="inlineStr">
         <is>
-          <t>Give a shared task a weekly repeat on a weekday that is not today. Look at it in the room.</t>
+          <t>Sign in to the same account on two devices (an iPhone and an Android, say). Change a row in Ours on the FIRST. Open Ours on the SECOND.</t>
         </is>
       </c>
       <c r="F496" s="9" t="inlineStr">
         <is>
-          <t>The line is indented under that row's title, inside the card, and reads 'Every Thu' rather than a bare 'Thu'. It used to be drawn BELOW the card, so it floated between two rows belonging to neither, and said only the weekday.</t>
+          <t>OPEN QUESTION, not a known-good expectation. The 'this edit was mine' record is stored PER DEVICE (noteOursMine writes to local storage), so the second device has no idea the first one did it and will most likely tint the row as changed-since-you-looked. It breaks none of the three laws, since the wording never names a person, but it may still read wrong: your own edit wearing the mark that means 'your person did something'. Only reachable when one person holds two phones, which nobody did until 2026-08-13. If it tints, the fix is to key `mine` on the account rather than the device.</t>
         </is>
       </c>
       <c r="G496" s="7" t="inlineStr">
@@ -20574,7 +20574,7 @@
     <row r="497">
       <c r="A497" s="6" t="inlineStr">
         <is>
-          <t>OUR-110</t>
+          <t>OUR-109</t>
         </is>
       </c>
       <c r="B497" s="7" t="inlineStr">
@@ -20589,17 +20589,17 @@
       </c>
       <c r="D497" s="9" t="inlineStr">
         <is>
-          <t>A circle you cannot tick LOOKS like one you cannot tick</t>
+          <t>A repeat's rhythm sits INSIDE its own card and reads as a rhythm</t>
         </is>
       </c>
       <c r="E497" s="9" t="inlineStr">
         <is>
-          <t>Find that same repeat on a day it is not due, or open any row on a closed list.</t>
+          <t>Give a shared task a weekly repeat on a weekday that is not today. Look at it in the room.</t>
         </is>
       </c>
       <c r="F497" s="9" t="inlineStr">
         <is>
-          <t>The circle is visibly faded. It used to render identically to a live one, so the row offered a control that looked tappable and did nothing, which is the exact failure the 'quiet-unavailable' rule was written to prevent.</t>
+          <t>The line is indented under that row's title, inside the card, and reads 'Every Thu' rather than a bare 'Thu'. It used to be drawn BELOW the card, so it floated between two rows belonging to neither, and said only the weekday.</t>
         </is>
       </c>
       <c r="G497" s="7" t="inlineStr">
@@ -20614,12 +20614,12 @@
     <row r="498">
       <c r="A498" s="6" t="inlineStr">
         <is>
-          <t>UPD-01</t>
+          <t>OUR-110</t>
         </is>
       </c>
       <c r="B498" s="7" t="inlineStr">
         <is>
-          <t>Updates</t>
+          <t>Ours</t>
         </is>
       </c>
       <c r="C498" s="8" t="inlineStr">
@@ -20629,17 +20629,17 @@
       </c>
       <c r="D498" s="9" t="inlineStr">
         <is>
-          <t>Settings states the version, and up-to-date is a fact</t>
+          <t>A circle you cannot tick LOOKS like one you cannot tick</t>
         </is>
       </c>
       <c r="E498" s="9" t="inlineStr">
         <is>
-          <t>Open Settings and scroll to the foot.</t>
+          <t>Find that same repeat on a day it is not due, or open any row on a closed list.</t>
         </is>
       </c>
       <c r="F498" s="9" t="inlineStr">
         <is>
-          <t>One line: 'v1.2.0 (11)  ·  Up to date'. It is a sage FACT, not a control. Nothing is offered when there is nothing to offer.</t>
+          <t>The circle is visibly faded. It used to render identically to a live one, so the row offered a control that looked tappable and did nothing, which is the exact failure the 'quiet-unavailable' rule was written to prevent.</t>
         </is>
       </c>
       <c r="G498" s="7" t="inlineStr">
@@ -20654,7 +20654,7 @@
     <row r="499">
       <c r="A499" s="6" t="inlineStr">
         <is>
-          <t>UPD-02</t>
+          <t>UPD-01</t>
         </is>
       </c>
       <c r="B499" s="7" t="inlineStr">
@@ -20669,22 +20669,22 @@
       </c>
       <c r="D499" s="9" t="inlineStr">
         <is>
-          <t>Web offers a reload, and says drafts are kept</t>
+          <t>Settings states the version, and up-to-date is a fact</t>
         </is>
       </c>
       <c r="E499" s="9" t="inlineStr">
         <is>
-          <t>With doubledone.app/version.json's "web" set ahead of the running build, open Settings on the web.</t>
+          <t>Open Settings and scroll to the foot.</t>
         </is>
       </c>
       <c r="F499" s="9" t="inlineStr">
         <is>
-          <t>'A newer version is ready.' + 'Reload to get it' + 'Anything you were typing is kept.' Type something into the capture box first and confirm it survives the reload.</t>
+          <t>One line: 'v1.2.0 (11)  ·  Up to date'. It is a sage FACT, not a control. Nothing is offered when there is nothing to offer.</t>
         </is>
       </c>
       <c r="G499" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H499" s="7" t="inlineStr"/>
@@ -20694,7 +20694,7 @@
     <row r="500">
       <c r="A500" s="6" t="inlineStr">
         <is>
-          <t>UPD-03</t>
+          <t>UPD-02</t>
         </is>
       </c>
       <c r="B500" s="7" t="inlineStr">
@@ -20709,22 +20709,22 @@
       </c>
       <c r="D500" s="9" t="inlineStr">
         <is>
-          <t>Native points at the store, and says lists are untouched</t>
+          <t>Web offers a reload, and says drafts are kept</t>
         </is>
       </c>
       <c r="E500" s="9" t="inlineStr">
         <is>
-          <t>With version.json's "ios" / "android" set ahead of the installed build, open Settings on a device.</t>
+          <t>With doubledone.app/version.json's "web" set ahead of the running build, open Settings on the web.</t>
         </is>
       </c>
       <c r="F500" s="9" t="inlineStr">
         <is>
-          <t>'This build is getting old.' + 'Open the store' + 'Your lists stay exactly as they are.' The button opens the correct store listing.</t>
+          <t>'A newer version is ready.' + 'Reload to get it' + 'Anything you were typing is kept.' Type something into the capture box first and confirm it survives the reload.</t>
         </is>
       </c>
       <c r="G500" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H500" s="7" t="inlineStr"/>
@@ -20734,7 +20734,7 @@
     <row r="501">
       <c r="A501" s="6" t="inlineStr">
         <is>
-          <t>UPD-04</t>
+          <t>UPD-03</t>
         </is>
       </c>
       <c r="B501" s="7" t="inlineStr">
@@ -20742,29 +20742,29 @@
           <t>Updates</t>
         </is>
       </c>
-      <c r="C501" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C501" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D501" s="9" t="inlineStr">
         <is>
-          <t>Unreachable server says NOTHING, never 'up to date'</t>
+          <t>Native points at the store, and says lists are untouched</t>
         </is>
       </c>
       <c r="E501" s="9" t="inlineStr">
         <is>
-          <t>Put the device in aeroplane mode and open Settings. Then, online, confirm doubledone.app/version.json returns JSON rather than the app's HTML (the SPA fallback would break it silently).</t>
+          <t>With version.json's "ios" / "android" set ahead of the installed build, open Settings on a device.</t>
         </is>
       </c>
       <c r="F501" s="9" t="inlineStr">
         <is>
-          <t>No update line at all, and no 'Up to date' either: it cannot tell, so it says nothing. No spinner and no error.</t>
+          <t>'This build is getting old.' + 'Open the store' + 'Your lists stay exactly as they are.' The button opens the correct store listing.</t>
         </is>
       </c>
       <c r="G501" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H501" s="7" t="inlineStr"/>
@@ -20774,7 +20774,7 @@
     <row r="502">
       <c r="A502" s="6" t="inlineStr">
         <is>
-          <t>UPD-05</t>
+          <t>UPD-04</t>
         </is>
       </c>
       <c r="B502" s="7" t="inlineStr">
@@ -20789,17 +20789,17 @@
       </c>
       <c r="D502" s="9" t="inlineStr">
         <is>
-          <t>The goodnight mention is rare, and framed for the other person</t>
+          <t>Unreachable server says NOTHING, never 'up to date'</t>
         </is>
       </c>
       <c r="E502" s="9" t="inlineStr">
         <is>
-          <t>Clear the day with a build two minor versions behind, and reach the rested screen.</t>
+          <t>Put the device in aeroplane mode and open Settings. Then, online, confirm doubledone.app/version.json returns JSON rather than the app's HTML (the SPA fallback would break it silently).</t>
         </is>
       </c>
       <c r="F502" s="9" t="inlineStr">
         <is>
-          <t>At most ONE offer shows. If it is the update one it reads 'The newer one can read everything your person sets, rhythms included.' 'Not now' dismisses it and it does not return for a fortnight. It never displaces the reminder, widget or scrapbook offer.</t>
+          <t>No update line at all, and no 'Up to date' either: it cannot tell, so it says nothing. No spinner and no error.</t>
         </is>
       </c>
       <c r="G502" s="7" t="inlineStr">
@@ -20814,7 +20814,7 @@
     <row r="503">
       <c r="A503" s="6" t="inlineStr">
         <is>
-          <t>UPD-06</t>
+          <t>UPD-05</t>
         </is>
       </c>
       <c r="B503" s="7" t="inlineStr">
@@ -20822,29 +20822,29 @@
           <t>Updates</t>
         </is>
       </c>
-      <c r="C503" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C503" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D503" s="9" t="inlineStr">
         <is>
-          <t>The web never says it is behind itself</t>
+          <t>The goodnight mention is rare, and framed for the other person</t>
         </is>
       </c>
       <c r="E503" s="9" t="inlineStr">
         <is>
-          <t>Right after a web deploy (or on any ordinary day), open Settings on doubledone.app in a fresh tab. Read the version line at the foot of Settings.</t>
+          <t>Clear the day with a build two minor versions behind, and reach the rested screen.</t>
         </is>
       </c>
       <c r="F503" s="9" t="inlineStr">
         <is>
-          <t>It reads v&lt;the app.json version&gt; (web), for example v1.8.0 (web), never v1.2.0, and there is NO 'A newer version is ready' line (UPD-02 covers the case where the web really is behind). Fixed 2026-10-05: the web used to fall back to 1.2.0 and nag forever.</t>
+          <t>At most ONE offer shows. If it is the update one it reads 'The newer one can read everything your person sets, rhythms included.' 'Not now' dismisses it and it does not return for a fortnight. It never displaces the reminder, widget or scrapbook offer.</t>
         </is>
       </c>
       <c r="G503" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H503" s="7" t="inlineStr"/>
@@ -20854,37 +20854,37 @@
     <row r="504">
       <c r="A504" s="6" t="inlineStr">
         <is>
-          <t>OUR-12</t>
+          <t>UPD-06</t>
         </is>
       </c>
       <c r="B504" s="7" t="inlineStr">
         <is>
-          <t>Ours</t>
-        </is>
-      </c>
-      <c r="C504" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>Updates</t>
+        </is>
+      </c>
+      <c r="C504" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D504" s="9" t="inlineStr">
         <is>
-          <t>Unnamed lists read in each person's language</t>
+          <t>The web never says it is behind itself</t>
         </is>
       </c>
       <c r="E504" s="9" t="inlineStr">
         <is>
-          <t>Create a list WITHOUT naming it. Set the two accounts' devices to different languages (e.g. English and Italian).</t>
+          <t>Right after a web deploy (or on any ordinary day), open Settings on doubledone.app in a fresh tab. Read the version line at the foot of Settings.</t>
         </is>
       </c>
       <c r="F504" s="9" t="inlineStr">
         <is>
-          <t>Each person sees the app's own word for a shared list in their own language, not the other person's.</t>
+          <t>It reads v&lt;the app.json version&gt; (web), for example v1.8.0 (web), never v1.2.0, and there is NO 'A newer version is ready' line (UPD-02 covers the case where the web really is behind). Fixed 2026-10-05: the web used to fall back to 1.2.0 and nag forever.</t>
         </is>
       </c>
       <c r="G504" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H504" s="7" t="inlineStr"/>
@@ -20894,32 +20894,32 @@
     <row r="505">
       <c r="A505" s="6" t="inlineStr">
         <is>
-          <t>LEFT-01</t>
+          <t>OUR-12</t>
         </is>
       </c>
       <c r="B505" s="7" t="inlineStr">
         <is>
-          <t>Left off</t>
-        </is>
-      </c>
-      <c r="C505" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Ours</t>
+        </is>
+      </c>
+      <c r="C505" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D505" s="9" t="inlineStr">
         <is>
-          <t>Write a line on the held card</t>
+          <t>Unnamed lists read in each person's language</t>
         </is>
       </c>
       <c r="E505" s="9" t="inlineStr">
         <is>
-          <t>Hold a one-off task with no line on Today. Under the title, BEFORE anything is tapped, the card shows the dog-ear and 'Where you left off, for next time' (a hairline under it; a filled slip on Quiet); Today's rows show nothing new. Tap that line: the editor opens with the line field focused. Type 'Called, ref 4471, ring back Thu' and press the keyboard's done key. (Tapping the title also opens the same editor.)</t>
+          <t>Create a list WITHOUT naming it. Set the two accounts' devices to different languages (e.g. English and Italian).</t>
         </is>
       </c>
       <c r="F505" s="9" t="inlineStr">
         <is>
-          <t>'Noted.' shows in the affirm line, once. The card stays open and shows the dog-ear (level with the FIRST line of the words, in the editor and on the card, never above it), the words and today's calendar date (e.g. 'Sun, 4 Oct', never 'today') directly under the title. Shut the card: the Today row shows the dog-ear straight after the title and nothing else; the row is the same height as before. A screen reader hears the row label end ', has a note'. Return on the title field moves to the line field rather than closing.</t>
+          <t>Each person sees the app's own word for a shared list in their own language, not the other person's.</t>
         </is>
       </c>
       <c r="G505" s="7" t="inlineStr">
@@ -20934,7 +20934,7 @@
     <row r="506">
       <c r="A506" s="6" t="inlineStr">
         <is>
-          <t>LEFT-02</t>
+          <t>LEFT-01</t>
         </is>
       </c>
       <c r="B506" s="7" t="inlineStr">
@@ -20949,17 +20949,17 @@
       </c>
       <c r="D506" s="9" t="inlineStr">
         <is>
-          <t>Edit it, leave it, clear it</t>
+          <t>Write a line on the held card</t>
         </is>
       </c>
       <c r="E506" s="9" t="inlineStr">
         <is>
-          <t>On a task with a line, hold it and tap the line itself. Change a word and press done. Then open it again and close it without changing anything. Then open it, clear the field completely, and close it.</t>
+          <t>Hold a one-off task with no line on Today. Under the title, BEFORE anything is tapped, the card shows the dog-ear and 'Where you left off, for next time' (a hairline under it; a filled slip on Quiet); Today's rows show nothing new. Tap that line: the editor opens with the line field focused. Type 'Called, ref 4471, ring back Thu' and press the keyboard's done key. (Tapping the title also opens the same editor.)</t>
         </is>
       </c>
       <c r="F506" s="9" t="inlineStr">
         <is>
-          <t>Tapping the line opens the editor with the LINE field focused (tapping the title opens the same editor on the title). A changed line says 'Noted.' and its date becomes today. Unchanged: closes silently and keeps its original date. Cleared: no 'Noted.', the line leaves the card and the dog-ear leaves the Today row. A screen reader hears the card line as 'Where you left off: {line}. {weekday day month}.' with the hint 'Edit it.'</t>
+          <t>'Noted.' shows in the affirm line, once. The card stays open and shows the dog-ear (level with the FIRST line of the words, in the editor and on the card, never above it), the words and today's calendar date (e.g. 'Sun, 4 Oct', never 'today') directly under the title. Shut the card: the Today row shows the dog-ear straight after the title and nothing else; the row is the same height as before. A screen reader hears the row label end ', has a note'. Return on the title field moves to the line field rather than closing.</t>
         </is>
       </c>
       <c r="G506" s="7" t="inlineStr">
@@ -20974,7 +20974,7 @@
     <row r="507">
       <c r="A507" s="6" t="inlineStr">
         <is>
-          <t>LEFT-03</t>
+          <t>LEFT-02</t>
         </is>
       </c>
       <c r="B507" s="7" t="inlineStr">
@@ -20989,17 +20989,17 @@
       </c>
       <c r="D507" s="9" t="inlineStr">
         <is>
-          <t>Another action saves the open editor silently</t>
+          <t>Edit it, leave it, clear it</t>
         </is>
       </c>
       <c r="E507" s="9" t="inlineStr">
         <is>
-          <t>Open the editor on a held card, change BOTH the title and the line, then tap a card action without closing the editor first (Tomorrow, Move to..., Break it down, Close, Remove...).</t>
+          <t>On a task with a line, hold it and tap the line itself. Change a word and press done. Then open it again and close it without changing anything. Then open it, clear the field completely, and close it.</t>
         </is>
       </c>
       <c r="F507" s="9" t="inlineStr">
         <is>
-          <t>Title and line are both kept (one save, check by reopening the card, or after Undo on Remove). No 'Noted.': the action's own feedback is the only feedback, and the tap is never swallowed (on the web too, with a mouse). Nothing typed is lost whichever action is tapped, and tapping ANOTHER row while the editor is open also keeps the words, silently. Break it down or Make it tiny right after a rename works from the NEW title.</t>
+          <t>Tapping the line opens the editor with the LINE field focused (tapping the title opens the same editor on the title). A changed line says 'Noted.' and its date becomes today. Unchanged: closes silently and keeps its original date. Cleared: no 'Noted.', the line leaves the card and the dog-ear leaves the Today row. A screen reader hears the card line as 'Where you left off: {line}. {weekday day month}.' with the hint 'Edit it.'</t>
         </is>
       </c>
       <c r="G507" s="7" t="inlineStr">
@@ -21014,7 +21014,7 @@
     <row r="508">
       <c r="A508" s="6" t="inlineStr">
         <is>
-          <t>LEFT-04</t>
+          <t>LEFT-03</t>
         </is>
       </c>
       <c r="B508" s="7" t="inlineStr">
@@ -21029,17 +21029,17 @@
       </c>
       <c r="D508" s="9" t="inlineStr">
         <is>
-          <t>Focus: the slip</t>
+          <t>Another action saves the open editor silently</t>
         </is>
       </c>
       <c r="E508" s="9" t="inlineStr">
         <is>
-          <t>Open Focus on a task with no line. Tap the slip, type a line, then tap empty paper. Exit and reopen Focus on the same task. Then type new words and tap Done (and, on another task, Choose another, and Exit).</t>
+          <t>Open the editor on a held card, change BOTH the title and the line, then tap a card action without closing the editor first (Tomorrow, Move to..., Break it down, Close, Remove...).</t>
         </is>
       </c>
       <c r="F508" s="9" t="inlineStr">
         <is>
-          <t>With no line the slip holds only the placeholder: no label, no question. After the first save 'Noted.' lands near the bottom of the screen, never over the task, and the slip shows the dog-ear + 'Where you left off', the words in full (never clamped) and the date. Reopening shows the same slip. Done, Choose another and Exit each SAVE what was typed but say nothing. On a TINY step, type a line and tap Done straight away: the real task comes back on Today carrying that line. Reopen Focus on a task whose line was changed on its card meanwhile: the slip shows the NEW line, never the old draft. The slip never appears or changes because of anything just done.</t>
+          <t>Title and line are both kept (one save, check by reopening the card, or after Undo on Remove). No 'Noted.': the action's own feedback is the only feedback, and the tap is never swallowed (on the web too, with a mouse). Nothing typed is lost whichever action is tapped, and tapping ANOTHER row while the editor is open also keeps the words, silently. Break it down or Make it tiny right after a rename works from the NEW title.</t>
         </is>
       </c>
       <c r="G508" s="7" t="inlineStr">
@@ -21054,7 +21054,7 @@
     <row r="509">
       <c r="A509" s="6" t="inlineStr">
         <is>
-          <t>LEFT-05</t>
+          <t>LEFT-04</t>
         </is>
       </c>
       <c r="B509" s="7" t="inlineStr">
@@ -21062,24 +21062,24 @@
           <t>Left off</t>
         </is>
       </c>
-      <c r="C509" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C509" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D509" s="9" t="inlineStr">
         <is>
-          <t>A step shows its big task's line in Focus, read-only</t>
+          <t>Focus: the slip</t>
         </is>
       </c>
       <c r="E509" s="9" t="inlineStr">
         <is>
-          <t>Give a task a line, then Break it down. Open Focus on one of its steps.</t>
+          <t>Open Focus on a task with no line. Tap the slip, type a line, then tap empty paper. Exit and reopen Focus on the same task. Then type new words and tap Done (and, on another task, Choose another, and Exit).</t>
         </is>
       </c>
       <c r="F509" s="9" t="inlineStr">
         <is>
-          <t>The step has its own empty slip. Below it, past a hairline: '{big task title}: {line}' with the big task's title bold, and its own date, on bare paper. It is not a field: no press state, not focusable, cannot be edited. Writing the step's own line never moves it. The steps' Today rows and held cards do NOT show the big task's line (their mark means their own). A tiny step shows no parent line.</t>
+          <t>With no line the slip holds only the placeholder: no label, no question. After the first save 'Noted.' lands near the bottom of the screen, never over the task, and the slip shows the dog-ear + 'Where you left off', the words in full (never clamped) and the date. Reopening shows the same slip. Done, Choose another and Exit each SAVE what was typed but say nothing. On a TINY step, type a line and tap Done straight away: the real task comes back on Today carrying that line. Reopen Focus on a task whose line was changed on its card meanwhile: the slip shows the NEW line, never the old draft. The slip never appears or changes because of anything just done.</t>
         </is>
       </c>
       <c r="G509" s="7" t="inlineStr">
@@ -21094,7 +21094,7 @@
     <row r="510">
       <c r="A510" s="6" t="inlineStr">
         <is>
-          <t>LEFT-06</t>
+          <t>LEFT-05</t>
         </is>
       </c>
       <c r="B510" s="7" t="inlineStr">
@@ -21109,17 +21109,17 @@
       </c>
       <c r="D510" s="9" t="inlineStr">
         <is>
-          <t>Where a line never appears</t>
+          <t>A step shows its big task's line in Focus, read-only</t>
         </is>
       </c>
       <c r="E510" s="9" t="inlineStr">
         <is>
-          <t>Hold a repeating task on Today; open the Ours list and hold a shared row; Share to Ours a task that has a line; Bring a shared row to your Today and give the copy a line.</t>
+          <t>Give a task a line, then Break it down. Open Focus on one of its steps.</t>
         </is>
       </c>
       <c r="F510" s="9" t="inlineStr">
         <is>
-          <t>The repeating card keeps today's single-field title editor and shows no mark, no line and no empty line under its title (nor does a done card). The Ours list rows have no line field. The shared row created from a task with a line carries NO line (the partner never sees it). Your '· Ours' copy on Today can carry a line of its own: the dog-ear sits after the title, before '· Ours', and the partner's devices never show it. A ticked (done) task shows no line or mark, and gets it back unchanged if un-ticked.</t>
+          <t>The step has its own empty slip. Below it, past a hairline: '{big task title}: {line}' with the big task's title bold, and its own date, on bare paper. It is not a field: no press state, not focusable, cannot be edited. Writing the step's own line never moves it. The steps' Today rows and held cards do NOT show the big task's line (their mark means their own). A tiny step shows no parent line.</t>
         </is>
       </c>
       <c r="G510" s="7" t="inlineStr">
@@ -21134,7 +21134,7 @@
     <row r="511">
       <c r="A511" s="6" t="inlineStr">
         <is>
-          <t>LEFT-07</t>
+          <t>LEFT-06</t>
         </is>
       </c>
       <c r="B511" s="7" t="inlineStr">
@@ -21142,24 +21142,24 @@
           <t>Left off</t>
         </is>
       </c>
-      <c r="C511" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C511" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D511" s="9" t="inlineStr">
         <is>
-          <t>A line follows the task to every device</t>
+          <t>Where a line never appears</t>
         </is>
       </c>
       <c r="E511" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: supabase/tasks-left-off.sql applied and `python scripts/check-migrations.py` reports all four new columns present. Signed in on two devices, write a line on device A. Open device B. Then make a task tiny on A and tick its tiny step on B.</t>
+          <t>Hold a repeating task on Today; open the Ours list and hold a shared row; Share to Ours a task that has a line; Bring a shared row to your Today and give the copy a line.</t>
         </is>
       </c>
       <c r="F511" s="9" t="inlineStr">
         <is>
-          <t>Device B shows the same line, mark and date after a sync. Last write wins like a rename. The tiny step ticked on B brings the REAL task back on Today on both devices with its line (the tiny flag now travels too), and the tiny step reads 'A tiny step toward {title}' on B as well. A device on an older build keeps working; a rename there never erases the line.</t>
+          <t>The repeating card keeps today's single-field title editor and shows no mark, no line and no empty line under its title (nor does a done card). The Ours list rows have no line field. The shared row created from a task with a line carries NO line (the partner never sees it). Your '· Ours' copy on Today can carry a line of its own: the dog-ear sits after the title, before '· Ours', and the partner's devices never show it. A ticked (done) task shows no line or mark, and gets it back unchanged if un-ticked.</t>
         </is>
       </c>
       <c r="G511" s="7" t="inlineStr">
@@ -21174,7 +21174,7 @@
     <row r="512">
       <c r="A512" s="6" t="inlineStr">
         <is>
-          <t>LEFT-08</t>
+          <t>LEFT-07</t>
         </is>
       </c>
       <c r="B512" s="7" t="inlineStr">
@@ -21182,24 +21182,24 @@
           <t>Left off</t>
         </is>
       </c>
-      <c r="C512" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C512" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D512" s="9" t="inlineStr">
         <is>
-          <t>Combine, Make it tiny, Remove and Undo keep the line</t>
+          <t>A line follows the task to every device</t>
         </is>
       </c>
       <c r="E512" s="9" t="inlineStr">
         <is>
-          <t>Give two tasks different lines, a day apart if you can, and Combine them. Make a task with a line tiny, then tick the tiny step. Remove a task with a line and tap Undo.</t>
+          <t>PREREQ: supabase/tasks-left-off.sql applied and `python scripts/check-migrations.py` reports all four new columns present. Signed in on two devices, write a line on device A. Open device B. Then make a task tiny on A and tick its tiny step on B.</t>
         </is>
       </c>
       <c r="F512" s="9" t="inlineStr">
         <is>
-          <t>The combined task keeps the most recently written line with its own date (text is never merged). The tiny step's real task comes back with its line. Undo restores the task with its line intact.</t>
+          <t>Device B shows the same line, mark and date after a sync. Last write wins like a rename. The tiny step ticked on B brings the REAL task back on Today on both devices with its line (the tiny flag now travels too), and the tiny step reads 'A tiny step toward {title}' on B as well. A device on an older build keeps working; a rename there never erases the line.</t>
         </is>
       </c>
       <c r="G512" s="7" t="inlineStr">
@@ -21214,7 +21214,7 @@
     <row r="513">
       <c r="A513" s="6" t="inlineStr">
         <is>
-          <t>LEFT-09</t>
+          <t>LEFT-08</t>
         </is>
       </c>
       <c r="B513" s="7" t="inlineStr">
@@ -21229,17 +21229,17 @@
       </c>
       <c r="D513" s="9" t="inlineStr">
         <is>
-          <t>The date, the limit and pasted breaks</t>
+          <t>Combine, Make it tiny, Remove and Undo keep the line</t>
         </is>
       </c>
       <c r="E513" s="9" t="inlineStr">
         <is>
-          <t>Write a line, then switch the app through English, German, Spanish, French and Italian. Paste text with line breaks into the line field. Paste or type past 280 characters. (Optional, export/import or a seeded task) a line written in a previous calendar year.</t>
+          <t>Give two tasks different lines, a day apart if you can, and Combine them. Make a task with a line tiny, then tick the tiny step. Remove a task with a line and tap Undo.</t>
         </is>
       </c>
       <c r="F513" s="9" t="inlineStr">
         <is>
-          <t>The date is always the calendar day it was written, in the language's own format (e.g. 'Wed, 30 Sept', 'Mi., 30. Sept.', 'mer. 30 sept.'), never 'today', 'yesterday' or 'ago', and identical at any age. Pasted breaks become single spaces. Input stops silently at 280: no counter, no message, no colour change. A line from another year shows the year. No crash on Android at launch or on first render of a line (the formatter is Intl.DateTimeFormat only).</t>
+          <t>The combined task keeps the most recently written line with its own date (text is never merged). The tiny step's real task comes back with its line. Undo restores the task with its line intact.</t>
         </is>
       </c>
       <c r="G513" s="7" t="inlineStr">
@@ -21254,7 +21254,7 @@
     <row r="514">
       <c r="A514" s="6" t="inlineStr">
         <is>
-          <t>LEFT-10</t>
+          <t>LEFT-09</t>
         </is>
       </c>
       <c r="B514" s="7" t="inlineStr">
@@ -21262,24 +21262,24 @@
           <t>Left off</t>
         </is>
       </c>
-      <c r="C514" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C514" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D514" s="9" t="inlineStr">
         <is>
-          <t>The keyboard never buries the line field</t>
+          <t>The date, the limit and pasted breaks</t>
         </is>
       </c>
       <c r="E514" s="9" t="inlineStr">
         <is>
-          <t>On a phone, fill Today so a task sits near the bottom of the list. Hold it and tap its title, then press return to move to the line. Then open Focus and tap the slip.</t>
+          <t>Write a line, then switch the app through English, German, Spanish, French and Italian. Paste text with line breaks into the line field. Paste or type past 280 characters. (Optional, export/import or a seeded task) a line written in a previous calendar year.</t>
         </is>
       </c>
       <c r="F514" s="9" t="inlineStr">
         <is>
-          <t>On Android and iOS the list scrolls BY ITSELF so the line field sits just above the keyboard, the moment the keyboard is up (Melroy's iPhone, 2026-10-05: before the fix it hid under it); a card already clear of the keyboard does not move at all. In Focus the slip stays visible above the keyboard, and Done and Choose another stay reachable by scrolling. On Android Chrome the page resizes rather than hiding the field.</t>
+          <t>The date is always the calendar day it was written, in the language's own format (e.g. 'Wed, 30 Sept', 'Mi., 30. Sept.', 'mer. 30 sept.'), never 'today', 'yesterday' or 'ago', and identical at any age. Pasted breaks become single spaces. Input stops silently at 280: no counter, no message, no colour change. A line from another year shows the year. No crash on Android at launch or on first render of a line (the formatter is Intl.DateTimeFormat only).</t>
         </is>
       </c>
       <c r="G514" s="7" t="inlineStr">
@@ -21294,7 +21294,7 @@
     <row r="515">
       <c r="A515" s="6" t="inlineStr">
         <is>
-          <t>LEFT-11</t>
+          <t>LEFT-10</t>
         </is>
       </c>
       <c r="B515" s="7" t="inlineStr">
@@ -21302,24 +21302,24 @@
           <t>Left off</t>
         </is>
       </c>
-      <c r="C515" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C515" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D515" s="9" t="inlineStr">
         <is>
-          <t>Quiet appearance and the export</t>
+          <t>The keyboard never buries the line field</t>
         </is>
       </c>
       <c r="E515" s="9" t="inlineStr">
         <is>
-          <t>Switch to the Quiet appearance and open a held card with a line, then edit it. Then Settings &gt; Export your tasks.</t>
+          <t>On a phone, fill Today so a task sits near the bottom of the list. Hold it and tap its title, then press return to move to the line. Then open Focus and tap the slip.</t>
         </is>
       </c>
       <c r="F515" s="9" t="inlineStr">
         <is>
-          <t>On Quiet the resting line reads in ink (not the soft grey) on the wash, and the editor's line field is a filled slip with an accent ring when focused. Only the focused field looks focused (the title's underline drops to a hairline while the line is focused). The export includes each task's line and its date.</t>
+          <t>On Android and iOS the list scrolls BY ITSELF so the line field sits just above the keyboard, the moment the keyboard is up (Melroy's iPhone, 2026-10-05: before the fix it hid under it); a card already clear of the keyboard does not move at all. In Focus the slip stays visible above the keyboard, and Done and Choose another stay reachable by scrolling. On Android Chrome the page resizes rather than hiding the field.</t>
         </is>
       </c>
       <c r="G515" s="7" t="inlineStr">
@@ -21334,12 +21334,12 @@
     <row r="516">
       <c r="A516" s="6" t="inlineStr">
         <is>
-          <t>TEL-02</t>
+          <t>LEFT-11</t>
         </is>
       </c>
       <c r="B516" s="7" t="inlineStr">
         <is>
-          <t>Telemetry</t>
+          <t>Left off</t>
         </is>
       </c>
       <c r="C516" s="11" t="inlineStr">
@@ -21349,22 +21349,22 @@
       </c>
       <c r="D516" s="9" t="inlineStr">
         <is>
-          <t>'Where you left off' counts as bare names, never a word of the line</t>
+          <t>Quiet appearance and the export</t>
         </is>
       </c>
       <c r="E516" s="9" t="inlineStr">
         <is>
-          <t>Against a LOCAL Worker as in TEL-01, never production: save a line on a held card, save one in Focus, and clear one. Then SELECT day, event, n FROM app_event_counts.</t>
+          <t>Switch to the Quiet appearance and open a held card with a line, then edit it. Then Settings &gt; Export your tasks.</t>
         </is>
       </c>
       <c r="F516" s="9" t="inlineStr">
         <is>
-          <t>leftoff.saved.card 1, leftoff.saved.focus 1, leftoff.cleared 1. Each /event body is the bare name: no properties, no length, never a word of the text. A title-only rename sends only task.renamed, and an unchanged line sends nothing.</t>
+          <t>On Quiet the resting line reads in ink (not the soft grey) on the wash, and the editor's line field is a filled slip with an accent ring when focused. Only the focused field looks focused (the title's underline drops to a hairline while the line is focused). The export includes each task's line and its date.</t>
         </is>
       </c>
       <c r="G516" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H516" s="7" t="inlineStr"/>
@@ -21374,37 +21374,37 @@
     <row r="517">
       <c r="A517" s="6" t="inlineStr">
         <is>
-          <t>REV-01</t>
+          <t>TEL-02</t>
         </is>
       </c>
       <c r="B517" s="7" t="inlineStr">
         <is>
-          <t>Review ask</t>
-        </is>
-      </c>
-      <c r="C517" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Telemetry</t>
+        </is>
+      </c>
+      <c r="C517" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D517" s="9" t="inlineStr">
         <is>
-          <t>The earned card appears about 1.2s after the rested screen</t>
+          <t>'Where you left off' counts as bare names, never a word of the line</t>
         </is>
       </c>
       <c r="E517" s="9" t="inlineStr">
         <is>
-          <t>Do a good close. Move the device date forward 4 days and do another. Repeat until there have been 5 good closes spanning 16 days or more. Watch the rested screen after each Goodnight. Afterwards set the clock back to today and clear the app's storage (Settings &gt; Apps &gt; DoubleDone &gt; Storage), because the ask is now stamped in the future.</t>
+          <t>Against a LOCAL Worker as in TEL-01, never production: save a line on a held card, save one in Focus, and clear one. Then SELECT day, event, n FROM app_event_counts.</t>
         </is>
       </c>
       <c r="F517" s="9" t="inlineStr">
         <is>
-          <t>Closes 1 to 4 show the rested screen and nothing else. On the 5th, Play's own rating card appears about 1.2s after the rested screen lands, on top of it, with not one word of DoubleDone's before it, on it or after it (no 'Enjoying DoubleDone?', no thank-you). Rating, or dismissing it, returns to the rested screen exactly as it was. The count is never shown anywhere in the app.</t>
+          <t>leftoff.saved.card 1, leftoff.saved.focus 1, leftoff.cleared 1. Each /event body is the bare name: no properties, no length, never a word of the text. A title-only rename sends only task.renamed, and an unchanged line sends nothing.</t>
         </is>
       </c>
       <c r="G517" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H517" s="7" t="inlineStr"/>
@@ -21414,7 +21414,7 @@
     <row r="518">
       <c r="A518" s="6" t="inlineStr">
         <is>
-          <t>REV-02</t>
+          <t>REV-01</t>
         </is>
       </c>
       <c r="B518" s="7" t="inlineStr">
@@ -21429,22 +21429,22 @@
       </c>
       <c r="D518" s="9" t="inlineStr">
         <is>
-          <t>Never asks on a Low, Settle, Lighten or re-entry day, or outside the gates</t>
+          <t>The earned card appears about 1.2s after the rested screen</t>
         </is>
       </c>
       <c r="E518" s="9" t="inlineStr">
         <is>
-          <t>Earn the ask as in REV-01 up to 4 closes over 16+ days, so the next good close would ask. On that 5th day, before closing, do ONE of: choose Low on the Energy pills; choose Low and then move it back to Normal; open Settle and leave; run Lighten today; or open the app after 4+ days away (the 'Welcome back.' note shows). Then do a good close. Repeat once per item, each on its own day. Then, on separate days: close at 16:30; close with nothing finished and no Goodnight note; close on a heavy day (Lighten is offered).</t>
+          <t>Do a good close. Move the device date forward 4 days and do another. Repeat until there have been 5 good closes spanning 16 days or more. Watch the rested screen after each Goodnight. Afterwards set the clock back to today and clear the app's storage (Settings &gt; Apps &gt; DoubleDone &gt; Storage), because the ask is now stamped in the future.</t>
         </is>
       </c>
       <c r="F518" s="9" t="inlineStr">
         <is>
-          <t>No card on any of them: the rested screen only, and nothing breaks. A tender day (Low, Settle, Lighten, a return) stays quiet all day even if Energy is moved back to Normal. The first later evening that passes every gate asks, as in REV-01. On the web none of this applies (REV-04).</t>
+          <t>Closes 1 to 4 show the rested screen and nothing else. On the 5th, Play's own rating card appears about 1.2s after the rested screen lands, on top of it, with not one word of DoubleDone's before it, on it or after it (no 'Enjoying DoubleDone?', no thank-you). Rating, or dismissing it, returns to the rested screen exactly as it was. The count is never shown anywhere in the app.</t>
         </is>
       </c>
       <c r="G518" s="7" t="inlineStr">
         <is>
-          <t>iOS + Android</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H518" s="7" t="inlineStr"/>
@@ -21454,7 +21454,7 @@
     <row r="519">
       <c r="A519" s="6" t="inlineStr">
         <is>
-          <t>REV-03</t>
+          <t>REV-02</t>
         </is>
       </c>
       <c r="B519" s="7" t="inlineStr">
@@ -21462,24 +21462,24 @@
           <t>Review ask</t>
         </is>
       </c>
-      <c r="C519" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C519" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D519" s="9" t="inlineStr">
         <is>
-          <t>Once per version, 180 days apart, and a re-closed day counts once</t>
+          <t>Never asks on a Low, Settle, Lighten or re-entry day, or outside the gates</t>
         </is>
       </c>
       <c r="E519" s="9" t="inlineStr">
         <is>
-          <t>Part A: after REV-01's card, keep doing good closes for a week (clock forward). Part B, on a fresh install: do good closes on days 1, 8 and 16 (3 closes). On day 17 do a good close, tap 'Reopen today', and close it again. Then on day 18 do a good close. Part C: on any qualifying 5th close, tap 'Reopen today' within a second of Goodnight.</t>
+          <t>Earn the ask as in REV-01 up to 4 closes over 16+ days, so the next good close would ask. On that 5th day, before closing, do ONE of: choose Low on the Energy pills; choose Low and then move it back to Normal; open Settle and leave; run Lighten today; or open the app after 4+ days away (the 'Welcome back.' note shows). Then do a good close. Repeat once per item, each on its own day. Then, on separate days: close at 16:30; close with nothing finished and no Goodnight note; close on a heavy day (Lighten is offered).</t>
         </is>
       </c>
       <c r="F519" s="9" t="inlineStr">
         <is>
-          <t>A: no second card on 1.9.0, however many good days follow (a later version also waits 180 days from the last ask). B: no card on day 17, because a reopened and re-closed day is still one close (4 so far); the card appears on day 18, the real 5th. C: reopening before the card cancels the pending ask, so no card appears over the reopened day.</t>
+          <t>No card on any of them: the rested screen only, and nothing breaks. A tender day (Low, Settle, Lighten, a return) stays quiet all day even if Energy is moved back to Normal. The first later evening that passes every gate asks, as in REV-01. On the web none of this applies (REV-04).</t>
         </is>
       </c>
       <c r="G519" s="7" t="inlineStr">
@@ -21494,7 +21494,7 @@
     <row r="520">
       <c r="A520" s="6" t="inlineStr">
         <is>
-          <t>REV-04</t>
+          <t>REV-03</t>
         </is>
       </c>
       <c r="B520" s="7" t="inlineStr">
@@ -21502,29 +21502,29 @@
           <t>Review ask</t>
         </is>
       </c>
-      <c r="C520" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C520" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D520" s="9" t="inlineStr">
         <is>
-          <t>The web never asks and writes nothing</t>
+          <t>Once per version, 180 days apart, and a re-closed day counts once</t>
         </is>
       </c>
       <c r="E520" s="9" t="inlineStr">
         <is>
-          <t>On doubledone.app with the browser's console open: choose Low, open Settle, run Lighten, then do a good close in the evening (for an earned-looking case, repeat over several days with the computer's clock moved forward). Then open DevTools &gt; Application &gt; Local Storage for doubledone.app.</t>
+          <t>Part A: after REV-01's card, keep doing good closes for a week (clock forward). Part B, on a fresh install: do good closes on days 1, 8 and 16 (3 closes). On day 17 do a good close, tap 'Reopen today', and close it again. Then on day 18 do a good close. Part C: on any qualifying 5th close, tap 'Reopen today' within a second of Goodnight.</t>
         </is>
       </c>
       <c r="F520" s="9" t="inlineStr">
         <is>
-          <t>No rating card or popup of any kind, ever. No console warning about a store URL (nothing mentioning playStoreUrl or appStoreUrl). Local Storage holds no 'doubledone.review.v1' and no 'doubledone.reviewquiet.v1'. Developer check: after npx expo export -p web, grep -l StoreReview client/dist/_expo/static/js/web/*.js finds nothing.</t>
+          <t>A: no second card on 1.9.0, however many good days follow (a later version also waits 180 days from the last ask). B: no card on day 17, because a reopened and re-closed day is still one close (4 so far); the card appears on day 18, the real 5th. C: reopening before the card cancels the pending ask, so no card appears over the reopened day.</t>
         </is>
       </c>
       <c r="G520" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>iOS + Android</t>
         </is>
       </c>
       <c r="H520" s="7" t="inlineStr"/>
@@ -21534,7 +21534,7 @@
     <row r="521">
       <c r="A521" s="6" t="inlineStr">
         <is>
-          <t>REV-05</t>
+          <t>REV-04</t>
         </is>
       </c>
       <c r="B521" s="7" t="inlineStr">
@@ -21542,29 +21542,29 @@
           <t>Review ask</t>
         </is>
       </c>
-      <c r="C521" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C521" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D521" s="9" t="inlineStr">
         <is>
-          <t>TestFlight shows no card and nothing breaks</t>
+          <t>The web never asks and writes nothing</t>
         </is>
       </c>
       <c r="E521" s="9" t="inlineStr">
         <is>
-          <t>On the 1.9.0 TestFlight build, run REV-01's clock trick through the 5th good close.</t>
+          <t>On doubledone.app with the browser's console open: choose Low, open Settle, run Lighten, then do a good close in the evening (for an earned-looking case, repeat over several days with the computer's clock moved forward). Then open DevTools &gt; Application &gt; Local Storage for doubledone.app.</t>
         </is>
       </c>
       <c r="F521" s="9" t="inlineStr">
         <is>
-          <t>No card (Apple never shows it in TestFlight, by design), no crash or freeze, and the rested screen stays as it is. The ask is not spent, so the App Store build can still ask on that phone. The real card can only be seen on the App Store build after release, and Apple may still decline it (its three-a-year cap, its own judgement, or Settings &gt; Apps &gt; App Store &gt; In-App Ratings &amp; Reviews switched off).</t>
+          <t>No rating card or popup of any kind, ever. No console warning about a store URL (nothing mentioning playStoreUrl or appStoreUrl). Local Storage holds no 'doubledone.review.v1' and no 'doubledone.reviewquiet.v1'. Developer check: after npx expo export -p web, grep -l StoreReview client/dist/_expo/static/js/web/*.js finds nothing.</t>
         </is>
       </c>
       <c r="G521" s="7" t="inlineStr">
         <is>
-          <t>iOS</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H521" s="7" t="inlineStr"/>
@@ -21574,7 +21574,7 @@
     <row r="522">
       <c r="A522" s="6" t="inlineStr">
         <is>
-          <t>REV-06</t>
+          <t>REV-05</t>
         </is>
       </c>
       <c r="B522" s="7" t="inlineStr">
@@ -21589,22 +21589,22 @@
       </c>
       <c r="D522" s="9" t="inlineStr">
         <is>
-          <t>Never stacks with a goodnight offer</t>
+          <t>TestFlight shows no card and nothing breaks</t>
         </is>
       </c>
       <c r="E522" s="9" t="inlineStr">
         <is>
-          <t>On a fresh install, leave the daily reminder OFF and leave the rested screen's reminder offer unanswered on every close. Do 5 good closes over 16+ days as in REV-01. On the 5th, read the rested screen. Then answer the offer ('Not now') and do one more good close the next evening.</t>
+          <t>On the 1.9.0 TestFlight build, run REV-01's clock trick through the 5th good close.</t>
         </is>
       </c>
       <c r="F522" s="9" t="inlineStr">
         <is>
-          <t>On the 5th close the rested screen shows its one offer and no rating card: never both at once. After the offer is answered, the next qualifying evening shows the card as in REV-01. The same holds for the widget, scrapbook and update offers: whichever one shows, the card waits.</t>
+          <t>No card (Apple never shows it in TestFlight, by design), no crash or freeze, and the rested screen stays as it is. The ask is not spent, so the App Store build can still ask on that phone. The real card can only be seen on the App Store build after release, and Apple may still decline it (its three-a-year cap, its own judgement, or Settings &gt; Apps &gt; App Store &gt; In-App Ratings &amp; Reviews switched off).</t>
         </is>
       </c>
       <c r="G522" s="7" t="inlineStr">
         <is>
-          <t>iOS + Android</t>
+          <t>iOS</t>
         </is>
       </c>
       <c r="H522" s="7" t="inlineStr"/>
@@ -21614,7 +21614,7 @@
     <row r="523">
       <c r="A523" s="6" t="inlineStr">
         <is>
-          <t>REV-07</t>
+          <t>REV-06</t>
         </is>
       </c>
       <c r="B523" s="7" t="inlineStr">
@@ -21629,17 +21629,17 @@
       </c>
       <c r="D523" s="9" t="inlineStr">
         <is>
-          <t>A Goodnight note that opens the scrapbook offer never brings the card with it</t>
+          <t>Never stacks with a goodnight offer</t>
         </is>
       </c>
       <c r="E523" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: AI on, the rested screen's reminder offer already answered (and on Android the widget offer too), and the scrapbook never made and never offered. Earn the ask as in REV-01 up to 4 good closes over 16+ days. On the 5th evening, make sure exactly 2 different tasks have been finished so far this week (the week runs Sunday to Saturday, and finishes from earlier closes count), then Close the day, write a Goodnight note ('Called the bank') and tap Goodnight.</t>
+          <t>On a fresh install, leave the daily reminder OFF and leave the rested screen's reminder offer unanswered on every close. Do 5 good closes over 16+ days as in REV-01. On the 5th, read the rested screen. Then answer the offer ('Not now') and do one more good close the next evening.</t>
         </is>
       </c>
       <c r="F523" s="9" t="inlineStr">
         <is>
-          <t>The note counts as the week's third finish, so the rested screen shows the scrapbook offer, and NO rating card appears, then or a few seconds later. Answering the offer (either way) brings no card that night either: the evening already had its one ask. The next qualifying evening asks as in REV-01.</t>
+          <t>On the 5th close the rested screen shows its one offer and no rating card: never both at once. After the offer is answered, the next qualifying evening shows the card as in REV-01. The same holds for the widget, scrapbook and update offers: whichever one shows, the card waits.</t>
         </is>
       </c>
       <c r="G523" s="7" t="inlineStr">
@@ -21654,7 +21654,7 @@
     <row r="524">
       <c r="A524" s="6" t="inlineStr">
         <is>
-          <t>REV-08</t>
+          <t>REV-07</t>
         </is>
       </c>
       <c r="B524" s="7" t="inlineStr">
@@ -21662,29 +21662,29 @@
           <t>Review ask</t>
         </is>
       </c>
-      <c r="C524" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C524" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D524" s="9" t="inlineStr">
         <is>
-          <t>A double tap on Goodnight asks the store once</t>
+          <t>A Goodnight note that opens the scrapbook offer never brings the card with it</t>
         </is>
       </c>
       <c r="E524" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: the Android 1.9.0 build on the internal track, a phone on USB with adb logcat -s ReactNativeJS running. Earn the ask as in REV-01 up to the 5th good close, then tap Goodnight twice, as fast as you can, while the close fades.</t>
+          <t>PREREQ: AI on, the rested screen's reminder offer already answered (and on Android the widget offer too), and the scrapbook never made and never offered. Earn the ask as in REV-01 up to 4 good closes over 16+ days. On the 5th evening, make sure exactly 2 different tasks have been finished so far this week (the week runs Sunday to Saturday, and finishes from earlier closes count), then Close the day, write a Goodnight note ('Called the bank') and tap Goodnight.</t>
         </is>
       </c>
       <c r="F524" s="9" t="inlineStr">
         <is>
-          <t>At most one rating card. The log shows exactly one [doubledone.review.asked] line for that close, never two, and nothing asks again on later evenings of 1.9.0.</t>
+          <t>The note counts as the week's third finish, so the rested screen shows the scrapbook offer, and NO rating card appears, then or a few seconds later. Answering the offer (either way) brings no card that night either: the evening already had its one ask. The next qualifying evening asks as in REV-01.</t>
         </is>
       </c>
       <c r="G524" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>iOS + Android</t>
         </is>
       </c>
       <c r="H524" s="7" t="inlineStr"/>
@@ -21694,12 +21694,12 @@
     <row r="525">
       <c r="A525" s="6" t="inlineStr">
         <is>
-          <t>TEL-03</t>
+          <t>REV-08</t>
         </is>
       </c>
       <c r="B525" s="7" t="inlineStr">
         <is>
-          <t>Telemetry</t>
+          <t>Review ask</t>
         </is>
       </c>
       <c r="C525" s="11" t="inlineStr">
@@ -21709,31 +21709,71 @@
       </c>
       <c r="D525" s="9" t="inlineStr">
         <is>
-          <t>review.asked.ios and review.asked.android counters appear, and nothing else</t>
+          <t>A double tap on Goodnight asks the store once</t>
         </is>
       </c>
       <c r="E525" s="9" t="inlineStr">
         <is>
-          <t>About 3 weeks after 1.9.0 is live in both stores (nothing can ask for 14 days after an update), and only once the Worker carrying the two names is deployed: from server/, npx wrangler d1 execute doubledone-telemetry --remote --command "SELECT day, event, n FROM app_event_counts WHERE event LIKE 'review.%'". Read only: never POST to production /event to test it.</t>
+          <t>PREREQ: the Android 1.9.0 build on the internal track, a phone on USB with adb logcat -s ReactNativeJS running. Earn the ask as in REV-01 up to the 5th good close, then tap Goodnight twice, as fast as you can, while the close fades.</t>
         </is>
       </c>
       <c r="F525" s="9" t="inlineStr">
         <is>
-          <t>Rows named review.asked.ios and review.asked.android only, each a day, the name and a count. Never a bare review.asked, never review.unavailable or review.failed (those stay on the device), and nothing holding a version, a rating or a number of closes. Asks from the Play internal test track are counted too (only dev sessions are kept out), so subtract them. Still zero 30 days after the earliest possible ask: read the gates in client/src/lib/review.ts before loosening anything.</t>
+          <t>At most one rating card. The log shows exactly one [doubledone.review.asked] line for that close, never two, and nothing asks again on later evenings of 1.9.0.</t>
         </is>
       </c>
       <c r="G525" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H525" s="7" t="inlineStr"/>
       <c r="I525" s="9" t="inlineStr"/>
       <c r="J525" s="7" t="inlineStr"/>
     </row>
+    <row r="526">
+      <c r="A526" s="6" t="inlineStr">
+        <is>
+          <t>TEL-03</t>
+        </is>
+      </c>
+      <c r="B526" s="7" t="inlineStr">
+        <is>
+          <t>Telemetry</t>
+        </is>
+      </c>
+      <c r="C526" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D526" s="9" t="inlineStr">
+        <is>
+          <t>review.asked.ios and review.asked.android counters appear, and nothing else</t>
+        </is>
+      </c>
+      <c r="E526" s="9" t="inlineStr">
+        <is>
+          <t>About 3 weeks after 1.9.0 is live in both stores (nothing can ask for 14 days after an update), and only once the Worker carrying the two names is deployed: from server/, npx wrangler d1 execute doubledone-telemetry --remote --command "SELECT day, event, n FROM app_event_counts WHERE event LIKE 'review.%'". Read only: never POST to production /event to test it.</t>
+        </is>
+      </c>
+      <c r="F526" s="9" t="inlineStr">
+        <is>
+          <t>Rows named review.asked.ios and review.asked.android only, each a day, the name and a count. Never a bare review.asked, never review.unavailable or review.failed (those stay on the device), and nothing holding a version, a rating or a number of closes. Asks from the Play internal test track are counted too (only dev sessions are kept out), so subtract them. Still zero 30 days after the earliest possible ask: read the gates in client/src/lib/review.ts before loosening anything.</t>
+        </is>
+      </c>
+      <c r="G526" s="7" t="inlineStr">
+        <is>
+          <t>Worker</t>
+        </is>
+      </c>
+      <c r="H526" s="7" t="inlineStr"/>
+      <c r="I526" s="9" t="inlineStr"/>
+      <c r="J526" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J525"/>
-  <conditionalFormatting sqref="H2:H525">
+  <autoFilter ref="A1:J526"/>
+  <conditionalFormatting sqref="H2:H526">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -21745,7 +21785,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H525" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H526" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -21781,7 +21821,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>524</t>
+          <t>525</t>
         </is>
       </c>
     </row>
@@ -21792,7 +21832,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$525,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$526,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -21803,7 +21843,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$525,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$526,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -21814,7 +21854,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$525,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$526,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -21825,7 +21865,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$525,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$526,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -21836,7 +21876,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>524-COUNTA('Test Suite'!$H$2:$H$525)</f>
+        <f>525-COUNTA('Test Suite'!$H$2:$H$526)</f>
         <v/>
       </c>
     </row>
@@ -21847,7 +21887,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$525,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$526,"P1")</f>
         <v/>
       </c>
     </row>
@@ -21858,7 +21898,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$525,"P1",'Test Suite'!$H$2:$H$525,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$526,"P1",'Test Suite'!$H$2:$H$526,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
test(qa): the review-ask cases' clock recipe can actually earn the card
REV-01 had three traps, and the other REV cases lean on it:

- Jumping the clock 4 days made the 5th evening a 'Welcome back.' return
  (REENTRY_GAP_DAYS is 4). That is a quiet day by design, so the case as
  written showed no card and looked like a bug. Every close still
  counts, so only the last jump has to be under 4 days. The recipe is
  now days 0, 4, 8, 12 and 15.
- It named no clock time, but the ask only comes from 17:00 to 01:59.
- It left the rested screen's offers unanswered. An evening with an
  offer never asks.

It also adds a prerequisite: a fresh install, signed out. With the clock
moved forward, every edit carries a future date, and sync keeps the
latest, so on a real account those rows would beat real edits for two
weeks.

REV-02, 03, 05, 06 and 07 now name the same days and setup.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -21434,12 +21434,12 @@
       </c>
       <c r="E518" s="9" t="inlineStr">
         <is>
-          <t>Do a good close. Move the device date forward 4 days and do another. Repeat until there have been 5 good closes spanning 16 days or more. Watch the rested screen after each Goodnight. Afterwards set the clock back to today and clear the app's storage (Settings &gt; Apps &gt; DoubleDone &gt; Storage), because the ask is now stamped in the future.</t>
+          <t>PREREQ: the Android 1.9.0 build installed from the Internal testing track, on a FRESH install that is NOT signed in. With the clock moved forward every edit carries a future date, and sync keeps the latest one, so on a real account those rows would beat real edits (a partner's on a shared list included) for two weeks. Turn the phone's automatic date and time OFF. Set the time to 19:00, because the ask only comes between 17:00 and 01:59. Do a good close: tick at least one task, leave Energy on Normal, do not open Settle or run Lighten, then tap Goodnight. Answer every offer the rested screen makes (the reminder, the widget, the scrapbook) with 'Not now', because an evening that shows an offer never asks (REV-06). Move the date forward 4 days and do another good close, then again to day 8 and day 12. Then move it forward only 3 days, to day 15, for the 5th: a jump of 4 days or more makes that evening a 'Welcome back.' return, which keeps the ask quiet by design (REV-02), so the asking evening must come less than 4 days after the last open. Watch the rested screen after each Goodnight, and dismiss the card rather than rate. Afterwards set the date and time back to automatic and clear the app's storage (Settings &gt; Apps &gt; DoubleDone &gt; Storage), because the ask is now stamped in the future.</t>
         </is>
       </c>
       <c r="F518" s="9" t="inlineStr">
         <is>
-          <t>Closes 1 to 4 show the rested screen and nothing else. On the 5th, Play's own rating card appears about 1.2s after the rested screen lands, on top of it, with not one word of DoubleDone's before it, on it or after it (no 'Enjoying DoubleDone?', no thank-you). Rating, or dismissing it, returns to the rested screen exactly as it was. The count is never shown anywhere in the app.</t>
+          <t>Closes 1 to 4 show the rested screen and nothing else (days 4, 8 and 12 open with a 'Welcome back.' note, as expected). If the 5th evening shows an offer instead, answer it and do one more good close the next evening: that one asks. On the 5th, Play's own rating card appears about 1.2s after the rested screen lands, on top of it, with not one word of DoubleDone's before it, on it or after it (no 'Enjoying DoubleDone?', no thank-you). Rating, or dismissing it, returns to the rested screen exactly as it was. The count is never shown anywhere in the app.</t>
         </is>
       </c>
       <c r="G518" s="7" t="inlineStr">
@@ -21474,7 +21474,7 @@
       </c>
       <c r="E519" s="9" t="inlineStr">
         <is>
-          <t>Earn the ask as in REV-01 up to 4 closes over 16+ days, so the next good close would ask. On that 5th day, before closing, do ONE of: choose Low on the Energy pills; choose Low and then move it back to Normal; open Settle and leave; run Lighten today; or open the app after 4+ days away (the 'Welcome back.' note shows). Then do a good close. Repeat once per item, each on its own day. Then, on separate days: close at 16:30; close with nothing finished and no Goodnight note; close on a heavy day (Lighten is offered).</t>
+          <t>Earn the ask as in REV-01 through its 4th close (day 12), so the next good close would ask. Move the date on 3 days (day 15) and, before closing, do ONE of: choose Low on the Energy pills; choose Low and then move it back to Normal; open Settle and leave; run Lighten today; or open the app after 4+ days away (the 'Welcome back.' note shows). Then do a good close. Repeat once per item, each on its own day, moving the date on ONE day at a time (only the return item jumps 4 days or more), because a quiet evening leaves the ask waiting and the next good evening would spend it. Then, on separate days: close at 16:30; close with nothing finished and no Goodnight note; close on a heavy day (Lighten is offered).</t>
         </is>
       </c>
       <c r="F519" s="9" t="inlineStr">
@@ -21514,7 +21514,7 @@
       </c>
       <c r="E520" s="9" t="inlineStr">
         <is>
-          <t>Part A: after REV-01's card, keep doing good closes for a week (clock forward). Part B, on a fresh install: do good closes on days 1, 8 and 16 (3 closes). On day 17 do a good close, tap 'Reopen today', and close it again. Then on day 18 do a good close. Part C: on any qualifying 5th close, tap 'Reopen today' within a second of Goodnight.</t>
+          <t>Part A: after REV-01's card, keep doing good closes for a week (clock forward). Part B, on a fresh install set up as in REV-01 (signed out, 19:00, offers answered): do good closes on days 1, 8 and 16 (3 closes). On day 17 do a good close, tap 'Reopen today', and close it again. Then on day 18 do a good close. Part C: on any qualifying 5th close, tap 'Reopen today' within a second of Goodnight.</t>
         </is>
       </c>
       <c r="F520" s="9" t="inlineStr">
@@ -21594,7 +21594,7 @@
       </c>
       <c r="E522" s="9" t="inlineStr">
         <is>
-          <t>On the 1.9.0 TestFlight build, run REV-01's clock trick through the 5th good close.</t>
+          <t>On the 1.9.0 TestFlight build, run REV-01's clock trick through the 5th good close (on iOS the switch is Settings &gt; General &gt; Date &amp; Time &gt; Set Automatically).</t>
         </is>
       </c>
       <c r="F522" s="9" t="inlineStr">
@@ -21634,7 +21634,7 @@
       </c>
       <c r="E523" s="9" t="inlineStr">
         <is>
-          <t>On a fresh install, leave the daily reminder OFF and leave the rested screen's reminder offer unanswered on every close. Do 5 good closes over 16+ days as in REV-01. On the 5th, read the rested screen. Then answer the offer ('Not now') and do one more good close the next evening.</t>
+          <t>On a fresh install, leave the daily reminder OFF and leave the rested screen's reminder offer unanswered on every close. Do 5 good closes on the days REV-01 uses (0, 4, 8, 12 and 15), signed out and at 19:00 as REV-01 sets up. On the 5th, read the rested screen. Then answer the offer ('Not now') and do one more good close the next evening.</t>
         </is>
       </c>
       <c r="F523" s="9" t="inlineStr">
@@ -21674,7 +21674,7 @@
       </c>
       <c r="E524" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: AI on, the rested screen's reminder offer already answered (and on Android the widget offer too), and the scrapbook never made and never offered. Earn the ask as in REV-01 up to 4 good closes over 16+ days. On the 5th evening, make sure exactly 2 different tasks have been finished so far this week (the week runs Sunday to Saturday, and finishes from earlier closes count), then Close the day, write a Goodnight note ('Called the bank') and tap Goodnight.</t>
+          <t>PREREQ: AI on, the rested screen's reminder offer already answered (and on Android the widget offer too), and the scrapbook never made and never offered. Earn the ask as in REV-01 through its 4th good close (day 12). On the 5th evening (day 15, 3 days on), make sure exactly 2 different tasks have been finished so far this week (the week runs Sunday to Saturday, and finishes from earlier closes count), then Close the day, write a Goodnight note ('Called the bank') and tap Goodnight.</t>
         </is>
       </c>
       <c r="F524" s="9" t="inlineStr">

</xml_diff>

<commit_message>
docs(build-plan): Android 1.9.0 passed its device checks, iOS 43 is in TestFlight
Melroy ran I18N-02, A11Y-09, A11Y-13, A11Y-08 and REV-01 on versionCode
36 from Internal testing, and all five passed. Play showed its rating
card on the 5th good close. That ask reached production as
review.asked.android = 1, which proves the counter end to end; TEL-03
will subtract it.

A11Y-08 now checks what TalkBack actually does. It reads the labelled
long press as the row's hint ("double tap and hold to Options") and, on
his version, gives it no Actions-menu entry. That is not a fail.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -10361,17 +10361,17 @@
       </c>
       <c r="D241" s="9" t="inlineStr">
         <is>
-          <t>TalkBack's double-tap-and-hold and its Actions menu open the card, and back closes it</t>
+          <t>TalkBack names the 'Options' action, double-tap-and-hold opens the card, and back closes it</t>
         </is>
       </c>
       <c r="E241" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: the 1.9.0 build, installed from Play. Turn on TalkBack. Focus a task row and double-tap and hold. Press the system back. Focus another row, open TalkBack's actions (a swipe up then right, or a three-finger tap, depending on the phone) and choose 'Options'. Press back again, then once more with no card open. Last, as a free user with a shared list, hold a row in Today's 'Due today' strip, choose Pin so Premium opens, and press back there.</t>
+          <t>PREREQ: the 1.9.0 build, installed from Play. Turn on TalkBack. Focus a task row and listen to the end of what TalkBack reads. Then double-tap and hold. Press the system back, then once more with no card open. If this phone's TalkBack also lists the action in its Actions menu (a three-finger tap, or a swipe up then right, depending on the version), focus another row and choose 'Options' there too. Last, as a free user with a shared list, hold a row in Today's 'Due today' strip, choose Pin so Premium opens, and press back there.</t>
         </is>
       </c>
       <c r="F241" s="9" t="inlineStr">
         <is>
-          <t>Both ways open that task's card, and TalkBack moves to the card's title. Back closes the card and TalkBack returns to the row. With no card open, back does what it always did. On Premium, back leaves Premium (it never closes the card left open behind it), and the next back on Today closes that card.</t>
+          <t>The row's hint ends 'double tap and hold to Options' (after 'Double tap to toggle'): that is the label working. TalkBack reads a labelled long press as a standard action, so on many versions it is offered only as that hint and has no Actions-menu entry, which is not a fail (Melroy's phone, 2026-10-19). Double-tap-and-hold, and the menu's 'Options' where it is listed, open that task's card, and TalkBack moves to the card's title. Back closes the card and TalkBack returns to the row. With no card open, back does what it always did. On Premium, back leaves Premium (it never closes the card left open behind it), and the next back on Today closes that card.</t>
         </is>
       </c>
       <c r="G241" s="7" t="inlineStr">

</xml_diff>

<commit_message>
test(qa): I18N-02 names the iPhone's two-language condition, A11Y-13 keeps a waiting draft
Two corrections from Melroy's iPhone pass of 1.9.0:

- iOS shows an app's Language row only when the phone has two or more
  preferred languages, so I18N-02 now says to add Deutsch first.
- The Brain dump shortcut deliberately never clears words still waiting
  to be added (seed(null) only focuses the field). A11Y-13 had expected
  an empty field, which is only true when nothing was waiting.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -10046,7 +10046,7 @@
       </c>
       <c r="E233" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: a store build made after 2026-10-05 (it is native config, so web and older builds cannot show it). Set the phone's language to German, open DoubleDone. On iOS also open Settings -&gt; DoubleDone -&gt; Language.</t>
+          <t>PREREQ: a store build made after 2026-10-05 (it is native config, so web and older builds cannot show it). Set the phone's language to German, open DoubleDone. On iOS also open Settings -&gt; Apps -&gt; DoubleDone -&gt; Language. iOS shows that row only when the phone has two or more languages under Settings -&gt; General -&gt; Language &amp; Region, so add Deutsch there first and choose 'Keep English' (Melroy's iPhone, 2026-10-19).</t>
         </is>
       </c>
       <c r="F233" s="9" t="inlineStr">
@@ -10571,7 +10571,7 @@
       </c>
       <c r="F246" s="9" t="inlineStr">
         <is>
-          <t>Both times the card closes by itself and the capture panel rises with the keyboard up: the shared words are in the field, ready to add, and the shortcut gives an empty field ready to type. Nothing is added without a tap. In select mode the share waits as the pill's draft dots, as before, and is in the panel once select mode ends and the pill is opened.</t>
+          <t>Both times the card closes by itself and the capture panel rises with the keyboard up: the shared words are in the field, ready to add, and the shortcut opens the field ready to type. The shortcut never clears waiting words (BrainDump's seed(null) only focuses), so if the shared text was not added it is still there, which is right; it is empty only when nothing was waiting. Nothing is added without a tap. In select mode the share waits as the pill's draft dots, as before, and is in the panel once select mode ends and the pill is opened.</t>
         </is>
       </c>
       <c r="G246" s="7" t="inlineStr">

</xml_diff>